<commit_message>
adding new plants to 2022 as well
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/vt_EST_ELC_v1.xlsx
+++ b/VerveStacks_EST/vt_EST_ELC_v1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E74863C6-8B33-463B-9104-D27CBEABF2FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA2ACDC1-770D-471A-9965-86EBEAA75F94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-10470" yWindow="10890" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{21C51102-B905-44E2-89DF-C1A7E31F8D9F}"/>
   </bookViews>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="608" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="620" uniqueCount="148">
   <si>
     <t>~fi_t</t>
   </si>
@@ -507,7 +507,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -522,13 +522,6 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
-      <charset val="186"/>
     </font>
   </fonts>
   <fills count="2">
@@ -3833,6 +3826,18 @@
       <c r="P38" t="s">
         <v>142</v>
       </c>
+      <c r="Q38" t="s">
+        <v>71</v>
+      </c>
+      <c r="R38" t="s">
+        <v>72</v>
+      </c>
+      <c r="S38" t="s">
+        <v>80</v>
+      </c>
+      <c r="T38" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="39" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B39" t="s">
@@ -3877,6 +3882,18 @@
       <c r="P39" t="s">
         <v>143</v>
       </c>
+      <c r="Q39" t="s">
+        <v>71</v>
+      </c>
+      <c r="R39" t="s">
+        <v>72</v>
+      </c>
+      <c r="S39" t="s">
+        <v>80</v>
+      </c>
+      <c r="T39" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="40" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B40" t="s">
@@ -3921,6 +3938,18 @@
       <c r="P40" t="s">
         <v>144</v>
       </c>
+      <c r="Q40" t="s">
+        <v>71</v>
+      </c>
+      <c r="R40" t="s">
+        <v>72</v>
+      </c>
+      <c r="S40" t="s">
+        <v>80</v>
+      </c>
+      <c r="T40" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="41" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B41" t="s">
@@ -4186,7 +4215,7 @@
         <v>14</v>
       </c>
       <c r="E49">
-        <v>2025</v>
+        <v>2022</v>
       </c>
       <c r="F49">
         <v>0.26</v>
@@ -4218,7 +4247,7 @@
         <v>14</v>
       </c>
       <c r="E50">
-        <v>2025</v>
+        <v>2022</v>
       </c>
       <c r="F50">
         <v>0.185</v>
@@ -4250,7 +4279,7 @@
         <v>14</v>
       </c>
       <c r="E51">
-        <v>2025</v>
+        <v>2022</v>
       </c>
       <c r="F51">
         <v>0.01</v>

</xml_diff>

<commit_message>
Reducing bioenergy active cost
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/vt_EST_ELC_v1.xlsx
+++ b/VerveStacks_EST/vt_EST_ELC_v1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA2ACDC1-770D-471A-9965-86EBEAA75F94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07E0C23C-4758-420D-871A-97A950AFB2C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-10470" yWindow="10890" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{21C51102-B905-44E2-89DF-C1A7E31F8D9F}"/>
   </bookViews>
@@ -41,10 +41,19 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
+    <author>tc={3057E3B1-7BF3-4718-B31B-0585028D4313}</author>
     <author>tc={E45DD652-654C-4828-8A13-679EDDC53E65}</author>
   </authors>
   <commentList>
-    <comment ref="F13" authorId="0" shapeId="0" xr:uid="{E45DD652-654C-4828-8A13-679EDDC53E65}">
+    <comment ref="J11" authorId="0" shapeId="0" xr:uid="{3057E3B1-7BF3-4718-B31B-0585028D4313}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    From 9,24 to 6</t>
+      </text>
+    </comment>
+    <comment ref="F13" authorId="1" shapeId="0" xr:uid="{E45DD652-654C-4828-8A13-679EDDC53E65}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -507,7 +516,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -522,6 +531,12 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="186"/>
     </font>
   </fonts>
   <fills count="2">
@@ -887,6 +902,9 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="J11" dT="2026-01-27T14:26:51.36" personId="{9CD26280-DD25-46DF-A708-6877D8A68AD8}" id="{3057E3B1-7BF3-4718-B31B-0585028D4313}">
+    <text>From 9,24 to 6</text>
+  </threadedComment>
   <threadedComment ref="F13" dT="2026-01-22T14:00:05.64" personId="{9CD26280-DD25-46DF-A708-6877D8A68AD8}" id="{E45DD652-654C-4828-8A13-679EDDC53E65}">
     <text>Iru produces only 17 MW in 2025 not 0.207 GW</text>
   </threadedComment>
@@ -2326,9 +2344,13 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="40.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="40.5703125" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="64.42578125" bestFit="1" customWidth="1"/>
   </cols>
@@ -2423,7 +2445,7 @@
         <v>157.30000000000001</v>
       </c>
       <c r="J11">
-        <v>9.240000000000002</v>
+        <v>6</v>
       </c>
       <c r="K11">
         <v>50</v>

</xml_diff>

<commit_message>
Adding power plants based on 2025 state
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/vt_EST_ELC_v1.xlsx
+++ b/VerveStacks_EST/vt_EST_ELC_v1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07E0C23C-4758-420D-871A-97A950AFB2C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0B2FAC8-88CE-4056-A720-FCCA62D973FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-10470" yWindow="10890" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{21C51102-B905-44E2-89DF-C1A7E31F8D9F}"/>
+    <workbookView xWindow="-10470" yWindow="10890" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{21C51102-B905-44E2-89DF-C1A7E31F8D9F}"/>
   </bookViews>
   <sheets>
     <sheet name="ccs_retrofits" sheetId="4" r:id="rId1"/>
@@ -41,11 +41,56 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
+    <author>tc={E45DD652-654C-4828-8A13-679EDDC53E65}</author>
+    <author>tc={06D70610-96F7-4BDA-B071-69925D70228B}</author>
+    <author>tc={A1B9CC12-DC46-488C-9BF3-3F8DFC23199D}</author>
+    <author>tc={4E0E017D-BAC7-4AA8-B401-A7330F2C0996}</author>
+    <author>tc={1905391B-2A5F-4643-B2AC-720AD8410CDA}</author>
     <author>tc={3057E3B1-7BF3-4718-B31B-0585028D4313}</author>
-    <author>tc={E45DD652-654C-4828-8A13-679EDDC53E65}</author>
   </authors>
   <commentList>
-    <comment ref="J11" authorId="0" shapeId="0" xr:uid="{3057E3B1-7BF3-4718-B31B-0585028D4313}">
+    <comment ref="F11" authorId="0" shapeId="0" xr:uid="{E45DD652-654C-4828-8A13-679EDDC53E65}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Iru produces only 17 MW in 2025 not 0.207 GW</t>
+      </text>
+    </comment>
+    <comment ref="G46" authorId="1" shapeId="0" xr:uid="{06D70610-96F7-4BDA-B071-69925D70228B}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Danish Energy agency - coal CHP 2020</t>
+      </text>
+    </comment>
+    <comment ref="G49" authorId="2" shapeId="0" xr:uid="{A1B9CC12-DC46-488C-9BF3-3F8DFC23199D}">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    DAE - gas engines 2020
+</t>
+      </text>
+    </comment>
+    <comment ref="G50" authorId="3" shapeId="0" xr:uid="{4E0E017D-BAC7-4AA8-B401-A7330F2C0996}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    DAE - Wood pellets, Medium 2020</t>
+      </text>
+    </comment>
+    <comment ref="N77" authorId="4" shapeId="0" xr:uid="{1905391B-2A5F-4643-B2AC-720AD8410CDA}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Frequency reserve</t>
+      </text>
+    </comment>
+    <comment ref="J80" authorId="5" shapeId="0" xr:uid="{3057E3B1-7BF3-4718-B31B-0585028D4313}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -53,20 +98,12 @@
     From 9,24 to 6</t>
       </text>
     </comment>
-    <comment ref="F13" authorId="1" shapeId="0" xr:uid="{E45DD652-654C-4828-8A13-679EDDC53E65}">
-      <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-    Iru produces only 17 MW in 2025 not 0.207 GW</t>
-      </text>
-    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="620" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="870" uniqueCount="201">
   <si>
     <t>~fi_t</t>
   </si>
@@ -494,28 +531,190 @@
     <t>Additions by Kristopher</t>
   </si>
   <si>
-    <t>Auvere elektrijaam</t>
-  </si>
-  <si>
-    <t>Balti elektrijaam</t>
-  </si>
-  <si>
-    <t>Enefit elektrijaam</t>
-  </si>
-  <si>
-    <t>ep_oil_internal_combustion_auvere</t>
-  </si>
-  <si>
-    <t>ep_oil_internal_combustion_balti</t>
-  </si>
-  <si>
-    <t>ep_oil_internal_combustion_enefit</t>
+    <t>ep_gas_combined_cycle_pohja</t>
+  </si>
+  <si>
+    <t>ep_bioenergy_tlnutilitas</t>
+  </si>
+  <si>
+    <t>ep_bioenergy_tartu</t>
+  </si>
+  <si>
+    <t>ep_bioenergy_parnu</t>
+  </si>
+  <si>
+    <t>ep_bioenergy_horizon</t>
+  </si>
+  <si>
+    <t>Horizon Tselluloosi ja paberi AS</t>
+  </si>
+  <si>
+    <t>Balti PP</t>
+  </si>
+  <si>
+    <t>Enefit PP</t>
+  </si>
+  <si>
+    <t>Eesti PP</t>
+  </si>
+  <si>
+    <t>Utilitas Tallinna PP</t>
+  </si>
+  <si>
+    <t>Tartu PP</t>
+  </si>
+  <si>
+    <t>Parnu PP</t>
+  </si>
+  <si>
+    <t>ep_bioenergy_imavere</t>
+  </si>
+  <si>
+    <t>Imavere CHP</t>
+  </si>
+  <si>
+    <t>ep_bioenergy_osula</t>
+  </si>
+  <si>
+    <t>Osula CHP</t>
+  </si>
+  <si>
+    <t>ep_bioenergy_sillamae1</t>
+  </si>
+  <si>
+    <t>Sillamae 1 CHP</t>
+  </si>
+  <si>
+    <t>Sillamae 2 CHP</t>
+  </si>
+  <si>
+    <t>Pohja TPP</t>
+  </si>
+  <si>
+    <t>Sillamae TPP</t>
+  </si>
+  <si>
+    <t>Auvere PP</t>
+  </si>
+  <si>
+    <t>ep_bioenergy_helme</t>
+  </si>
+  <si>
+    <t>Helme CHP</t>
+  </si>
+  <si>
+    <t>Grune Fee Eesti AS</t>
+  </si>
+  <si>
+    <t>Kivioli Keemiatoostuse OU TPP</t>
+  </si>
+  <si>
+    <t>ep_gas_gas_turbine_grune</t>
+  </si>
+  <si>
+    <t>ep_gas_gas_turbine_sillamae2</t>
+  </si>
+  <si>
+    <t>ep_bioenergy_mustamae</t>
+  </si>
+  <si>
+    <t>Mustamae CHP</t>
+  </si>
+  <si>
+    <t>ep_bioenergy_kuressaare</t>
+  </si>
+  <si>
+    <t>Kuressare CHP</t>
+  </si>
+  <si>
+    <t>ep_bioenergy_paide</t>
+  </si>
+  <si>
+    <t>Paide CHP</t>
+  </si>
+  <si>
+    <t>ep_gas_gas_turbine_jamejala</t>
+  </si>
+  <si>
+    <t>Jamejala CHP</t>
+  </si>
+  <si>
+    <t>ep_gas_gas_turbine_pussi</t>
+  </si>
+  <si>
+    <t>Pussi CHP</t>
+  </si>
+  <si>
+    <t>ep_bioenergy_ilmatsalu</t>
+  </si>
+  <si>
+    <t>Ilmatsalu CHP</t>
+  </si>
+  <si>
+    <t>ep_bioenergy_vinni</t>
+  </si>
+  <si>
+    <t>Vinni CHP</t>
+  </si>
+  <si>
+    <t>ep_bioenergy_oisu</t>
+  </si>
+  <si>
+    <t>Oisu CHP</t>
+  </si>
+  <si>
+    <t>ep_bioenergy_tlnprugilagaas</t>
+  </si>
+  <si>
+    <t>ep_bioenergy_rakverepaikese</t>
+  </si>
+  <si>
+    <t>Tallinna Prugilagaas OU CHP</t>
+  </si>
+  <si>
+    <t>Rakvere Paikese CHP</t>
+  </si>
+  <si>
+    <t>ep_bioenergy_tartuaardlapalu</t>
+  </si>
+  <si>
+    <t>Tartu Aardlapalu CHP</t>
+  </si>
+  <si>
+    <t>coal</t>
+  </si>
+  <si>
+    <t>ep_coal_cfb_balti</t>
+  </si>
+  <si>
+    <t>ep_coal_cfb_auvere</t>
+  </si>
+  <si>
+    <t>ep_coal_cfb_enefit</t>
+  </si>
+  <si>
+    <t>ep_coal_cfb_eesti</t>
+  </si>
+  <si>
+    <t>ep_coal_cfb_sillamae</t>
+  </si>
+  <si>
+    <t>ep_coal_cfb_kivioli</t>
+  </si>
+  <si>
+    <t>en_a_coal_cfb_G100001030965</t>
+  </si>
+  <si>
+    <t>en_a_coal_cfb_G100001030961</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="169" formatCode="0.0"/>
+  </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -559,9 +758,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -902,18 +1104,31 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="J11" dT="2026-01-27T14:26:51.36" personId="{9CD26280-DD25-46DF-A708-6877D8A68AD8}" id="{3057E3B1-7BF3-4718-B31B-0585028D4313}">
+  <threadedComment ref="F11" dT="2026-01-22T14:00:05.64" personId="{9CD26280-DD25-46DF-A708-6877D8A68AD8}" id="{E45DD652-654C-4828-8A13-679EDDC53E65}">
+    <text>Iru produces only 17 MW in 2025 not 0.207 GW</text>
+  </threadedComment>
+  <threadedComment ref="G46" dT="2026-01-28T09:05:36.66" personId="{9CD26280-DD25-46DF-A708-6877D8A68AD8}" id="{06D70610-96F7-4BDA-B071-69925D70228B}">
+    <text>Danish Energy agency - coal CHP 2020</text>
+  </threadedComment>
+  <threadedComment ref="G49" dT="2026-01-28T11:16:21.05" personId="{9CD26280-DD25-46DF-A708-6877D8A68AD8}" id="{A1B9CC12-DC46-488C-9BF3-3F8DFC23199D}">
+    <text xml:space="preserve">DAE - gas engines 2020
+</text>
+  </threadedComment>
+  <threadedComment ref="G50" dT="2026-01-28T11:17:46.06" personId="{9CD26280-DD25-46DF-A708-6877D8A68AD8}" id="{4E0E017D-BAC7-4AA8-B401-A7330F2C0996}">
+    <text>DAE - Wood pellets, Medium 2020</text>
+  </threadedComment>
+  <threadedComment ref="N77" dT="2026-01-28T08:41:02.80" personId="{9CD26280-DD25-46DF-A708-6877D8A68AD8}" id="{1905391B-2A5F-4643-B2AC-720AD8410CDA}">
+    <text>Frequency reserve</text>
+  </threadedComment>
+  <threadedComment ref="J80" dT="2026-01-27T14:26:51.36" personId="{9CD26280-DD25-46DF-A708-6877D8A68AD8}" id="{3057E3B1-7BF3-4718-B31B-0585028D4313}">
     <text>From 9,24 to 6</text>
-  </threadedComment>
-  <threadedComment ref="F13" dT="2026-01-22T14:00:05.64" personId="{9CD26280-DD25-46DF-A708-6877D8A68AD8}" id="{E45DD652-654C-4828-8A13-679EDDC53E65}">
-    <text>Iru produces only 17 MW in 2025 not 0.207 GW</text>
   </threadedComment>
 </ThreadedComments>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C047CB67-FC18-43CA-8AA0-0CA09A11D4D8}">
-  <dimension ref="B9:T15"/>
+  <dimension ref="B9:T17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="46.7109375" bestFit="1" customWidth="1"/>
@@ -985,121 +1200,9 @@
         <v>68</v>
       </c>
     </row>
-    <row r="11" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="B11" t="s">
-        <v>130</v>
-      </c>
-      <c r="C11" t="s">
-        <v>16</v>
-      </c>
-      <c r="D11" t="s">
-        <v>14</v>
-      </c>
-      <c r="E11">
-        <v>0.52272499999999988</v>
-      </c>
-      <c r="F11">
-        <v>1365</v>
-      </c>
-      <c r="G11">
-        <v>34.200000000000003</v>
-      </c>
-      <c r="H11">
-        <v>3.75</v>
-      </c>
-      <c r="I11">
-        <v>0.84455000000000002</v>
-      </c>
-      <c r="J11" t="s">
-        <v>84</v>
-      </c>
-      <c r="K11">
-        <v>1</v>
-      </c>
-      <c r="L11">
-        <v>20</v>
-      </c>
-      <c r="N11" t="s">
-        <v>69</v>
-      </c>
-      <c r="O11" t="s">
-        <v>130</v>
-      </c>
-      <c r="P11" t="s">
-        <v>135</v>
-      </c>
-      <c r="Q11" t="s">
-        <v>71</v>
-      </c>
-      <c r="R11" t="s">
-        <v>72</v>
-      </c>
-      <c r="S11" t="s">
-        <v>73</v>
-      </c>
-      <c r="T11" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="12" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="B12" t="s">
-        <v>131</v>
-      </c>
-      <c r="C12" t="s">
-        <v>16</v>
-      </c>
-      <c r="D12" t="s">
-        <v>14</v>
-      </c>
-      <c r="E12">
-        <v>0.52272499999999988</v>
-      </c>
-      <c r="F12">
-        <v>1365</v>
-      </c>
-      <c r="G12">
-        <v>34.200000000000003</v>
-      </c>
-      <c r="H12">
-        <v>3.75</v>
-      </c>
-      <c r="I12">
-        <v>0.84455000000000002</v>
-      </c>
-      <c r="J12" t="s">
-        <v>85</v>
-      </c>
-      <c r="K12">
-        <v>1</v>
-      </c>
-      <c r="L12">
-        <v>20</v>
-      </c>
-      <c r="N12" t="s">
-        <v>69</v>
-      </c>
-      <c r="O12" t="s">
-        <v>131</v>
-      </c>
-      <c r="P12" t="s">
-        <v>136</v>
-      </c>
-      <c r="Q12" t="s">
-        <v>71</v>
-      </c>
-      <c r="R12" t="s">
-        <v>72</v>
-      </c>
-      <c r="S12" t="s">
-        <v>73</v>
-      </c>
-      <c r="T12" t="s">
-        <v>77</v>
-      </c>
-    </row>
     <row r="13" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C13" t="s">
         <v>16</v>
@@ -1108,7 +1211,7 @@
         <v>14</v>
       </c>
       <c r="E13">
-        <v>0.28982625000000001</v>
+        <v>0.52272499999999988</v>
       </c>
       <c r="F13">
         <v>1365</v>
@@ -1123,7 +1226,7 @@
         <v>0.84455000000000002</v>
       </c>
       <c r="J13" t="s">
-        <v>15</v>
+        <v>84</v>
       </c>
       <c r="K13">
         <v>1</v>
@@ -1135,10 +1238,10 @@
         <v>69</v>
       </c>
       <c r="O13" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="P13" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="Q13" t="s">
         <v>71</v>
@@ -1155,7 +1258,7 @@
     </row>
     <row r="14" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="C14" t="s">
         <v>16</v>
@@ -1164,7 +1267,7 @@
         <v>14</v>
       </c>
       <c r="E14">
-        <v>0.38753750000000003</v>
+        <v>0.52272499999999988</v>
       </c>
       <c r="F14">
         <v>1365</v>
@@ -1179,7 +1282,7 @@
         <v>0.84455000000000002</v>
       </c>
       <c r="J14" t="s">
-        <v>17</v>
+        <v>85</v>
       </c>
       <c r="K14">
         <v>1</v>
@@ -1191,10 +1294,10 @@
         <v>69</v>
       </c>
       <c r="O14" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="P14" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="Q14" t="s">
         <v>71</v>
@@ -1211,16 +1314,16 @@
     </row>
     <row r="15" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="C15" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="D15" t="s">
         <v>14</v>
       </c>
       <c r="E15">
-        <v>0.31543749999999998</v>
+        <v>0.28982625000000001</v>
       </c>
       <c r="F15">
         <v>1365</v>
@@ -1235,7 +1338,7 @@
         <v>0.84455000000000002</v>
       </c>
       <c r="J15" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="K15">
         <v>1</v>
@@ -1247,10 +1350,10 @@
         <v>69</v>
       </c>
       <c r="O15" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="P15" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="Q15" t="s">
         <v>71</v>
@@ -1262,6 +1365,118 @@
         <v>73</v>
       </c>
       <c r="T15" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="16" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B16" t="s">
+        <v>133</v>
+      </c>
+      <c r="C16" t="s">
+        <v>16</v>
+      </c>
+      <c r="D16" t="s">
+        <v>14</v>
+      </c>
+      <c r="E16">
+        <v>0.38753750000000003</v>
+      </c>
+      <c r="F16">
+        <v>1365</v>
+      </c>
+      <c r="G16">
+        <v>34.200000000000003</v>
+      </c>
+      <c r="H16">
+        <v>3.75</v>
+      </c>
+      <c r="I16">
+        <v>0.84455000000000002</v>
+      </c>
+      <c r="J16" t="s">
+        <v>17</v>
+      </c>
+      <c r="K16">
+        <v>1</v>
+      </c>
+      <c r="L16">
+        <v>20</v>
+      </c>
+      <c r="N16" t="s">
+        <v>69</v>
+      </c>
+      <c r="O16" t="s">
+        <v>133</v>
+      </c>
+      <c r="P16" t="s">
+        <v>138</v>
+      </c>
+      <c r="Q16" t="s">
+        <v>71</v>
+      </c>
+      <c r="R16" t="s">
+        <v>72</v>
+      </c>
+      <c r="S16" t="s">
+        <v>73</v>
+      </c>
+      <c r="T16" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="17" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B17" t="s">
+        <v>134</v>
+      </c>
+      <c r="C17" t="s">
+        <v>21</v>
+      </c>
+      <c r="D17" t="s">
+        <v>14</v>
+      </c>
+      <c r="E17">
+        <v>0.31543749999999998</v>
+      </c>
+      <c r="F17">
+        <v>1365</v>
+      </c>
+      <c r="G17">
+        <v>34.200000000000003</v>
+      </c>
+      <c r="H17">
+        <v>3.75</v>
+      </c>
+      <c r="I17">
+        <v>0.84455000000000002</v>
+      </c>
+      <c r="J17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K17">
+        <v>1</v>
+      </c>
+      <c r="L17">
+        <v>20</v>
+      </c>
+      <c r="N17" t="s">
+        <v>69</v>
+      </c>
+      <c r="O17" t="s">
+        <v>134</v>
+      </c>
+      <c r="P17" t="s">
+        <v>139</v>
+      </c>
+      <c r="Q17" t="s">
+        <v>71</v>
+      </c>
+      <c r="R17" t="s">
+        <v>72</v>
+      </c>
+      <c r="S17" t="s">
+        <v>73</v>
+      </c>
+      <c r="T17" t="s">
         <v>77</v>
       </c>
     </row>
@@ -1276,6 +1491,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="39.28515625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="39.28515625" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="48.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1345,10 +1561,10 @@
     </row>
     <row r="11" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
-        <v>84</v>
+        <v>200</v>
       </c>
       <c r="C11" t="s">
-        <v>16</v>
+        <v>192</v>
       </c>
       <c r="D11" t="s">
         <v>14</v>
@@ -1363,13 +1579,13 @@
         <v>0.59739999999999993</v>
       </c>
       <c r="H11">
-        <v>1265</v>
-      </c>
-      <c r="I11">
-        <v>36.300000000000004</v>
+        <v>2150</v>
+      </c>
+      <c r="I11" s="3">
+        <v>35.053609999999999</v>
       </c>
       <c r="J11">
-        <v>3.4650000000000007</v>
+        <v>3.28</v>
       </c>
       <c r="K11">
         <v>50</v>
@@ -1378,7 +1594,7 @@
         <v>69</v>
       </c>
       <c r="O11" t="s">
-        <v>84</v>
+        <v>200</v>
       </c>
       <c r="P11" t="s">
         <v>108</v>
@@ -1398,10 +1614,10 @@
     </row>
     <row r="12" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
-        <v>85</v>
+        <v>199</v>
       </c>
       <c r="C12" t="s">
-        <v>16</v>
+        <v>192</v>
       </c>
       <c r="D12" t="s">
         <v>14</v>
@@ -1416,13 +1632,13 @@
         <v>0.59739999999999993</v>
       </c>
       <c r="H12">
-        <v>1265</v>
-      </c>
-      <c r="I12">
-        <v>36.300000000000004</v>
+        <v>2150</v>
+      </c>
+      <c r="I12" s="3">
+        <v>35.053609999999999</v>
       </c>
       <c r="J12">
-        <v>3.4650000000000007</v>
+        <v>3.28</v>
       </c>
       <c r="K12">
         <v>50</v>
@@ -1431,7 +1647,7 @@
         <v>69</v>
       </c>
       <c r="O12" t="s">
-        <v>85</v>
+        <v>199</v>
       </c>
       <c r="P12" t="s">
         <v>109</v>
@@ -2340,17 +2556,19 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A79DDA4A-BC9F-4D47-BDC9-53442001A438}">
-  <dimension ref="B9:T51"/>
+  <dimension ref="B9:T80"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="40.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.85546875" customWidth="1"/>
+    <col min="4" max="4" width="12.140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="9.28515625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="12.5703125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="9.28515625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.85546875" style="3" bestFit="1" customWidth="1"/>
     <col min="10" max="11" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12" bestFit="1" customWidth="1"/>
+    <col min="12" max="13" width="12" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="40.5703125" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="64.42578125" bestFit="1" customWidth="1"/>
   </cols>
@@ -2385,7 +2603,7 @@
       <c r="H10" t="s">
         <v>7</v>
       </c>
-      <c r="I10" t="s">
+      <c r="I10" s="3" t="s">
         <v>8</v>
       </c>
       <c r="J10" t="s">
@@ -2421,43 +2639,43 @@
     </row>
     <row r="11" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="C11" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="D11" t="s">
         <v>14</v>
       </c>
       <c r="E11">
-        <v>2022</v>
+        <v>1982</v>
       </c>
       <c r="F11">
-        <v>0.3</v>
+        <v>1.6999999999999999E-3</v>
       </c>
       <c r="G11">
-        <v>0.33990000000000004</v>
+        <v>0.44290000000000002</v>
       </c>
       <c r="H11">
-        <v>4427.5</v>
-      </c>
-      <c r="I11">
-        <v>157.30000000000001</v>
+        <v>1265</v>
+      </c>
+      <c r="I11" s="3">
+        <v>36.300000000000004</v>
       </c>
       <c r="J11">
-        <v>6</v>
+        <v>3.4650000000000007</v>
       </c>
       <c r="K11">
-        <v>50</v>
+        <v>73</v>
       </c>
       <c r="N11" t="s">
         <v>69</v>
       </c>
       <c r="O11" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="P11" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="Q11" t="s">
         <v>71</v>
@@ -2469,36 +2687,39 @@
         <v>73</v>
       </c>
       <c r="T11" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="12" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="C12" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="D12" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E12">
         <v>2022</v>
       </c>
       <c r="F12">
-        <v>0.21299999999999999</v>
+        <v>4.3091615634383719E-2</v>
       </c>
       <c r="G12">
         <v>0.33123000000000002</v>
       </c>
+      <c r="L12">
+        <v>0.14986856628506873</v>
+      </c>
       <c r="N12" t="s">
         <v>69</v>
       </c>
       <c r="O12" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="P12" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="Q12" t="s">
         <v>71</v>
@@ -2507,7 +2728,7 @@
         <v>72</v>
       </c>
       <c r="S12" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="T12" t="s">
         <v>74</v>
@@ -2515,43 +2736,34 @@
     </row>
     <row r="13" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="C13" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="D13" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="E13">
-        <v>1982</v>
+        <v>2022</v>
       </c>
       <c r="F13">
-        <v>0.20699999999999999</v>
+        <v>4.3344722222460344E-2</v>
       </c>
       <c r="G13">
-        <v>0.44290000000000002</v>
-      </c>
-      <c r="H13">
-        <v>1265</v>
-      </c>
-      <c r="I13">
-        <v>36.300000000000004</v>
-      </c>
-      <c r="J13">
-        <v>3.4650000000000007</v>
-      </c>
-      <c r="K13">
-        <v>73</v>
+        <v>0.33123000000000002</v>
+      </c>
+      <c r="L13">
+        <v>0.14986856628506873</v>
       </c>
       <c r="N13" t="s">
         <v>69</v>
       </c>
       <c r="O13" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="P13" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="Q13" t="s">
         <v>71</v>
@@ -2560,36 +2772,39 @@
         <v>72</v>
       </c>
       <c r="S13" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="T13" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="14" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="C14" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="D14" t="s">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="E14">
         <v>2022</v>
       </c>
       <c r="F14">
-        <v>8.0000000000000002E-3</v>
+        <v>3.9363662143155967E-2</v>
       </c>
       <c r="G14">
         <v>0.33123000000000002</v>
       </c>
+      <c r="L14">
+        <v>0.14986856628506873</v>
+      </c>
       <c r="N14" t="s">
         <v>69</v>
       </c>
       <c r="O14" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="P14" t="s">
         <v>78</v>
@@ -2601,7 +2816,7 @@
         <v>72</v>
       </c>
       <c r="S14" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="T14" t="s">
         <v>74</v>
@@ -2609,43 +2824,46 @@
     </row>
     <row r="15" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="C15" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D15" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E15">
-        <v>2013</v>
+        <v>2015</v>
       </c>
       <c r="F15">
-        <v>0.25109999999999999</v>
+        <v>7.6700000000000004E-2</v>
       </c>
       <c r="G15">
-        <v>0.36049999999999999</v>
+        <v>1</v>
       </c>
       <c r="H15">
-        <v>1265</v>
-      </c>
-      <c r="I15">
-        <v>48.400000000000006</v>
+        <v>1336.4999999999998</v>
+      </c>
+      <c r="I15" s="3">
+        <v>21.45</v>
       </c>
       <c r="J15">
-        <v>7.5075000000000003</v>
+        <v>0</v>
       </c>
       <c r="K15">
-        <v>42</v>
+        <v>40</v>
+      </c>
+      <c r="L15">
+        <v>0.1461854238754417</v>
       </c>
       <c r="N15" t="s">
         <v>69</v>
       </c>
       <c r="O15" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="P15" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="Q15" t="s">
         <v>71</v>
@@ -2654,15 +2872,15 @@
         <v>72</v>
       </c>
       <c r="S15" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="T15" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="16" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="C16" t="s">
         <v>23</v>
@@ -2671,22 +2889,34 @@
         <v>24</v>
       </c>
       <c r="E16">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="F16">
-        <v>4.3091615634383719E-2</v>
+        <v>3.2000000000000001E-2</v>
       </c>
       <c r="G16">
-        <v>0.33123000000000002</v>
+        <v>1</v>
+      </c>
+      <c r="H16">
+        <v>1336.5</v>
+      </c>
+      <c r="I16" s="3">
+        <v>21.450000000000003</v>
+      </c>
+      <c r="J16">
+        <v>0</v>
+      </c>
+      <c r="K16">
+        <v>32</v>
       </c>
       <c r="L16">
-        <v>0.14986856628506873</v>
+        <v>0.1461854238754417</v>
       </c>
       <c r="N16" t="s">
         <v>69</v>
       </c>
       <c r="O16" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="P16" t="s">
         <v>78</v>
@@ -2706,31 +2936,43 @@
     </row>
     <row r="17" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="C17" t="s">
         <v>23</v>
       </c>
       <c r="D17" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="E17">
-        <v>2022</v>
+        <v>2015</v>
       </c>
       <c r="F17">
-        <v>4.3344722222460344E-2</v>
+        <v>5.8200000000000002E-2</v>
       </c>
       <c r="G17">
-        <v>0.33123000000000002</v>
+        <v>1</v>
+      </c>
+      <c r="H17">
+        <v>1336.5</v>
+      </c>
+      <c r="I17" s="3">
+        <v>21.450000000000003</v>
+      </c>
+      <c r="J17">
+        <v>0</v>
+      </c>
+      <c r="K17">
+        <v>40</v>
       </c>
       <c r="L17">
-        <v>0.14986856628506873</v>
+        <v>0.14867925344692126</v>
       </c>
       <c r="N17" t="s">
         <v>69</v>
       </c>
       <c r="O17" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="P17" t="s">
         <v>78</v>
@@ -2750,31 +2992,43 @@
     </row>
     <row r="18" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="C18" t="s">
         <v>23</v>
       </c>
       <c r="D18" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="E18">
-        <v>2022</v>
+        <v>2015</v>
       </c>
       <c r="F18">
-        <v>3.9363662143155967E-2</v>
+        <v>2.9599999999999998E-2</v>
       </c>
       <c r="G18">
-        <v>0.33123000000000002</v>
+        <v>1</v>
+      </c>
+      <c r="H18">
+        <v>1336.5000000000002</v>
+      </c>
+      <c r="I18" s="3">
+        <v>21.450000000000003</v>
+      </c>
+      <c r="J18">
+        <v>0</v>
+      </c>
+      <c r="K18">
+        <v>40</v>
       </c>
       <c r="L18">
-        <v>0.14986856628506873</v>
+        <v>0.14701259708091721</v>
       </c>
       <c r="N18" t="s">
         <v>69</v>
       </c>
       <c r="O18" t="s">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="P18" t="s">
         <v>78</v>
@@ -2794,19 +3048,19 @@
     </row>
     <row r="19" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="C19" t="s">
         <v>23</v>
       </c>
       <c r="D19" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E19">
         <v>2015</v>
       </c>
       <c r="F19">
-        <v>7.6700000000000004E-2</v>
+        <v>5.3800000000000008E-2</v>
       </c>
       <c r="G19">
         <v>1</v>
@@ -2814,7 +3068,7 @@
       <c r="H19">
         <v>1336.4999999999998</v>
       </c>
-      <c r="I19">
+      <c r="I19" s="3">
         <v>21.45</v>
       </c>
       <c r="J19">
@@ -2824,13 +3078,13 @@
         <v>40</v>
       </c>
       <c r="L19">
-        <v>0.1461854238754417</v>
+        <v>0.15309859852159369</v>
       </c>
       <c r="N19" t="s">
         <v>69</v>
       </c>
       <c r="O19" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="P19" t="s">
         <v>78</v>
@@ -2850,43 +3104,43 @@
     </row>
     <row r="20" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B20" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="C20" t="s">
         <v>23</v>
       </c>
       <c r="D20" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E20">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="F20">
-        <v>3.2000000000000001E-2</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="G20">
         <v>1</v>
       </c>
       <c r="H20">
-        <v>1336.5</v>
-      </c>
-      <c r="I20">
-        <v>21.450000000000003</v>
+        <v>1138.5</v>
+      </c>
+      <c r="I20" s="3">
+        <v>18.150000000000002</v>
       </c>
       <c r="J20">
         <v>0</v>
       </c>
       <c r="K20">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="L20">
-        <v>0.1461854238754417</v>
+        <v>0.15309859852159369</v>
       </c>
       <c r="N20" t="s">
         <v>69</v>
       </c>
       <c r="O20" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="P20" t="s">
         <v>78</v>
@@ -2906,19 +3160,19 @@
     </row>
     <row r="21" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B21" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="C21" t="s">
         <v>23</v>
       </c>
       <c r="D21" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="E21">
         <v>2015</v>
       </c>
       <c r="F21">
-        <v>5.8200000000000002E-2</v>
+        <v>7.3000000000000009E-3</v>
       </c>
       <c r="G21">
         <v>1</v>
@@ -2926,8 +3180,8 @@
       <c r="H21">
         <v>1336.5</v>
       </c>
-      <c r="I21">
-        <v>21.450000000000003</v>
+      <c r="I21" s="3">
+        <v>21.45</v>
       </c>
       <c r="J21">
         <v>0</v>
@@ -2936,13 +3190,13 @@
         <v>40</v>
       </c>
       <c r="L21">
-        <v>0.14867925344692126</v>
+        <v>0.15619560585976827</v>
       </c>
       <c r="N21" t="s">
         <v>69</v>
       </c>
       <c r="O21" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="P21" t="s">
         <v>78</v>
@@ -2962,27 +3216,27 @@
     </row>
     <row r="22" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B22" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="C22" t="s">
         <v>23</v>
       </c>
       <c r="D22" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="E22">
         <v>2015</v>
       </c>
       <c r="F22">
-        <v>2.9599999999999998E-2</v>
+        <v>2.81E-2</v>
       </c>
       <c r="G22">
         <v>1</v>
       </c>
       <c r="H22">
-        <v>1336.5000000000002</v>
-      </c>
-      <c r="I22">
+        <v>1336.5</v>
+      </c>
+      <c r="I22" s="3">
         <v>21.450000000000003</v>
       </c>
       <c r="J22">
@@ -2992,13 +3246,13 @@
         <v>40</v>
       </c>
       <c r="L22">
-        <v>0.14701259708091721</v>
+        <v>0.14537310453496291</v>
       </c>
       <c r="N22" t="s">
         <v>69</v>
       </c>
       <c r="O22" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="P22" t="s">
         <v>78</v>
@@ -3018,28 +3272,28 @@
     </row>
     <row r="23" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B23" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="C23" t="s">
         <v>23</v>
       </c>
       <c r="D23" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E23">
         <v>2015</v>
       </c>
       <c r="F23">
-        <v>5.3800000000000008E-2</v>
+        <v>8.4900000000000003E-2</v>
       </c>
       <c r="G23">
         <v>1</v>
       </c>
       <c r="H23">
-        <v>1336.4999999999998</v>
-      </c>
-      <c r="I23">
-        <v>21.45</v>
+        <v>1336.5</v>
+      </c>
+      <c r="I23" s="3">
+        <v>21.450000000000003</v>
       </c>
       <c r="J23">
         <v>0</v>
@@ -3048,13 +3302,13 @@
         <v>40</v>
       </c>
       <c r="L23">
-        <v>0.15309859852159369</v>
+        <v>0.14763873655681015</v>
       </c>
       <c r="N23" t="s">
         <v>69</v>
       </c>
       <c r="O23" t="s">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="P23" t="s">
         <v>78</v>
@@ -3074,43 +3328,43 @@
     </row>
     <row r="24" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B24" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C24" t="s">
         <v>23</v>
       </c>
       <c r="D24" t="s">
-        <v>26</v>
+        <v>41</v>
       </c>
       <c r="E24">
-        <v>2024</v>
+        <v>2015</v>
       </c>
       <c r="F24">
-        <v>7.0000000000000007E-2</v>
+        <v>5.2399999999999995E-2</v>
       </c>
       <c r="G24">
         <v>1</v>
       </c>
       <c r="H24">
-        <v>1138.5</v>
-      </c>
-      <c r="I24">
-        <v>18.150000000000002</v>
+        <v>1336.5000000000002</v>
+      </c>
+      <c r="I24" s="3">
+        <v>21.45</v>
       </c>
       <c r="J24">
         <v>0</v>
       </c>
       <c r="K24">
-        <v>31</v>
+        <v>40</v>
       </c>
       <c r="L24">
-        <v>0.15309859852159369</v>
+        <v>0.1532628310027955</v>
       </c>
       <c r="N24" t="s">
         <v>69</v>
       </c>
       <c r="O24" t="s">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="P24" t="s">
         <v>78</v>
@@ -3130,19 +3384,19 @@
     </row>
     <row r="25" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B25" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="C25" t="s">
         <v>23</v>
       </c>
       <c r="D25" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="E25">
-        <v>2015</v>
+        <v>2023</v>
       </c>
       <c r="F25">
-        <v>7.3000000000000009E-3</v>
+        <v>0.02</v>
       </c>
       <c r="G25">
         <v>1</v>
@@ -3150,23 +3404,23 @@
       <c r="H25">
         <v>1336.5</v>
       </c>
-      <c r="I25">
-        <v>21.45</v>
+      <c r="I25" s="3">
+        <v>21.450000000000003</v>
       </c>
       <c r="J25">
         <v>0</v>
       </c>
       <c r="K25">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="L25">
-        <v>0.15619560585976827</v>
+        <v>0.1532628310027955</v>
       </c>
       <c r="N25" t="s">
         <v>69</v>
       </c>
       <c r="O25" t="s">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="P25" t="s">
         <v>78</v>
@@ -3186,19 +3440,19 @@
     </row>
     <row r="26" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B26" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="C26" t="s">
         <v>23</v>
       </c>
       <c r="D26" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="E26">
         <v>2015</v>
       </c>
       <c r="F26">
-        <v>2.81E-2</v>
+        <v>3.2000000000000002E-3</v>
       </c>
       <c r="G26">
         <v>1</v>
@@ -3206,7 +3460,7 @@
       <c r="H26">
         <v>1336.5</v>
       </c>
-      <c r="I26">
+      <c r="I26" s="3">
         <v>21.450000000000003</v>
       </c>
       <c r="J26">
@@ -3216,13 +3470,13 @@
         <v>40</v>
       </c>
       <c r="L26">
-        <v>0.14537310453496291</v>
+        <v>0.1451997589052581</v>
       </c>
       <c r="N26" t="s">
         <v>69</v>
       </c>
       <c r="O26" t="s">
-        <v>40</v>
+        <v>49</v>
       </c>
       <c r="P26" t="s">
         <v>78</v>
@@ -3242,43 +3496,31 @@
     </row>
     <row r="27" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B27" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="C27" t="s">
-        <v>23</v>
+        <v>45</v>
       </c>
       <c r="D27" t="s">
-        <v>28</v>
+        <v>46</v>
       </c>
       <c r="E27">
-        <v>2015</v>
+        <v>2022</v>
       </c>
       <c r="F27">
-        <v>8.4900000000000003E-2</v>
+        <v>1.5040605442498314E-2</v>
       </c>
       <c r="G27">
-        <v>1</v>
-      </c>
-      <c r="H27">
-        <v>1336.5</v>
-      </c>
-      <c r="I27">
-        <v>21.450000000000003</v>
-      </c>
-      <c r="J27">
-        <v>0</v>
-      </c>
-      <c r="K27">
-        <v>40</v>
+        <v>0.33123000000000002</v>
       </c>
       <c r="L27">
-        <v>0.14763873655681015</v>
+        <v>0.42012333946150526</v>
       </c>
       <c r="N27" t="s">
         <v>69</v>
       </c>
       <c r="O27" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="P27" t="s">
         <v>78</v>
@@ -3298,43 +3540,31 @@
     </row>
     <row r="28" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B28" t="s">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="C28" t="s">
-        <v>23</v>
+        <v>45</v>
       </c>
       <c r="D28" t="s">
-        <v>41</v>
+        <v>48</v>
       </c>
       <c r="E28">
-        <v>2015</v>
+        <v>2022</v>
       </c>
       <c r="F28">
-        <v>5.2399999999999995E-2</v>
+        <v>1.5497656626156837E-2</v>
       </c>
       <c r="G28">
-        <v>1</v>
-      </c>
-      <c r="H28">
-        <v>1336.5000000000002</v>
-      </c>
-      <c r="I28">
-        <v>21.45</v>
-      </c>
-      <c r="J28">
-        <v>0</v>
-      </c>
-      <c r="K28">
-        <v>40</v>
+        <v>0.33123000000000002</v>
       </c>
       <c r="L28">
-        <v>0.1532628310027955</v>
+        <v>0.42012333946150526</v>
       </c>
       <c r="N28" t="s">
         <v>69</v>
       </c>
       <c r="O28" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="P28" t="s">
         <v>78</v>
@@ -3354,43 +3584,31 @@
     </row>
     <row r="29" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B29" t="s">
-        <v>40</v>
+        <v>49</v>
       </c>
       <c r="C29" t="s">
-        <v>23</v>
+        <v>45</v>
       </c>
       <c r="D29" t="s">
-        <v>41</v>
+        <v>50</v>
       </c>
       <c r="E29">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="F29">
-        <v>0.02</v>
+        <v>1.4461737931344828E-2</v>
       </c>
       <c r="G29">
-        <v>1</v>
-      </c>
-      <c r="H29">
-        <v>1336.5</v>
-      </c>
-      <c r="I29">
-        <v>21.450000000000003</v>
-      </c>
-      <c r="J29">
-        <v>0</v>
-      </c>
-      <c r="K29">
-        <v>32</v>
+        <v>0.33123000000000002</v>
       </c>
       <c r="L29">
-        <v>0.1532628310027955</v>
+        <v>0.42012333946150526</v>
       </c>
       <c r="N29" t="s">
         <v>69</v>
       </c>
       <c r="O29" t="s">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="P29" t="s">
         <v>78</v>
@@ -3410,43 +3628,43 @@
     </row>
     <row r="30" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B30" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="C30" t="s">
-        <v>23</v>
+        <v>45</v>
       </c>
       <c r="D30" t="s">
-        <v>43</v>
+        <v>52</v>
       </c>
       <c r="E30">
-        <v>2015</v>
+        <v>2009</v>
       </c>
       <c r="F30">
-        <v>3.2000000000000002E-3</v>
+        <v>3.9E-2</v>
       </c>
       <c r="G30">
         <v>1</v>
       </c>
       <c r="H30">
-        <v>1336.5</v>
-      </c>
-      <c r="I30">
-        <v>21.450000000000003</v>
+        <v>2376</v>
+      </c>
+      <c r="I30" s="3">
+        <v>57.2</v>
       </c>
       <c r="J30">
-        <v>0</v>
+        <v>2.52</v>
       </c>
       <c r="K30">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="L30">
-        <v>0.1451997589052581</v>
+        <v>0.47763777043344691</v>
       </c>
       <c r="N30" t="s">
         <v>69</v>
       </c>
       <c r="O30" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="P30" t="s">
         <v>78</v>
@@ -3466,31 +3684,43 @@
     </row>
     <row r="31" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B31" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="C31" t="s">
         <v>45</v>
       </c>
       <c r="D31" t="s">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="E31">
-        <v>2022</v>
+        <v>2010</v>
       </c>
       <c r="F31">
-        <v>1.5040605442498314E-2</v>
+        <v>1.6E-2</v>
       </c>
       <c r="G31">
-        <v>0.33123000000000002</v>
+        <v>1</v>
+      </c>
+      <c r="H31">
+        <v>2376</v>
+      </c>
+      <c r="I31" s="3">
+        <v>57.2</v>
+      </c>
+      <c r="J31">
+        <v>2.52</v>
+      </c>
+      <c r="K31">
+        <v>45</v>
       </c>
       <c r="L31">
-        <v>0.42012333946150526</v>
+        <v>0.47814004703314078</v>
       </c>
       <c r="N31" t="s">
         <v>69</v>
       </c>
       <c r="O31" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="P31" t="s">
         <v>78</v>
@@ -3510,34 +3740,46 @@
     </row>
     <row r="32" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B32" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="C32" t="s">
         <v>45</v>
       </c>
       <c r="D32" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="E32">
-        <v>2022</v>
+        <v>2015</v>
       </c>
       <c r="F32">
-        <v>1.5497656626156837E-2</v>
+        <v>1.7999999999999999E-2</v>
       </c>
       <c r="G32">
-        <v>0.33123000000000002</v>
+        <v>1</v>
+      </c>
+      <c r="H32">
+        <v>2376</v>
+      </c>
+      <c r="I32" s="3">
+        <v>57.20000000000001</v>
+      </c>
+      <c r="J32">
+        <v>2.52</v>
+      </c>
+      <c r="K32">
+        <v>40</v>
       </c>
       <c r="L32">
-        <v>0.42012333946150526</v>
+        <v>0.47814004703314084</v>
       </c>
       <c r="N32" t="s">
         <v>69</v>
       </c>
       <c r="O32" t="s">
-        <v>53</v>
+        <v>61</v>
       </c>
       <c r="P32" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="Q32" t="s">
         <v>71</v>
@@ -3549,68 +3791,65 @@
         <v>80</v>
       </c>
       <c r="T32" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="33" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B33" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="C33" t="s">
         <v>45</v>
       </c>
       <c r="D33" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="E33">
-        <v>2022</v>
+        <v>2020</v>
       </c>
       <c r="F33">
-        <v>1.4461737931344828E-2</v>
+        <v>1.2E-2</v>
       </c>
       <c r="G33">
-        <v>0.33123000000000002</v>
+        <v>1</v>
+      </c>
+      <c r="H33">
+        <v>2376</v>
+      </c>
+      <c r="I33" s="3">
+        <v>57.20000000000001</v>
+      </c>
+      <c r="J33">
+        <v>2.52</v>
+      </c>
+      <c r="K33">
+        <v>35</v>
       </c>
       <c r="L33">
-        <v>0.42012333946150526</v>
+        <v>0.47814004703314078</v>
       </c>
       <c r="N33" t="s">
-        <v>69</v>
-      </c>
-      <c r="O33" t="s">
-        <v>55</v>
-      </c>
-      <c r="P33" t="s">
-        <v>78</v>
-      </c>
-      <c r="Q33" t="s">
-        <v>71</v>
-      </c>
-      <c r="R33" t="s">
-        <v>72</v>
-      </c>
-      <c r="S33" t="s">
-        <v>80</v>
-      </c>
-      <c r="T33" t="s">
-        <v>74</v>
+        <v>140</v>
+      </c>
+      <c r="O33" s="1" t="s">
+        <v>141</v>
       </c>
     </row>
     <row r="34" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B34" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="C34" t="s">
         <v>45</v>
       </c>
       <c r="D34" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="E34">
-        <v>2009</v>
+        <v>2007</v>
       </c>
       <c r="F34">
-        <v>3.9E-2</v>
+        <v>2.1000000000000001E-2</v>
       </c>
       <c r="G34">
         <v>1</v>
@@ -3618,26 +3857,26 @@
       <c r="H34">
         <v>2376</v>
       </c>
-      <c r="I34">
+      <c r="I34" s="3">
         <v>57.2</v>
       </c>
       <c r="J34">
         <v>2.52</v>
       </c>
       <c r="K34">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="L34">
-        <v>0.47763777043344691</v>
+        <v>0.40144059976798208</v>
       </c>
       <c r="N34" t="s">
         <v>69</v>
       </c>
       <c r="O34" t="s">
-        <v>57</v>
+        <v>194</v>
       </c>
       <c r="P34" t="s">
-        <v>78</v>
+        <v>163</v>
       </c>
       <c r="Q34" t="s">
         <v>71</v>
@@ -3649,24 +3888,24 @@
         <v>80</v>
       </c>
       <c r="T34" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="35" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B35" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C35" t="s">
         <v>45</v>
       </c>
       <c r="D35" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="E35">
-        <v>2010</v>
+        <v>2011</v>
       </c>
       <c r="F35">
-        <v>1.6E-2</v>
+        <v>2.4E-2</v>
       </c>
       <c r="G35">
         <v>1</v>
@@ -3674,26 +3913,26 @@
       <c r="H35">
         <v>2376</v>
       </c>
-      <c r="I35">
-        <v>57.2</v>
+      <c r="I35" s="3">
+        <v>57.20000000000001</v>
       </c>
       <c r="J35">
         <v>2.52</v>
       </c>
       <c r="K35">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="L35">
-        <v>0.47814004703314078</v>
+        <v>0.40144059976798202</v>
       </c>
       <c r="N35" t="s">
         <v>69</v>
       </c>
       <c r="O35" t="s">
-        <v>59</v>
+        <v>193</v>
       </c>
       <c r="P35" t="s">
-        <v>78</v>
+        <v>148</v>
       </c>
       <c r="Q35" t="s">
         <v>71</v>
@@ -3705,24 +3944,24 @@
         <v>80</v>
       </c>
       <c r="T35" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="36" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B36" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C36" t="s">
         <v>45</v>
       </c>
       <c r="D36" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="E36">
-        <v>2015</v>
+        <v>2012</v>
       </c>
       <c r="F36">
-        <v>1.7999999999999999E-2</v>
+        <v>7.9000000000000001E-2</v>
       </c>
       <c r="G36">
         <v>1</v>
@@ -3730,26 +3969,26 @@
       <c r="H36">
         <v>2376</v>
       </c>
-      <c r="I36">
-        <v>57.20000000000001</v>
+      <c r="I36" s="3">
+        <v>57.2</v>
       </c>
       <c r="J36">
         <v>2.52</v>
       </c>
       <c r="K36">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="L36">
-        <v>0.47814004703314084</v>
+        <v>0.40144059976798202</v>
       </c>
       <c r="N36" t="s">
         <v>69</v>
       </c>
       <c r="O36" t="s">
-        <v>61</v>
+        <v>195</v>
       </c>
       <c r="P36" t="s">
-        <v>81</v>
+        <v>149</v>
       </c>
       <c r="Q36" t="s">
         <v>71</v>
@@ -3766,19 +4005,19 @@
     </row>
     <row r="37" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B37" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C37" t="s">
         <v>45</v>
       </c>
       <c r="D37" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="E37">
-        <v>2020</v>
+        <v>2023</v>
       </c>
       <c r="F37">
-        <v>1.2E-2</v>
+        <v>2.1000000000000001E-2</v>
       </c>
       <c r="G37">
         <v>1</v>
@@ -3786,23 +4025,38 @@
       <c r="H37">
         <v>2376</v>
       </c>
-      <c r="I37">
-        <v>57.20000000000001</v>
+      <c r="I37" s="3">
+        <v>57.2</v>
       </c>
       <c r="J37">
         <v>2.52</v>
       </c>
       <c r="K37">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="L37">
-        <v>0.47814004703314078</v>
+        <v>0.40144059976798208</v>
       </c>
       <c r="N37" t="s">
-        <v>140</v>
-      </c>
-      <c r="O37" s="1" t="s">
-        <v>141</v>
+        <v>69</v>
+      </c>
+      <c r="O37" t="s">
+        <v>196</v>
+      </c>
+      <c r="P37" t="s">
+        <v>150</v>
+      </c>
+      <c r="Q37" t="s">
+        <v>71</v>
+      </c>
+      <c r="R37" t="s">
+        <v>72</v>
+      </c>
+      <c r="S37" t="s">
+        <v>80</v>
+      </c>
+      <c r="T37" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="38" spans="2:20" x14ac:dyDescent="0.25">
@@ -3816,37 +4070,37 @@
         <v>56</v>
       </c>
       <c r="E38">
-        <v>2007</v>
+        <v>2024</v>
       </c>
       <c r="F38">
-        <v>2.1000000000000001E-2</v>
+        <v>0.10199999999999999</v>
       </c>
       <c r="G38">
         <v>1</v>
       </c>
       <c r="H38">
-        <v>2376</v>
-      </c>
-      <c r="I38">
-        <v>57.2</v>
+        <v>2024</v>
+      </c>
+      <c r="I38" s="3">
+        <v>48.4</v>
       </c>
       <c r="J38">
-        <v>2.52</v>
+        <v>2.3100000000000005</v>
       </c>
       <c r="K38">
-        <v>48</v>
+        <v>31</v>
       </c>
       <c r="L38">
-        <v>0.40144059976798208</v>
+        <v>0.40144059976798202</v>
       </c>
       <c r="N38" t="s">
         <v>69</v>
       </c>
       <c r="O38" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="P38" t="s">
-        <v>142</v>
+        <v>161</v>
       </c>
       <c r="Q38" t="s">
         <v>71</v>
@@ -3863,19 +4117,19 @@
     </row>
     <row r="39" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B39" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C39" t="s">
         <v>45</v>
       </c>
       <c r="D39" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="E39">
-        <v>2011</v>
+        <v>2023</v>
       </c>
       <c r="F39">
-        <v>2.4E-2</v>
+        <v>3.9E-2</v>
       </c>
       <c r="G39">
         <v>1</v>
@@ -3883,26 +4137,26 @@
       <c r="H39">
         <v>2376</v>
       </c>
-      <c r="I39">
-        <v>57.20000000000001</v>
+      <c r="I39" s="3">
+        <v>57.2</v>
       </c>
       <c r="J39">
         <v>2.52</v>
       </c>
       <c r="K39">
-        <v>44</v>
+        <v>32</v>
       </c>
       <c r="L39">
-        <v>0.40144059976798202</v>
+        <v>0.365520596150406</v>
       </c>
       <c r="N39" t="s">
         <v>69</v>
       </c>
       <c r="O39" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="P39" t="s">
-        <v>143</v>
+        <v>151</v>
       </c>
       <c r="Q39" t="s">
         <v>71</v>
@@ -3919,19 +4173,19 @@
     </row>
     <row r="40" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B40" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="C40" t="s">
         <v>45</v>
       </c>
       <c r="D40" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="E40">
-        <v>2012</v>
+        <v>2005</v>
       </c>
       <c r="F40">
-        <v>7.9000000000000001E-2</v>
+        <v>1.7999999999999999E-2</v>
       </c>
       <c r="G40">
         <v>1</v>
@@ -3939,26 +4193,26 @@
       <c r="H40">
         <v>2376</v>
       </c>
-      <c r="I40">
-        <v>57.2</v>
+      <c r="I40" s="3">
+        <v>57.20000000000001</v>
       </c>
       <c r="J40">
         <v>2.52</v>
       </c>
       <c r="K40">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="L40">
-        <v>0.40144059976798202</v>
+        <v>0.41047488326249421</v>
       </c>
       <c r="N40" t="s">
         <v>69</v>
       </c>
       <c r="O40" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="P40" t="s">
-        <v>144</v>
+        <v>152</v>
       </c>
       <c r="Q40" t="s">
         <v>71</v>
@@ -3975,19 +4229,19 @@
     </row>
     <row r="41" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B41" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="C41" t="s">
         <v>45</v>
       </c>
       <c r="D41" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="E41">
-        <v>2023</v>
+        <v>2012</v>
       </c>
       <c r="F41">
-        <v>2.1000000000000001E-2</v>
+        <v>2.1999999999999999E-2</v>
       </c>
       <c r="G41">
         <v>1</v>
@@ -3995,57 +4249,99 @@
       <c r="H41">
         <v>2376</v>
       </c>
-      <c r="I41">
+      <c r="I41" s="3">
         <v>57.2</v>
       </c>
       <c r="J41">
         <v>2.52</v>
       </c>
       <c r="K41">
-        <v>32</v>
+        <v>43</v>
       </c>
       <c r="L41">
-        <v>0.40144059976798208</v>
+        <v>0.41047488326249421</v>
+      </c>
+      <c r="N41" t="s">
+        <v>69</v>
+      </c>
+      <c r="O41" t="s">
+        <v>145</v>
+      </c>
+      <c r="P41" t="s">
+        <v>153</v>
+      </c>
+      <c r="Q41" t="s">
+        <v>71</v>
+      </c>
+      <c r="R41" t="s">
+        <v>72</v>
+      </c>
+      <c r="S41" t="s">
+        <v>80</v>
+      </c>
+      <c r="T41" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="42" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B42" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="C42" t="s">
         <v>45</v>
       </c>
       <c r="D42" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="E42">
-        <v>2024</v>
+        <v>2013</v>
       </c>
       <c r="F42">
-        <v>0.10199999999999999</v>
+        <v>2.1999999999999999E-2</v>
       </c>
       <c r="G42">
         <v>1</v>
       </c>
       <c r="H42">
-        <v>2024</v>
-      </c>
-      <c r="I42">
-        <v>48.4</v>
+        <v>2376</v>
+      </c>
+      <c r="I42" s="3">
+        <v>57.2</v>
       </c>
       <c r="J42">
-        <v>2.3100000000000005</v>
+        <v>2.52</v>
       </c>
       <c r="K42">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="L42">
-        <v>0.40144059976798202</v>
+        <v>0.41047488326249421</v>
+      </c>
+      <c r="N42" t="s">
+        <v>69</v>
+      </c>
+      <c r="O42" t="s">
+        <v>146</v>
+      </c>
+      <c r="P42" t="s">
+        <v>147</v>
+      </c>
+      <c r="Q42" t="s">
+        <v>71</v>
+      </c>
+      <c r="R42" t="s">
+        <v>72</v>
+      </c>
+      <c r="S42" t="s">
+        <v>80</v>
+      </c>
+      <c r="T42" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="43" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B43" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="C43" t="s">
         <v>45</v>
@@ -4054,184 +4350,298 @@
         <v>58</v>
       </c>
       <c r="E43">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="F43">
-        <v>3.9E-2</v>
+        <v>0.255</v>
       </c>
       <c r="G43">
         <v>1</v>
       </c>
       <c r="H43">
-        <v>2376</v>
-      </c>
-      <c r="I43">
-        <v>57.2</v>
+        <v>2024</v>
+      </c>
+      <c r="I43" s="3">
+        <v>48.400000000000006</v>
       </c>
       <c r="J43">
-        <v>2.52</v>
+        <v>2.3100000000000005</v>
       </c>
       <c r="K43">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="L43">
         <v>0.365520596150406</v>
       </c>
+      <c r="N43" t="s">
+        <v>69</v>
+      </c>
+      <c r="O43" t="s">
+        <v>197</v>
+      </c>
+      <c r="P43" t="s">
+        <v>162</v>
+      </c>
+      <c r="Q43" t="s">
+        <v>71</v>
+      </c>
+      <c r="R43" t="s">
+        <v>72</v>
+      </c>
+      <c r="S43" t="s">
+        <v>80</v>
+      </c>
+      <c r="T43" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="44" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B44" t="s">
-        <v>59</v>
-      </c>
-      <c r="C44" t="s">
-        <v>45</v>
-      </c>
-      <c r="D44" t="s">
-        <v>60</v>
-      </c>
-      <c r="E44">
-        <v>2005</v>
-      </c>
-      <c r="F44">
-        <v>1.7999999999999999E-2</v>
-      </c>
-      <c r="G44">
-        <v>1</v>
-      </c>
-      <c r="H44">
-        <v>2376</v>
-      </c>
-      <c r="I44">
-        <v>57.20000000000001</v>
-      </c>
-      <c r="J44">
-        <v>2.52</v>
-      </c>
-      <c r="K44">
-        <v>50</v>
-      </c>
-      <c r="L44">
-        <v>0.41047488326249421</v>
+        <v>140</v>
+      </c>
+      <c r="C44" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="N44" t="s">
+        <v>69</v>
+      </c>
+      <c r="O44" t="s">
+        <v>154</v>
+      </c>
+      <c r="P44" t="s">
+        <v>155</v>
+      </c>
+      <c r="Q44" t="s">
+        <v>71</v>
+      </c>
+      <c r="R44" t="s">
+        <v>72</v>
+      </c>
+      <c r="S44" t="s">
+        <v>80</v>
+      </c>
+      <c r="T44" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="45" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B45" t="s">
-        <v>59</v>
+        <v>196</v>
       </c>
       <c r="C45" t="s">
-        <v>45</v>
+        <v>192</v>
       </c>
       <c r="D45" t="s">
-        <v>60</v>
+        <v>14</v>
       </c>
       <c r="E45">
-        <v>2012</v>
+        <v>2022</v>
       </c>
       <c r="F45">
-        <v>2.1999999999999999E-2</v>
+        <v>0.77</v>
       </c>
       <c r="G45">
-        <v>1</v>
+        <v>0.49</v>
       </c>
       <c r="H45">
-        <v>2376</v>
-      </c>
-      <c r="I45">
-        <v>57.2</v>
+        <v>2150</v>
+      </c>
+      <c r="I45" s="3">
+        <v>35.053609999999999</v>
       </c>
       <c r="J45">
-        <v>2.52</v>
+        <v>3.28</v>
       </c>
       <c r="K45">
-        <v>43</v>
-      </c>
-      <c r="L45">
-        <v>0.41047488326249421</v>
+        <v>40</v>
+      </c>
+      <c r="N45" t="s">
+        <v>69</v>
+      </c>
+      <c r="O45" t="s">
+        <v>156</v>
+      </c>
+      <c r="P45" t="s">
+        <v>157</v>
+      </c>
+      <c r="Q45" t="s">
+        <v>71</v>
+      </c>
+      <c r="R45" t="s">
+        <v>72</v>
+      </c>
+      <c r="S45" t="s">
+        <v>80</v>
+      </c>
+      <c r="T45" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="46" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B46" t="s">
-        <v>59</v>
+        <v>194</v>
       </c>
       <c r="C46" t="s">
-        <v>45</v>
+        <v>192</v>
       </c>
       <c r="D46" t="s">
-        <v>60</v>
+        <v>14</v>
       </c>
       <c r="E46">
-        <v>2013</v>
+        <v>2022</v>
       </c>
       <c r="F46">
-        <v>2.1999999999999999E-2</v>
+        <v>0.26</v>
       </c>
       <c r="G46">
-        <v>1</v>
+        <v>0.49</v>
       </c>
       <c r="H46">
-        <v>2376</v>
-      </c>
-      <c r="I46">
-        <v>57.2</v>
+        <v>2150</v>
+      </c>
+      <c r="I46" s="3">
+        <v>35.053609999999999</v>
       </c>
       <c r="J46">
-        <v>2.52</v>
+        <v>3.28</v>
       </c>
       <c r="K46">
-        <v>42</v>
-      </c>
-      <c r="L46">
-        <v>0.41047488326249421</v>
+        <v>40</v>
+      </c>
+      <c r="N46" t="s">
+        <v>69</v>
+      </c>
+      <c r="O46" t="s">
+        <v>170</v>
+      </c>
+      <c r="P46" t="s">
+        <v>171</v>
+      </c>
+      <c r="Q46" t="s">
+        <v>71</v>
+      </c>
+      <c r="R46" t="s">
+        <v>72</v>
+      </c>
+      <c r="S46" t="s">
+        <v>80</v>
+      </c>
+      <c r="T46" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="47" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B47" t="s">
-        <v>61</v>
+        <v>193</v>
       </c>
       <c r="C47" t="s">
-        <v>45</v>
+        <v>192</v>
       </c>
       <c r="D47" t="s">
-        <v>58</v>
+        <v>14</v>
       </c>
       <c r="E47">
-        <v>2024</v>
+        <v>2022</v>
       </c>
       <c r="F47">
-        <v>0.255</v>
+        <v>0.185</v>
       </c>
       <c r="G47">
-        <v>1</v>
+        <v>0.49</v>
       </c>
       <c r="H47">
-        <v>2024</v>
-      </c>
-      <c r="I47">
-        <v>48.400000000000006</v>
+        <v>2150</v>
+      </c>
+      <c r="I47" s="3">
+        <v>35.053609999999999</v>
       </c>
       <c r="J47">
-        <v>2.3100000000000005</v>
+        <v>3.28</v>
       </c>
       <c r="K47">
-        <v>31</v>
-      </c>
-      <c r="L47">
-        <v>0.365520596150406</v>
+        <v>37</v>
+      </c>
+      <c r="N47" t="s">
+        <v>69</v>
+      </c>
+      <c r="O47" t="s">
+        <v>158</v>
+      </c>
+      <c r="P47" t="s">
+        <v>159</v>
+      </c>
+      <c r="Q47" t="s">
+        <v>71</v>
+      </c>
+      <c r="R47" t="s">
+        <v>72</v>
+      </c>
+      <c r="S47" t="s">
+        <v>80</v>
+      </c>
+      <c r="T47" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="48" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B48" t="s">
-        <v>140</v>
-      </c>
-      <c r="C48" s="1" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="49" spans="2:11" x14ac:dyDescent="0.25">
+        <v>195</v>
+      </c>
+      <c r="C48" t="s">
+        <v>192</v>
+      </c>
+      <c r="D48" t="s">
+        <v>14</v>
+      </c>
+      <c r="E48">
+        <v>2022</v>
+      </c>
+      <c r="F48">
+        <v>0.01</v>
+      </c>
+      <c r="G48">
+        <v>0.49</v>
+      </c>
+      <c r="H48">
+        <v>2150</v>
+      </c>
+      <c r="I48" s="3">
+        <v>35.053609999999999</v>
+      </c>
+      <c r="J48">
+        <v>3.28</v>
+      </c>
+      <c r="K48">
+        <v>40</v>
+      </c>
+      <c r="N48" t="s">
+        <v>69</v>
+      </c>
+      <c r="O48" t="s">
+        <v>169</v>
+      </c>
+      <c r="P48" t="s">
+        <v>160</v>
+      </c>
+      <c r="Q48" t="s">
+        <v>71</v>
+      </c>
+      <c r="R48" t="s">
+        <v>72</v>
+      </c>
+      <c r="S48" t="s">
+        <v>80</v>
+      </c>
+      <c r="T48" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="49" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B49" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="C49" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="D49" t="s">
         <v>14</v>
@@ -4240,30 +4650,51 @@
         <v>2022</v>
       </c>
       <c r="F49">
-        <v>0.26</v>
+        <v>7.6999999999999999E-2</v>
       </c>
       <c r="G49">
-        <v>1</v>
+        <v>0.41</v>
       </c>
       <c r="H49">
-        <v>1265</v>
-      </c>
-      <c r="I49">
-        <v>48.4</v>
+        <v>360</v>
+      </c>
+      <c r="I49" s="3">
+        <v>9.3576800000000002</v>
       </c>
       <c r="J49">
-        <v>7.5075000000000003</v>
+        <v>6.38</v>
       </c>
       <c r="K49">
         <v>40</v>
       </c>
-    </row>
-    <row r="50" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="N49" t="s">
+        <v>69</v>
+      </c>
+      <c r="O49" t="s">
+        <v>164</v>
+      </c>
+      <c r="P49" t="s">
+        <v>165</v>
+      </c>
+      <c r="Q49" t="s">
+        <v>71</v>
+      </c>
+      <c r="R49" t="s">
+        <v>72</v>
+      </c>
+      <c r="S49" t="s">
+        <v>80</v>
+      </c>
+      <c r="T49" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="50" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B50" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="C50" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="D50" t="s">
         <v>14</v>
@@ -4272,30 +4703,51 @@
         <v>2022</v>
       </c>
       <c r="F50">
-        <v>0.185</v>
+        <v>3.9E-2</v>
       </c>
       <c r="G50">
-        <v>1</v>
-      </c>
-      <c r="H50">
-        <v>1265</v>
-      </c>
-      <c r="I50">
-        <v>48.4</v>
-      </c>
-      <c r="J50">
-        <v>7.5075000000000003</v>
+        <v>0.28999999999999998</v>
+      </c>
+      <c r="H50" s="2">
+        <v>3200.7518811800001</v>
+      </c>
+      <c r="I50" s="3">
+        <v>131.85821703200003</v>
+      </c>
+      <c r="J50" s="4">
+        <v>1.9778732554800003</v>
       </c>
       <c r="K50">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="51" spans="2:11" x14ac:dyDescent="0.25">
+        <v>40</v>
+      </c>
+      <c r="N50" t="s">
+        <v>69</v>
+      </c>
+      <c r="O50" t="s">
+        <v>168</v>
+      </c>
+      <c r="P50" t="s">
+        <v>166</v>
+      </c>
+      <c r="Q50" t="s">
+        <v>71</v>
+      </c>
+      <c r="R50" t="s">
+        <v>72</v>
+      </c>
+      <c r="S50" t="s">
+        <v>80</v>
+      </c>
+      <c r="T50" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="51" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B51" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="C51" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="D51" t="s">
         <v>14</v>
@@ -4304,22 +4756,1113 @@
         <v>2022</v>
       </c>
       <c r="F51">
-        <v>0.01</v>
+        <v>2.2100000000000002E-2</v>
       </c>
       <c r="G51">
-        <v>1</v>
-      </c>
-      <c r="H51">
-        <v>1265</v>
-      </c>
-      <c r="I51">
-        <v>48.4</v>
-      </c>
-      <c r="J51">
-        <v>7.5075000000000003</v>
+        <v>0.28999999999999998</v>
+      </c>
+      <c r="H51" s="2">
+        <v>3200.7518811800001</v>
+      </c>
+      <c r="I51" s="3">
+        <v>131.85821703200003</v>
+      </c>
+      <c r="J51" s="4">
+        <v>1.9778732554800003</v>
       </c>
       <c r="K51">
         <v>40</v>
+      </c>
+      <c r="N51" t="s">
+        <v>69</v>
+      </c>
+      <c r="O51" t="s">
+        <v>198</v>
+      </c>
+      <c r="P51" t="s">
+        <v>167</v>
+      </c>
+      <c r="Q51" t="s">
+        <v>71</v>
+      </c>
+      <c r="R51" t="s">
+        <v>72</v>
+      </c>
+      <c r="S51" t="s">
+        <v>80</v>
+      </c>
+      <c r="T51" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="52" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B52" t="s">
+        <v>145</v>
+      </c>
+      <c r="C52" t="s">
+        <v>13</v>
+      </c>
+      <c r="D52" t="s">
+        <v>14</v>
+      </c>
+      <c r="E52">
+        <v>2022</v>
+      </c>
+      <c r="F52">
+        <v>2.0500000000000001E-2</v>
+      </c>
+      <c r="G52">
+        <v>0.28999999999999998</v>
+      </c>
+      <c r="H52" s="2">
+        <v>3200.7518811800001</v>
+      </c>
+      <c r="I52" s="3">
+        <v>131.85821703200003</v>
+      </c>
+      <c r="J52" s="4">
+        <v>1.9778732554800003</v>
+      </c>
+      <c r="K52">
+        <v>40</v>
+      </c>
+      <c r="N52" t="s">
+        <v>69</v>
+      </c>
+      <c r="O52" t="s">
+        <v>172</v>
+      </c>
+      <c r="P52" t="s">
+        <v>173</v>
+      </c>
+      <c r="Q52" t="s">
+        <v>71</v>
+      </c>
+      <c r="R52" t="s">
+        <v>72</v>
+      </c>
+      <c r="S52" t="s">
+        <v>80</v>
+      </c>
+      <c r="T52" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="53" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B53" t="s">
+        <v>146</v>
+      </c>
+      <c r="C53" t="s">
+        <v>13</v>
+      </c>
+      <c r="D53" t="s">
+        <v>14</v>
+      </c>
+      <c r="E53">
+        <v>2022</v>
+      </c>
+      <c r="F53">
+        <v>1.3900000000000001E-2</v>
+      </c>
+      <c r="G53">
+        <v>0.28999999999999998</v>
+      </c>
+      <c r="H53" s="2">
+        <v>3200.7518811800001</v>
+      </c>
+      <c r="I53" s="3">
+        <v>131.85821703200003</v>
+      </c>
+      <c r="J53" s="4">
+        <v>1.9778732554800003</v>
+      </c>
+      <c r="K53">
+        <v>40</v>
+      </c>
+      <c r="N53" t="s">
+        <v>69</v>
+      </c>
+      <c r="O53" t="s">
+        <v>174</v>
+      </c>
+      <c r="P53" t="s">
+        <v>175</v>
+      </c>
+      <c r="Q53" t="s">
+        <v>71</v>
+      </c>
+      <c r="R53" t="s">
+        <v>72</v>
+      </c>
+      <c r="S53" t="s">
+        <v>80</v>
+      </c>
+      <c r="T53" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="54" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B54" t="s">
+        <v>197</v>
+      </c>
+      <c r="C54" t="s">
+        <v>192</v>
+      </c>
+      <c r="D54" t="s">
+        <v>14</v>
+      </c>
+      <c r="E54">
+        <v>2022</v>
+      </c>
+      <c r="F54">
+        <v>0.01</v>
+      </c>
+      <c r="G54">
+        <v>0.49</v>
+      </c>
+      <c r="H54" s="2">
+        <v>2150</v>
+      </c>
+      <c r="I54" s="3">
+        <v>35.053609999999999</v>
+      </c>
+      <c r="J54" s="4">
+        <v>3.28</v>
+      </c>
+      <c r="K54">
+        <v>40</v>
+      </c>
+      <c r="N54" t="s">
+        <v>69</v>
+      </c>
+      <c r="O54" t="s">
+        <v>176</v>
+      </c>
+      <c r="P54" t="s">
+        <v>177</v>
+      </c>
+      <c r="Q54" t="s">
+        <v>71</v>
+      </c>
+      <c r="R54" t="s">
+        <v>72</v>
+      </c>
+      <c r="S54" t="s">
+        <v>80</v>
+      </c>
+      <c r="T54" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="55" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B55" t="s">
+        <v>154</v>
+      </c>
+      <c r="C55" t="s">
+        <v>13</v>
+      </c>
+      <c r="D55" t="s">
+        <v>14</v>
+      </c>
+      <c r="E55">
+        <v>2022</v>
+      </c>
+      <c r="F55">
+        <v>0.01</v>
+      </c>
+      <c r="G55">
+        <v>0.28999999999999998</v>
+      </c>
+      <c r="H55" s="2">
+        <v>3200.7518811800001</v>
+      </c>
+      <c r="I55" s="3">
+        <v>131.85821703200003</v>
+      </c>
+      <c r="J55" s="4">
+        <v>1.9778732554800003</v>
+      </c>
+      <c r="K55">
+        <v>40</v>
+      </c>
+      <c r="N55" t="s">
+        <v>69</v>
+      </c>
+      <c r="O55" t="s">
+        <v>178</v>
+      </c>
+      <c r="P55" t="s">
+        <v>179</v>
+      </c>
+      <c r="Q55" t="s">
+        <v>71</v>
+      </c>
+      <c r="R55" t="s">
+        <v>72</v>
+      </c>
+      <c r="S55" t="s">
+        <v>80</v>
+      </c>
+      <c r="T55" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="56" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B56" t="s">
+        <v>156</v>
+      </c>
+      <c r="C56" t="s">
+        <v>13</v>
+      </c>
+      <c r="D56" t="s">
+        <v>14</v>
+      </c>
+      <c r="E56">
+        <v>2022</v>
+      </c>
+      <c r="F56">
+        <v>0.01</v>
+      </c>
+      <c r="G56">
+        <v>0.28999999999999998</v>
+      </c>
+      <c r="H56" s="2">
+        <v>3200.7518811800001</v>
+      </c>
+      <c r="I56" s="3">
+        <v>131.85821703200003</v>
+      </c>
+      <c r="J56" s="4">
+        <v>1.9778732554800003</v>
+      </c>
+      <c r="K56">
+        <v>40</v>
+      </c>
+      <c r="N56" t="s">
+        <v>69</v>
+      </c>
+      <c r="O56" t="s">
+        <v>180</v>
+      </c>
+      <c r="P56" t="s">
+        <v>181</v>
+      </c>
+      <c r="Q56" t="s">
+        <v>71</v>
+      </c>
+      <c r="R56" t="s">
+        <v>72</v>
+      </c>
+      <c r="S56" t="s">
+        <v>80</v>
+      </c>
+      <c r="T56" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="57" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B57" t="s">
+        <v>170</v>
+      </c>
+      <c r="C57" t="s">
+        <v>13</v>
+      </c>
+      <c r="D57" t="s">
+        <v>14</v>
+      </c>
+      <c r="E57">
+        <v>2022</v>
+      </c>
+      <c r="F57">
+        <v>9.300000000000001E-3</v>
+      </c>
+      <c r="G57">
+        <v>0.28999999999999998</v>
+      </c>
+      <c r="H57" s="2">
+        <v>3200.7518811800001</v>
+      </c>
+      <c r="I57" s="3">
+        <v>131.85821703200003</v>
+      </c>
+      <c r="J57" s="4">
+        <v>1.9778732554800003</v>
+      </c>
+      <c r="K57">
+        <v>40</v>
+      </c>
+      <c r="N57" t="s">
+        <v>69</v>
+      </c>
+      <c r="O57" t="s">
+        <v>182</v>
+      </c>
+      <c r="P57" t="s">
+        <v>183</v>
+      </c>
+      <c r="Q57" t="s">
+        <v>71</v>
+      </c>
+      <c r="R57" t="s">
+        <v>72</v>
+      </c>
+      <c r="S57" t="s">
+        <v>80</v>
+      </c>
+      <c r="T57" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="58" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B58" t="s">
+        <v>158</v>
+      </c>
+      <c r="C58" t="s">
+        <v>13</v>
+      </c>
+      <c r="D58" t="s">
+        <v>14</v>
+      </c>
+      <c r="E58">
+        <v>2022</v>
+      </c>
+      <c r="F58">
+        <v>7.0999999999999995E-3</v>
+      </c>
+      <c r="G58">
+        <v>0.28999999999999998</v>
+      </c>
+      <c r="H58" s="2">
+        <v>3200.7518811800001</v>
+      </c>
+      <c r="I58" s="3">
+        <v>131.85821703200003</v>
+      </c>
+      <c r="J58" s="4">
+        <v>1.9778732554800003</v>
+      </c>
+      <c r="K58">
+        <v>40</v>
+      </c>
+      <c r="N58" t="s">
+        <v>69</v>
+      </c>
+      <c r="O58" t="s">
+        <v>184</v>
+      </c>
+      <c r="P58" t="s">
+        <v>185</v>
+      </c>
+      <c r="Q58" t="s">
+        <v>71</v>
+      </c>
+      <c r="R58" t="s">
+        <v>72</v>
+      </c>
+      <c r="S58" t="s">
+        <v>80</v>
+      </c>
+      <c r="T58" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="59" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B59" t="s">
+        <v>169</v>
+      </c>
+      <c r="C59" t="s">
+        <v>16</v>
+      </c>
+      <c r="D59" t="s">
+        <v>14</v>
+      </c>
+      <c r="E59">
+        <v>2022</v>
+      </c>
+      <c r="F59">
+        <v>5.7999999999999996E-3</v>
+      </c>
+      <c r="G59">
+        <v>0.41</v>
+      </c>
+      <c r="H59" s="2">
+        <v>521.0526318200001</v>
+      </c>
+      <c r="I59" s="3">
+        <v>6.9119226670000007</v>
+      </c>
+      <c r="J59" s="4">
+        <v>6.38</v>
+      </c>
+      <c r="K59">
+        <v>40</v>
+      </c>
+      <c r="N59" t="s">
+        <v>69</v>
+      </c>
+      <c r="O59" t="s">
+        <v>186</v>
+      </c>
+      <c r="P59" t="s">
+        <v>188</v>
+      </c>
+      <c r="Q59" t="s">
+        <v>71</v>
+      </c>
+      <c r="R59" t="s">
+        <v>72</v>
+      </c>
+      <c r="S59" t="s">
+        <v>80</v>
+      </c>
+      <c r="T59" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="60" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B60" t="s">
+        <v>164</v>
+      </c>
+      <c r="C60" t="s">
+        <v>13</v>
+      </c>
+      <c r="D60" t="s">
+        <v>14</v>
+      </c>
+      <c r="E60">
+        <v>2022</v>
+      </c>
+      <c r="F60">
+        <v>6.4999999999999997E-3</v>
+      </c>
+      <c r="G60">
+        <v>0.28999999999999998</v>
+      </c>
+      <c r="H60" s="2">
+        <v>3200.7518811800001</v>
+      </c>
+      <c r="I60" s="3">
+        <v>131.85821703200003</v>
+      </c>
+      <c r="J60" s="4">
+        <v>1.9778732554800003</v>
+      </c>
+      <c r="K60">
+        <v>40</v>
+      </c>
+      <c r="N60" t="s">
+        <v>69</v>
+      </c>
+      <c r="O60" t="s">
+        <v>187</v>
+      </c>
+      <c r="P60" t="s">
+        <v>189</v>
+      </c>
+      <c r="Q60" t="s">
+        <v>71</v>
+      </c>
+      <c r="R60" t="s">
+        <v>72</v>
+      </c>
+      <c r="S60" t="s">
+        <v>80</v>
+      </c>
+      <c r="T60" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="61" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B61" t="s">
+        <v>168</v>
+      </c>
+      <c r="C61" t="s">
+        <v>16</v>
+      </c>
+      <c r="D61" t="s">
+        <v>14</v>
+      </c>
+      <c r="E61">
+        <v>2022</v>
+      </c>
+      <c r="F61">
+        <v>4.0999999999999995E-3</v>
+      </c>
+      <c r="G61">
+        <v>0.41</v>
+      </c>
+      <c r="H61" s="2">
+        <v>521.0526318200001</v>
+      </c>
+      <c r="I61" s="3">
+        <v>6.9119226670000007</v>
+      </c>
+      <c r="J61" s="4">
+        <v>6.38</v>
+      </c>
+      <c r="K61">
+        <v>40</v>
+      </c>
+      <c r="N61" t="s">
+        <v>69</v>
+      </c>
+      <c r="O61" t="s">
+        <v>190</v>
+      </c>
+      <c r="P61" t="s">
+        <v>191</v>
+      </c>
+      <c r="Q61" t="s">
+        <v>71</v>
+      </c>
+      <c r="R61" t="s">
+        <v>72</v>
+      </c>
+      <c r="S61" t="s">
+        <v>80</v>
+      </c>
+      <c r="T61" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="62" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B62" t="s">
+        <v>198</v>
+      </c>
+      <c r="C62" t="s">
+        <v>192</v>
+      </c>
+      <c r="D62" t="s">
+        <v>14</v>
+      </c>
+      <c r="E62">
+        <v>2022</v>
+      </c>
+      <c r="F62">
+        <v>1.4E-3</v>
+      </c>
+      <c r="G62">
+        <v>0.49</v>
+      </c>
+      <c r="H62" s="2">
+        <v>2150</v>
+      </c>
+      <c r="I62" s="3">
+        <v>35.053609999999999</v>
+      </c>
+      <c r="J62" s="4">
+        <v>3.28</v>
+      </c>
+      <c r="K62">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="63" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B63" t="s">
+        <v>172</v>
+      </c>
+      <c r="C63" t="s">
+        <v>13</v>
+      </c>
+      <c r="D63" t="s">
+        <v>14</v>
+      </c>
+      <c r="E63">
+        <v>2022</v>
+      </c>
+      <c r="F63">
+        <v>1.8E-3</v>
+      </c>
+      <c r="G63">
+        <v>0.28999999999999998</v>
+      </c>
+      <c r="H63" s="2">
+        <v>6444.0386710800003</v>
+      </c>
+      <c r="I63" s="3">
+        <v>288.17400657800005</v>
+      </c>
+      <c r="J63" s="4">
+        <v>4.1365198730200001</v>
+      </c>
+      <c r="K63">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="64" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B64" t="s">
+        <v>174</v>
+      </c>
+      <c r="C64" t="s">
+        <v>13</v>
+      </c>
+      <c r="D64" t="s">
+        <v>14</v>
+      </c>
+      <c r="E64">
+        <v>2022</v>
+      </c>
+      <c r="F64">
+        <v>1.6999999999999999E-3</v>
+      </c>
+      <c r="G64">
+        <v>0.28999999999999998</v>
+      </c>
+      <c r="H64" s="2">
+        <v>6444.0386710800003</v>
+      </c>
+      <c r="I64" s="3">
+        <v>288.17400657800005</v>
+      </c>
+      <c r="J64" s="4">
+        <v>4.1365198730200001</v>
+      </c>
+      <c r="K64">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="65" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B65" t="s">
+        <v>176</v>
+      </c>
+      <c r="C65" t="s">
+        <v>16</v>
+      </c>
+      <c r="D65" t="s">
+        <v>14</v>
+      </c>
+      <c r="E65">
+        <v>2022</v>
+      </c>
+      <c r="F65">
+        <v>1.8E-3</v>
+      </c>
+      <c r="G65">
+        <v>0.41</v>
+      </c>
+      <c r="H65" s="2">
+        <v>521.0526318200001</v>
+      </c>
+      <c r="I65" s="3">
+        <v>6.9119226670000007</v>
+      </c>
+      <c r="J65" s="4">
+        <v>6.38</v>
+      </c>
+      <c r="K65">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="66" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B66" t="s">
+        <v>178</v>
+      </c>
+      <c r="C66" t="s">
+        <v>16</v>
+      </c>
+      <c r="D66" t="s">
+        <v>14</v>
+      </c>
+      <c r="E66">
+        <v>2022</v>
+      </c>
+      <c r="F66">
+        <v>1.8E-3</v>
+      </c>
+      <c r="G66">
+        <v>0.41</v>
+      </c>
+      <c r="H66" s="2">
+        <v>521.0526318200001</v>
+      </c>
+      <c r="I66" s="3">
+        <v>6.9119226670000007</v>
+      </c>
+      <c r="J66" s="4">
+        <v>6.38</v>
+      </c>
+      <c r="K66">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="67" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B67" t="s">
+        <v>180</v>
+      </c>
+      <c r="C67" t="s">
+        <v>13</v>
+      </c>
+      <c r="D67" t="s">
+        <v>14</v>
+      </c>
+      <c r="E67">
+        <v>2022</v>
+      </c>
+      <c r="F67">
+        <v>1.5E-3</v>
+      </c>
+      <c r="G67">
+        <v>0.28999999999999998</v>
+      </c>
+      <c r="H67" s="2">
+        <v>1010.2040821000001</v>
+      </c>
+      <c r="I67" s="3">
+        <v>10.3678840005</v>
+      </c>
+      <c r="J67" s="4">
+        <v>7.9752953850000008</v>
+      </c>
+      <c r="K67">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="68" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B68" t="s">
+        <v>182</v>
+      </c>
+      <c r="C68" t="s">
+        <v>13</v>
+      </c>
+      <c r="D68" t="s">
+        <v>14</v>
+      </c>
+      <c r="E68">
+        <v>2022</v>
+      </c>
+      <c r="F68">
+        <v>1.4E-3</v>
+      </c>
+      <c r="G68">
+        <v>0.28999999999999998</v>
+      </c>
+      <c r="H68" s="2">
+        <v>1010.2040821000001</v>
+      </c>
+      <c r="I68" s="3">
+        <v>10.3678840005</v>
+      </c>
+      <c r="J68" s="4">
+        <v>7.9752953850000008</v>
+      </c>
+      <c r="K68">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="69" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B69" t="s">
+        <v>184</v>
+      </c>
+      <c r="C69" t="s">
+        <v>13</v>
+      </c>
+      <c r="D69" t="s">
+        <v>14</v>
+      </c>
+      <c r="E69">
+        <v>2022</v>
+      </c>
+      <c r="F69">
+        <v>1.1999999999999999E-3</v>
+      </c>
+      <c r="G69">
+        <v>0.28999999999999998</v>
+      </c>
+      <c r="H69" s="2">
+        <v>1010.2040821000001</v>
+      </c>
+      <c r="I69" s="3">
+        <v>10.3678840005</v>
+      </c>
+      <c r="J69" s="4">
+        <v>7.9752953850000008</v>
+      </c>
+      <c r="K69">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="70" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B70" t="s">
+        <v>186</v>
+      </c>
+      <c r="C70" t="s">
+        <v>13</v>
+      </c>
+      <c r="D70" t="s">
+        <v>14</v>
+      </c>
+      <c r="E70">
+        <v>2022</v>
+      </c>
+      <c r="F70">
+        <v>1.9E-3</v>
+      </c>
+      <c r="G70">
+        <v>0.28999999999999998</v>
+      </c>
+      <c r="H70" s="2">
+        <v>11048.442540020002</v>
+      </c>
+      <c r="I70" s="3">
+        <v>437.04618709800002</v>
+      </c>
+      <c r="J70" s="4">
+        <v>27.520085941840001</v>
+      </c>
+      <c r="K70">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="71" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B71" t="s">
+        <v>187</v>
+      </c>
+      <c r="C71" t="s">
+        <v>13</v>
+      </c>
+      <c r="D71" t="s">
+        <v>14</v>
+      </c>
+      <c r="E71">
+        <v>2022</v>
+      </c>
+      <c r="F71">
+        <v>8.9999999999999998E-4</v>
+      </c>
+      <c r="G71">
+        <v>0.28999999999999998</v>
+      </c>
+      <c r="H71" s="2">
+        <v>6444.0386710800003</v>
+      </c>
+      <c r="I71" s="3">
+        <v>288.17400657800005</v>
+      </c>
+      <c r="J71" s="4">
+        <v>4.1365198730200001</v>
+      </c>
+      <c r="K71">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="72" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B72" t="s">
+        <v>190</v>
+      </c>
+      <c r="C72" t="s">
+        <v>13</v>
+      </c>
+      <c r="D72" t="s">
+        <v>14</v>
+      </c>
+      <c r="E72">
+        <v>2022</v>
+      </c>
+      <c r="F72">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="G72">
+        <v>0.28999999999999998</v>
+      </c>
+      <c r="H72" s="2">
+        <v>11048.442540020002</v>
+      </c>
+      <c r="I72" s="3">
+        <v>437.04618709800002</v>
+      </c>
+      <c r="J72" s="4">
+        <v>27.520085941840001</v>
+      </c>
+      <c r="K72">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="77" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B77" t="s">
+        <v>20</v>
+      </c>
+      <c r="C77" t="s">
+        <v>21</v>
+      </c>
+      <c r="D77" t="s">
+        <v>14</v>
+      </c>
+      <c r="E77">
+        <v>2013</v>
+      </c>
+      <c r="F77">
+        <v>0.25109999999999999</v>
+      </c>
+      <c r="G77">
+        <v>0.36049999999999999</v>
+      </c>
+      <c r="H77">
+        <v>1265</v>
+      </c>
+      <c r="I77" s="3">
+        <v>48.400000000000006</v>
+      </c>
+      <c r="J77">
+        <v>7.5075000000000003</v>
+      </c>
+      <c r="K77">
+        <v>42</v>
+      </c>
+      <c r="N77" t="s">
+        <v>69</v>
+      </c>
+      <c r="O77" t="s">
+        <v>20</v>
+      </c>
+      <c r="P77" t="s">
+        <v>79</v>
+      </c>
+      <c r="Q77" t="s">
+        <v>71</v>
+      </c>
+      <c r="R77" t="s">
+        <v>72</v>
+      </c>
+      <c r="S77" t="s">
+        <v>73</v>
+      </c>
+      <c r="T77" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="78" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B78" t="s">
+        <v>15</v>
+      </c>
+      <c r="C78" t="s">
+        <v>16</v>
+      </c>
+      <c r="D78" t="s">
+        <v>14</v>
+      </c>
+      <c r="E78">
+        <v>2022</v>
+      </c>
+      <c r="F78">
+        <v>0.21299999999999999</v>
+      </c>
+      <c r="G78">
+        <v>0.33123000000000002</v>
+      </c>
+      <c r="N78" t="s">
+        <v>69</v>
+      </c>
+      <c r="O78" t="s">
+        <v>15</v>
+      </c>
+      <c r="P78" t="s">
+        <v>75</v>
+      </c>
+      <c r="Q78" t="s">
+        <v>71</v>
+      </c>
+      <c r="R78" t="s">
+        <v>72</v>
+      </c>
+      <c r="S78" t="s">
+        <v>73</v>
+      </c>
+      <c r="T78" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="79" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B79" t="s">
+        <v>18</v>
+      </c>
+      <c r="C79" t="s">
+        <v>19</v>
+      </c>
+      <c r="D79" t="s">
+        <v>14</v>
+      </c>
+      <c r="E79">
+        <v>2022</v>
+      </c>
+      <c r="F79">
+        <v>8.0000000000000002E-3</v>
+      </c>
+      <c r="G79">
+        <v>0.33123000000000002</v>
+      </c>
+      <c r="N79" t="s">
+        <v>69</v>
+      </c>
+      <c r="O79" t="s">
+        <v>18</v>
+      </c>
+      <c r="P79" t="s">
+        <v>78</v>
+      </c>
+      <c r="Q79" t="s">
+        <v>71</v>
+      </c>
+      <c r="R79" t="s">
+        <v>72</v>
+      </c>
+      <c r="S79" t="s">
+        <v>73</v>
+      </c>
+      <c r="T79" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="80" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B80" t="s">
+        <v>12</v>
+      </c>
+      <c r="C80" t="s">
+        <v>13</v>
+      </c>
+      <c r="D80" t="s">
+        <v>14</v>
+      </c>
+      <c r="E80">
+        <v>2022</v>
+      </c>
+      <c r="F80">
+        <v>0.3</v>
+      </c>
+      <c r="G80">
+        <v>0.33990000000000004</v>
+      </c>
+      <c r="H80">
+        <v>4427.5</v>
+      </c>
+      <c r="I80" s="3">
+        <v>157.30000000000001</v>
+      </c>
+      <c r="J80">
+        <v>9.24</v>
+      </c>
+      <c r="K80">
+        <v>50</v>
+      </c>
+      <c r="N80" t="s">
+        <v>69</v>
+      </c>
+      <c r="O80" t="s">
+        <v>12</v>
+      </c>
+      <c r="P80" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q80" t="s">
+        <v>71</v>
+      </c>
+      <c r="R80" t="s">
+        <v>72</v>
+      </c>
+      <c r="S80" t="s">
+        <v>73</v>
+      </c>
+      <c r="T80" t="s">
+        <v>74</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Adding investments to past
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/vt_EST_ELC_v1.xlsx
+++ b/VerveStacks_EST/vt_EST_ELC_v1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBF99D7B-4C1B-4CC1-9323-B322FFD6BBC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FC64D7C-6183-4BE9-8A7A-7FE1B408D8FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-10470" yWindow="10890" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{21C51102-B905-44E2-89DF-C1A7E31F8D9F}"/>
+    <workbookView xWindow="-10470" yWindow="10890" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{21C51102-B905-44E2-89DF-C1A7E31F8D9F}"/>
   </bookViews>
   <sheets>
     <sheet name="ccs_retrofits" sheetId="4" r:id="rId1"/>
@@ -69,6 +69,7 @@
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>tc={E45DD652-654C-4828-8A13-679EDDC53E65}</author>
+    <author>tc={5D0B02A9-24B3-4F36-8683-2AD26D1E0821}</author>
     <author>tc={06D70610-96F7-4BDA-B071-69925D70228B}</author>
     <author>tc={A1B9CC12-DC46-488C-9BF3-3F8DFC23199D}</author>
     <author>tc={4E0E017D-BAC7-4AA8-B401-A7330F2C0996}</author>
@@ -84,7 +85,15 @@
     Iru produces only 17 MW in 2025 not 0.207 GW</t>
       </text>
     </comment>
-    <comment ref="G46" authorId="1" shapeId="0" xr:uid="{06D70610-96F7-4BDA-B071-69925D70228B}">
+    <comment ref="B45" authorId="1" shapeId="0" xr:uid="{5D0B02A9-24B3-4F36-8683-2AD26D1E0821}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    TODO: set their actual start date and then add how much they produce in 2025</t>
+      </text>
+    </comment>
+    <comment ref="G46" authorId="2" shapeId="0" xr:uid="{06D70610-96F7-4BDA-B071-69925D70228B}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -92,7 +101,7 @@
     Danish Energy agency - coal CHP 2020</t>
       </text>
     </comment>
-    <comment ref="G49" authorId="2" shapeId="0" xr:uid="{A1B9CC12-DC46-488C-9BF3-3F8DFC23199D}">
+    <comment ref="G49" authorId="3" shapeId="0" xr:uid="{A1B9CC12-DC46-488C-9BF3-3F8DFC23199D}">
       <text>
         <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -101,7 +110,7 @@
 </t>
       </text>
     </comment>
-    <comment ref="G50" authorId="3" shapeId="0" xr:uid="{4E0E017D-BAC7-4AA8-B401-A7330F2C0996}">
+    <comment ref="G50" authorId="4" shapeId="0" xr:uid="{4E0E017D-BAC7-4AA8-B401-A7330F2C0996}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -109,7 +118,7 @@
     DAE - Wood pellets, Medium 2020</t>
       </text>
     </comment>
-    <comment ref="N77" authorId="4" shapeId="0" xr:uid="{1905391B-2A5F-4643-B2AC-720AD8410CDA}">
+    <comment ref="N77" authorId="5" shapeId="0" xr:uid="{1905391B-2A5F-4643-B2AC-720AD8410CDA}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -117,7 +126,7 @@
     Frequency reserve</t>
       </text>
     </comment>
-    <comment ref="J80" authorId="5" shapeId="0" xr:uid="{3057E3B1-7BF3-4718-B31B-0585028D4313}">
+    <comment ref="J80" authorId="6" shapeId="0" xr:uid="{3057E3B1-7BF3-4718-B31B-0585028D4313}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -1154,6 +1163,9 @@
   <threadedComment ref="F11" dT="2026-01-22T14:00:05.64" personId="{9CD26280-DD25-46DF-A708-6877D8A68AD8}" id="{E45DD652-654C-4828-8A13-679EDDC53E65}">
     <text>Iru produces only 17 MW in 2025 not 0.207 GW</text>
   </threadedComment>
+  <threadedComment ref="B45" dT="2026-02-02T06:49:06.81" personId="{9CD26280-DD25-46DF-A708-6877D8A68AD8}" id="{5D0B02A9-24B3-4F36-8683-2AD26D1E0821}">
+    <text>TODO: set their actual start date and then add how much they produce in 2025</text>
+  </threadedComment>
   <threadedComment ref="G46" dT="2026-01-28T09:05:36.66" personId="{9CD26280-DD25-46DF-A708-6877D8A68AD8}" id="{06D70610-96F7-4BDA-B071-69925D70228B}">
     <text>Danish Energy agency - coal CHP 2020</text>
   </threadedComment>
@@ -2647,7 +2659,7 @@
         <v>80</v>
       </c>
       <c r="T29" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
   </sheetData>
@@ -3990,7 +4002,7 @@
         <v>80</v>
       </c>
       <c r="T34" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="35" spans="2:20" x14ac:dyDescent="0.25">
@@ -4046,7 +4058,7 @@
         <v>80</v>
       </c>
       <c r="T35" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="36" spans="2:20" x14ac:dyDescent="0.25">
@@ -4102,7 +4114,7 @@
         <v>80</v>
       </c>
       <c r="T36" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="37" spans="2:20" x14ac:dyDescent="0.25">
@@ -4158,7 +4170,7 @@
         <v>80</v>
       </c>
       <c r="T37" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="38" spans="2:20" x14ac:dyDescent="0.25">
@@ -4214,7 +4226,7 @@
         <v>80</v>
       </c>
       <c r="T38" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="39" spans="2:20" x14ac:dyDescent="0.25">
@@ -4270,7 +4282,7 @@
         <v>80</v>
       </c>
       <c r="T39" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="40" spans="2:20" x14ac:dyDescent="0.25">
@@ -4326,7 +4338,7 @@
         <v>80</v>
       </c>
       <c r="T40" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="41" spans="2:20" x14ac:dyDescent="0.25">
@@ -4382,7 +4394,7 @@
         <v>80</v>
       </c>
       <c r="T41" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="42" spans="2:20" x14ac:dyDescent="0.25">
@@ -4438,7 +4450,7 @@
         <v>80</v>
       </c>
       <c r="T42" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="43" spans="2:20" x14ac:dyDescent="0.25">
@@ -4494,7 +4506,7 @@
         <v>80</v>
       </c>
       <c r="T43" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="44" spans="2:20" x14ac:dyDescent="0.25">
@@ -4523,7 +4535,7 @@
         <v>80</v>
       </c>
       <c r="T44" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="45" spans="2:20" x14ac:dyDescent="0.25">
@@ -4537,7 +4549,7 @@
         <v>14</v>
       </c>
       <c r="E45">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="F45">
         <v>0.77</v>
@@ -4576,7 +4588,7 @@
         <v>80</v>
       </c>
       <c r="T45" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="46" spans="2:20" x14ac:dyDescent="0.25">
@@ -4590,7 +4602,7 @@
         <v>14</v>
       </c>
       <c r="E46">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="F46">
         <v>0.26</v>
@@ -4629,7 +4641,7 @@
         <v>80</v>
       </c>
       <c r="T46" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="47" spans="2:20" x14ac:dyDescent="0.25">
@@ -4643,7 +4655,7 @@
         <v>14</v>
       </c>
       <c r="E47">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="F47">
         <v>0.185</v>
@@ -4661,7 +4673,7 @@
         <v>3.28</v>
       </c>
       <c r="K47">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="N47" t="s">
         <v>69</v>
@@ -4682,7 +4694,7 @@
         <v>80</v>
       </c>
       <c r="T47" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="48" spans="2:20" x14ac:dyDescent="0.25">
@@ -4696,7 +4708,7 @@
         <v>14</v>
       </c>
       <c r="E48">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="F48">
         <v>0.01</v>
@@ -4735,7 +4747,7 @@
         <v>80</v>
       </c>
       <c r="T48" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="49" spans="2:20" x14ac:dyDescent="0.25">
@@ -4749,7 +4761,7 @@
         <v>14</v>
       </c>
       <c r="E49">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="F49">
         <v>7.6999999999999999E-2</v>
@@ -4788,7 +4800,7 @@
         <v>80</v>
       </c>
       <c r="T49" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="50" spans="2:20" x14ac:dyDescent="0.25">
@@ -4802,7 +4814,7 @@
         <v>14</v>
       </c>
       <c r="E50">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="F50">
         <v>3.9E-2</v>
@@ -4841,7 +4853,7 @@
         <v>80</v>
       </c>
       <c r="T50" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="51" spans="2:20" x14ac:dyDescent="0.25">
@@ -4855,7 +4867,7 @@
         <v>14</v>
       </c>
       <c r="E51">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="F51">
         <v>2.2100000000000002E-2</v>
@@ -4894,7 +4906,7 @@
         <v>80</v>
       </c>
       <c r="T51" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="52" spans="2:20" x14ac:dyDescent="0.25">
@@ -4908,7 +4920,7 @@
         <v>14</v>
       </c>
       <c r="E52">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="F52">
         <v>2.0500000000000001E-2</v>
@@ -4947,7 +4959,7 @@
         <v>80</v>
       </c>
       <c r="T52" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="53" spans="2:20" x14ac:dyDescent="0.25">
@@ -4961,7 +4973,7 @@
         <v>14</v>
       </c>
       <c r="E53">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="F53">
         <v>1.3900000000000001E-2</v>
@@ -5000,7 +5012,7 @@
         <v>80</v>
       </c>
       <c r="T53" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="54" spans="2:20" x14ac:dyDescent="0.25">
@@ -5014,7 +5026,7 @@
         <v>14</v>
       </c>
       <c r="E54">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="F54">
         <v>0.01</v>
@@ -5053,7 +5065,7 @@
         <v>80</v>
       </c>
       <c r="T54" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="55" spans="2:20" x14ac:dyDescent="0.25">
@@ -5067,7 +5079,7 @@
         <v>14</v>
       </c>
       <c r="E55">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="F55">
         <v>0.01</v>
@@ -5106,7 +5118,7 @@
         <v>80</v>
       </c>
       <c r="T55" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="56" spans="2:20" x14ac:dyDescent="0.25">
@@ -5120,7 +5132,7 @@
         <v>14</v>
       </c>
       <c r="E56">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="F56">
         <v>0.01</v>
@@ -5159,7 +5171,7 @@
         <v>80</v>
       </c>
       <c r="T56" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="57" spans="2:20" x14ac:dyDescent="0.25">
@@ -5173,7 +5185,7 @@
         <v>14</v>
       </c>
       <c r="E57">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="F57">
         <v>9.300000000000001E-3</v>
@@ -5212,7 +5224,7 @@
         <v>80</v>
       </c>
       <c r="T57" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="58" spans="2:20" x14ac:dyDescent="0.25">
@@ -5226,7 +5238,7 @@
         <v>14</v>
       </c>
       <c r="E58">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="F58">
         <v>7.0999999999999995E-3</v>
@@ -5265,7 +5277,7 @@
         <v>80</v>
       </c>
       <c r="T58" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="59" spans="2:20" x14ac:dyDescent="0.25">
@@ -5279,7 +5291,7 @@
         <v>14</v>
       </c>
       <c r="E59">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="F59">
         <v>5.7999999999999996E-3</v>
@@ -5318,7 +5330,7 @@
         <v>80</v>
       </c>
       <c r="T59" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="60" spans="2:20" x14ac:dyDescent="0.25">
@@ -5332,7 +5344,7 @@
         <v>14</v>
       </c>
       <c r="E60">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="F60">
         <v>6.4999999999999997E-3</v>
@@ -5371,7 +5383,7 @@
         <v>80</v>
       </c>
       <c r="T60" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="61" spans="2:20" x14ac:dyDescent="0.25">
@@ -5385,7 +5397,7 @@
         <v>14</v>
       </c>
       <c r="E61">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="F61">
         <v>4.0999999999999995E-3</v>
@@ -5424,7 +5436,7 @@
         <v>80</v>
       </c>
       <c r="T61" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="62" spans="2:20" x14ac:dyDescent="0.25">
@@ -5438,7 +5450,7 @@
         <v>14</v>
       </c>
       <c r="E62">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="F62">
         <v>1.4E-3</v>
@@ -5470,7 +5482,7 @@
         <v>14</v>
       </c>
       <c r="E63">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="F63">
         <v>1.8E-3</v>
@@ -5502,7 +5514,7 @@
         <v>14</v>
       </c>
       <c r="E64">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="F64">
         <v>1.6999999999999999E-3</v>
@@ -5534,7 +5546,7 @@
         <v>14</v>
       </c>
       <c r="E65">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="F65">
         <v>1.8E-3</v>
@@ -5566,7 +5578,7 @@
         <v>14</v>
       </c>
       <c r="E66">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="F66">
         <v>1.8E-3</v>
@@ -5598,7 +5610,7 @@
         <v>14</v>
       </c>
       <c r="E67">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="F67">
         <v>1.5E-3</v>
@@ -5630,7 +5642,7 @@
         <v>14</v>
       </c>
       <c r="E68">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="F68">
         <v>1.4E-3</v>
@@ -5662,7 +5674,7 @@
         <v>14</v>
       </c>
       <c r="E69">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="F69">
         <v>1.1999999999999999E-3</v>
@@ -5694,7 +5706,7 @@
         <v>14</v>
       </c>
       <c r="E70">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="F70">
         <v>1.9E-3</v>
@@ -5726,7 +5738,7 @@
         <v>14</v>
       </c>
       <c r="E71">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="F71">
         <v>8.9999999999999998E-4</v>
@@ -5758,7 +5770,7 @@
         <v>14</v>
       </c>
       <c r="E72">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="F72">
         <v>5.0000000000000001E-4</v>

</xml_diff>

<commit_message>
Adding windonshore timsliced ncap_af attempt 2
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/vt_EST_ELC_v1.xlsx
+++ b/VerveStacks_EST/vt_EST_ELC_v1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FC64D7C-6183-4BE9-8A7A-7FE1B408D8FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B5799CF-688A-4AD3-892E-93B97A30D83F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-10470" yWindow="10890" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{21C51102-B905-44E2-89DF-C1A7E31F8D9F}"/>
+    <workbookView xWindow="10" yWindow="10" windowWidth="19180" windowHeight="11260" activeTab="2" xr2:uid="{21C51102-B905-44E2-89DF-C1A7E31F8D9F}"/>
   </bookViews>
   <sheets>
     <sheet name="ccs_retrofits" sheetId="4" r:id="rId1"/>
@@ -118,7 +118,7 @@
     DAE - Wood pellets, Medium 2020</t>
       </text>
     </comment>
-    <comment ref="N77" authorId="5" shapeId="0" xr:uid="{1905391B-2A5F-4643-B2AC-720AD8410CDA}">
+    <comment ref="O77" authorId="5" shapeId="0" xr:uid="{1905391B-2A5F-4643-B2AC-720AD8410CDA}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -760,7 +760,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -775,12 +775,6 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="186"/>
     </font>
   </fonts>
   <fills count="2">
@@ -1176,7 +1170,7 @@
   <threadedComment ref="G50" dT="2026-01-28T11:17:46.06" personId="{9CD26280-DD25-46DF-A708-6877D8A68AD8}" id="{4E0E017D-BAC7-4AA8-B401-A7330F2C0996}">
     <text>DAE - Wood pellets, Medium 2020</text>
   </threadedComment>
-  <threadedComment ref="N77" dT="2026-01-28T08:41:02.80" personId="{9CD26280-DD25-46DF-A708-6877D8A68AD8}" id="{1905391B-2A5F-4643-B2AC-720AD8410CDA}">
+  <threadedComment ref="O77" dT="2026-01-28T08:41:02.80" personId="{9CD26280-DD25-46DF-A708-6877D8A68AD8}" id="{1905391B-2A5F-4643-B2AC-720AD8410CDA}">
     <text>Frequency reserve</text>
   </threadedComment>
   <threadedComment ref="J80" dT="2026-01-27T14:26:51.36" personId="{9CD26280-DD25-46DF-A708-6877D8A68AD8}" id="{3057E3B1-7BF3-4718-B31B-0585028D4313}">
@@ -1188,14 +1182,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C047CB67-FC18-43CA-8AA0-0CA09A11D4D8}">
   <dimension ref="B9:T17"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="46.7109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="40.5703125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="73.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="46.7265625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="40.54296875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="73.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="9" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B9" t="s">
         <v>0</v>
       </c>
@@ -1203,7 +1197,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="10" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B10" t="s">
         <v>1</v>
       </c>
@@ -1259,7 +1253,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="13" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B13" t="s">
         <v>130</v>
       </c>
@@ -1315,7 +1309,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="14" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B14" t="s">
         <v>131</v>
       </c>
@@ -1371,7 +1365,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="15" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B15" t="s">
         <v>132</v>
       </c>
@@ -1427,7 +1421,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="16" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B16" t="s">
         <v>133</v>
       </c>
@@ -1483,7 +1477,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="17" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B17" t="s">
         <v>134</v>
       </c>
@@ -1547,15 +1541,15 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B41A4FEF-80F2-457D-B441-6C3DD45005FF}">
   <dimension ref="B9:T29"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="39.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="39.28515625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="48.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="39.26953125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="39.26953125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="48.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="9" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B9" t="s">
         <v>0</v>
       </c>
@@ -1563,7 +1557,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="10" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B10" t="s">
         <v>1</v>
       </c>
@@ -1619,7 +1613,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="11" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B11" t="s">
         <v>200</v>
       </c>
@@ -1672,7 +1666,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="12" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B12" t="s">
         <v>199</v>
       </c>
@@ -1725,7 +1719,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="13" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B13" t="s">
         <v>86</v>
       </c>
@@ -1781,7 +1775,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="14" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B14" t="s">
         <v>89</v>
       </c>
@@ -1837,7 +1831,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="15" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B15" t="s">
         <v>91</v>
       </c>
@@ -1893,7 +1887,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="16" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B16" t="s">
         <v>93</v>
       </c>
@@ -1949,7 +1943,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="17" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B17" t="s">
         <v>94</v>
       </c>
@@ -2005,7 +1999,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="18" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B18" t="s">
         <v>95</v>
       </c>
@@ -2061,7 +2055,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="19" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B19" t="s">
         <v>96</v>
       </c>
@@ -2117,7 +2111,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="20" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B20" t="s">
         <v>97</v>
       </c>
@@ -2167,7 +2161,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="21" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B21" t="s">
         <v>98</v>
       </c>
@@ -2217,7 +2211,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="22" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B22" t="s">
         <v>99</v>
       </c>
@@ -2273,7 +2267,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="23" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B23" t="s">
         <v>100</v>
       </c>
@@ -2329,7 +2323,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="24" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B24" t="s">
         <v>101</v>
       </c>
@@ -2385,7 +2379,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="25" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B25" t="s">
         <v>103</v>
       </c>
@@ -2441,7 +2435,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="26" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B26" t="s">
         <v>105</v>
       </c>
@@ -2497,7 +2491,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="27" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B27" t="s">
         <v>106</v>
       </c>
@@ -2553,7 +2547,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="28" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B28" t="s">
         <v>107</v>
       </c>
@@ -2609,7 +2603,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="29" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B29" t="s">
         <v>201</v>
       </c>
@@ -2670,32 +2664,34 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A79DDA4A-BC9F-4D47-BDC9-53442001A438}">
-  <dimension ref="B9:T80"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="B9:U80"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="40.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.85546875" customWidth="1"/>
-    <col min="4" max="4" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="12" max="13" width="12" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="40.5703125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="64.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="40.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.81640625" customWidth="1"/>
+    <col min="4" max="4" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.26953125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.54296875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.26953125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.1796875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.81640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="9.26953125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12" customWidth="1"/>
+    <col min="14" max="14" width="12" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="40.54296875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="64.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="9" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B9" t="s">
         <v>0</v>
       </c>
-      <c r="N9" t="s">
+      <c r="O9" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="10" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B10" t="s">
         <v>1</v>
       </c>
@@ -2729,29 +2725,29 @@
       <c r="L10" t="s">
         <v>11</v>
       </c>
-      <c r="N10" t="s">
+      <c r="O10" t="s">
         <v>63</v>
       </c>
-      <c r="O10" t="s">
+      <c r="P10" t="s">
         <v>1</v>
       </c>
-      <c r="P10" t="s">
+      <c r="Q10" t="s">
         <v>64</v>
       </c>
-      <c r="Q10" t="s">
+      <c r="R10" t="s">
         <v>65</v>
       </c>
-      <c r="R10" t="s">
+      <c r="S10" t="s">
         <v>66</v>
       </c>
-      <c r="S10" t="s">
+      <c r="T10" t="s">
         <v>67</v>
       </c>
-      <c r="T10" t="s">
+      <c r="U10" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="11" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B11" t="s">
         <v>17</v>
       </c>
@@ -2782,29 +2778,29 @@
       <c r="K11">
         <v>73</v>
       </c>
-      <c r="N11" t="s">
-        <v>69</v>
-      </c>
       <c r="O11" t="s">
+        <v>69</v>
+      </c>
+      <c r="P11" t="s">
         <v>17</v>
       </c>
-      <c r="P11" t="s">
+      <c r="Q11" t="s">
         <v>76</v>
       </c>
-      <c r="Q11" t="s">
-        <v>71</v>
-      </c>
       <c r="R11" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="S11" t="s">
+        <v>72</v>
+      </c>
+      <c r="T11" t="s">
         <v>73</v>
       </c>
-      <c r="T11" t="s">
+      <c r="U11" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="12" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B12" t="s">
         <v>22</v>
       </c>
@@ -2826,29 +2822,29 @@
       <c r="L12">
         <v>0.14986856628506873</v>
       </c>
-      <c r="N12" t="s">
-        <v>69</v>
-      </c>
       <c r="O12" t="s">
+        <v>69</v>
+      </c>
+      <c r="P12" t="s">
         <v>22</v>
       </c>
-      <c r="P12" t="s">
+      <c r="Q12" t="s">
         <v>78</v>
       </c>
-      <c r="Q12" t="s">
-        <v>71</v>
-      </c>
       <c r="R12" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="S12" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="T12" t="s">
+        <v>80</v>
+      </c>
+      <c r="U12" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="13" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B13" t="s">
         <v>25</v>
       </c>
@@ -2870,29 +2866,29 @@
       <c r="L13">
         <v>0.14986856628506873</v>
       </c>
-      <c r="N13" t="s">
-        <v>69</v>
-      </c>
       <c r="O13" t="s">
+        <v>69</v>
+      </c>
+      <c r="P13" t="s">
         <v>25</v>
       </c>
-      <c r="P13" t="s">
+      <c r="Q13" t="s">
         <v>78</v>
       </c>
-      <c r="Q13" t="s">
-        <v>71</v>
-      </c>
       <c r="R13" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="S13" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="T13" t="s">
+        <v>80</v>
+      </c>
+      <c r="U13" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="14" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B14" t="s">
         <v>27</v>
       </c>
@@ -2914,29 +2910,29 @@
       <c r="L14">
         <v>0.14986856628506873</v>
       </c>
-      <c r="N14" t="s">
-        <v>69</v>
-      </c>
       <c r="O14" t="s">
+        <v>69</v>
+      </c>
+      <c r="P14" t="s">
         <v>27</v>
       </c>
-      <c r="P14" t="s">
+      <c r="Q14" t="s">
         <v>78</v>
       </c>
-      <c r="Q14" t="s">
-        <v>71</v>
-      </c>
       <c r="R14" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="S14" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="T14" t="s">
+        <v>80</v>
+      </c>
+      <c r="U14" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="15" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B15" t="s">
         <v>29</v>
       </c>
@@ -2970,29 +2966,29 @@
       <c r="L15">
         <v>0.1461854238754417</v>
       </c>
-      <c r="N15" t="s">
-        <v>69</v>
-      </c>
       <c r="O15" t="s">
+        <v>69</v>
+      </c>
+      <c r="P15" t="s">
         <v>29</v>
       </c>
-      <c r="P15" t="s">
+      <c r="Q15" t="s">
         <v>78</v>
       </c>
-      <c r="Q15" t="s">
-        <v>71</v>
-      </c>
       <c r="R15" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="S15" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="T15" t="s">
+        <v>80</v>
+      </c>
+      <c r="U15" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="16" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B16" t="s">
         <v>29</v>
       </c>
@@ -3026,29 +3022,29 @@
       <c r="L16">
         <v>0.1461854238754417</v>
       </c>
-      <c r="N16" t="s">
-        <v>69</v>
-      </c>
       <c r="O16" t="s">
+        <v>69</v>
+      </c>
+      <c r="P16" t="s">
         <v>30</v>
       </c>
-      <c r="P16" t="s">
+      <c r="Q16" t="s">
         <v>78</v>
       </c>
-      <c r="Q16" t="s">
-        <v>71</v>
-      </c>
       <c r="R16" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="S16" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="T16" t="s">
+        <v>80</v>
+      </c>
+      <c r="U16" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="17" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B17" t="s">
         <v>30</v>
       </c>
@@ -3082,29 +3078,29 @@
       <c r="L17">
         <v>0.14867925344692126</v>
       </c>
-      <c r="N17" t="s">
-        <v>69</v>
-      </c>
       <c r="O17" t="s">
+        <v>69</v>
+      </c>
+      <c r="P17" t="s">
         <v>32</v>
       </c>
-      <c r="P17" t="s">
+      <c r="Q17" t="s">
         <v>78</v>
       </c>
-      <c r="Q17" t="s">
-        <v>71</v>
-      </c>
       <c r="R17" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="S17" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="T17" t="s">
+        <v>80</v>
+      </c>
+      <c r="U17" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="18" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B18" t="s">
         <v>32</v>
       </c>
@@ -3138,29 +3134,29 @@
       <c r="L18">
         <v>0.14701259708091721</v>
       </c>
-      <c r="N18" t="s">
-        <v>69</v>
-      </c>
       <c r="O18" t="s">
+        <v>69</v>
+      </c>
+      <c r="P18" t="s">
         <v>34</v>
       </c>
-      <c r="P18" t="s">
+      <c r="Q18" t="s">
         <v>78</v>
       </c>
-      <c r="Q18" t="s">
-        <v>71</v>
-      </c>
       <c r="R18" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="S18" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="T18" t="s">
+        <v>80</v>
+      </c>
+      <c r="U18" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="19" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B19" t="s">
         <v>34</v>
       </c>
@@ -3194,29 +3190,29 @@
       <c r="L19">
         <v>0.15309859852159369</v>
       </c>
-      <c r="N19" t="s">
-        <v>69</v>
-      </c>
       <c r="O19" t="s">
+        <v>69</v>
+      </c>
+      <c r="P19" t="s">
         <v>35</v>
       </c>
-      <c r="P19" t="s">
+      <c r="Q19" t="s">
         <v>78</v>
       </c>
-      <c r="Q19" t="s">
-        <v>71</v>
-      </c>
       <c r="R19" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="S19" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="T19" t="s">
+        <v>80</v>
+      </c>
+      <c r="U19" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="20" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B20" t="s">
         <v>34</v>
       </c>
@@ -3250,29 +3246,29 @@
       <c r="L20">
         <v>0.15309859852159369</v>
       </c>
-      <c r="N20" t="s">
-        <v>69</v>
-      </c>
       <c r="O20" t="s">
+        <v>69</v>
+      </c>
+      <c r="P20" t="s">
         <v>37</v>
       </c>
-      <c r="P20" t="s">
+      <c r="Q20" t="s">
         <v>78</v>
       </c>
-      <c r="Q20" t="s">
-        <v>71</v>
-      </c>
       <c r="R20" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="S20" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="T20" t="s">
+        <v>80</v>
+      </c>
+      <c r="U20" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="21" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B21" t="s">
         <v>35</v>
       </c>
@@ -3306,29 +3302,29 @@
       <c r="L21">
         <v>0.15619560585976827</v>
       </c>
-      <c r="N21" t="s">
-        <v>69</v>
-      </c>
       <c r="O21" t="s">
+        <v>69</v>
+      </c>
+      <c r="P21" t="s">
         <v>39</v>
       </c>
-      <c r="P21" t="s">
+      <c r="Q21" t="s">
         <v>78</v>
       </c>
-      <c r="Q21" t="s">
-        <v>71</v>
-      </c>
       <c r="R21" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="S21" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="T21" t="s">
+        <v>80</v>
+      </c>
+      <c r="U21" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="22" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B22" t="s">
         <v>37</v>
       </c>
@@ -3362,29 +3358,29 @@
       <c r="L22">
         <v>0.14537310453496291</v>
       </c>
-      <c r="N22" t="s">
-        <v>69</v>
-      </c>
       <c r="O22" t="s">
+        <v>69</v>
+      </c>
+      <c r="P22" t="s">
         <v>40</v>
       </c>
-      <c r="P22" t="s">
+      <c r="Q22" t="s">
         <v>78</v>
       </c>
-      <c r="Q22" t="s">
-        <v>71</v>
-      </c>
       <c r="R22" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="S22" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="T22" t="s">
+        <v>80</v>
+      </c>
+      <c r="U22" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="23" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B23" t="s">
         <v>39</v>
       </c>
@@ -3418,29 +3414,29 @@
       <c r="L23">
         <v>0.14763873655681015</v>
       </c>
-      <c r="N23" t="s">
-        <v>69</v>
-      </c>
       <c r="O23" t="s">
+        <v>69</v>
+      </c>
+      <c r="P23" t="s">
         <v>42</v>
       </c>
-      <c r="P23" t="s">
+      <c r="Q23" t="s">
         <v>78</v>
       </c>
-      <c r="Q23" t="s">
-        <v>71</v>
-      </c>
       <c r="R23" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="S23" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="T23" t="s">
+        <v>80</v>
+      </c>
+      <c r="U23" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="24" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B24" t="s">
         <v>40</v>
       </c>
@@ -3474,29 +3470,29 @@
       <c r="L24">
         <v>0.1532628310027955</v>
       </c>
-      <c r="N24" t="s">
-        <v>69</v>
-      </c>
       <c r="O24" t="s">
+        <v>69</v>
+      </c>
+      <c r="P24" t="s">
         <v>44</v>
       </c>
-      <c r="P24" t="s">
+      <c r="Q24" t="s">
         <v>78</v>
       </c>
-      <c r="Q24" t="s">
-        <v>71</v>
-      </c>
       <c r="R24" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="S24" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="T24" t="s">
+        <v>80</v>
+      </c>
+      <c r="U24" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="25" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B25" t="s">
         <v>40</v>
       </c>
@@ -3530,29 +3526,29 @@
       <c r="L25">
         <v>0.1532628310027955</v>
       </c>
-      <c r="N25" t="s">
-        <v>69</v>
-      </c>
       <c r="O25" t="s">
+        <v>69</v>
+      </c>
+      <c r="P25" t="s">
         <v>47</v>
       </c>
-      <c r="P25" t="s">
+      <c r="Q25" t="s">
         <v>78</v>
       </c>
-      <c r="Q25" t="s">
-        <v>71</v>
-      </c>
       <c r="R25" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="S25" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="T25" t="s">
+        <v>80</v>
+      </c>
+      <c r="U25" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="26" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B26" t="s">
         <v>42</v>
       </c>
@@ -3586,29 +3582,29 @@
       <c r="L26">
         <v>0.1451997589052581</v>
       </c>
-      <c r="N26" t="s">
-        <v>69</v>
-      </c>
       <c r="O26" t="s">
+        <v>69</v>
+      </c>
+      <c r="P26" t="s">
         <v>49</v>
       </c>
-      <c r="P26" t="s">
+      <c r="Q26" t="s">
         <v>78</v>
       </c>
-      <c r="Q26" t="s">
-        <v>71</v>
-      </c>
       <c r="R26" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="S26" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="T26" t="s">
+        <v>80</v>
+      </c>
+      <c r="U26" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="27" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B27" t="s">
         <v>44</v>
       </c>
@@ -3627,32 +3623,32 @@
       <c r="G27">
         <v>0.33123000000000002</v>
       </c>
-      <c r="L27">
+      <c r="M27">
         <v>0.42012333946150526</v>
       </c>
-      <c r="N27" t="s">
-        <v>69</v>
-      </c>
       <c r="O27" t="s">
+        <v>69</v>
+      </c>
+      <c r="P27" t="s">
         <v>51</v>
       </c>
-      <c r="P27" t="s">
+      <c r="Q27" t="s">
         <v>78</v>
       </c>
-      <c r="Q27" t="s">
-        <v>71</v>
-      </c>
       <c r="R27" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="S27" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="T27" t="s">
+        <v>80</v>
+      </c>
+      <c r="U27" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="28" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B28" t="s">
         <v>47</v>
       </c>
@@ -3671,32 +3667,32 @@
       <c r="G28">
         <v>0.33123000000000002</v>
       </c>
-      <c r="L28">
+      <c r="M28">
         <v>0.42012333946150526</v>
       </c>
-      <c r="N28" t="s">
-        <v>69</v>
-      </c>
       <c r="O28" t="s">
+        <v>69</v>
+      </c>
+      <c r="P28" t="s">
         <v>53</v>
       </c>
-      <c r="P28" t="s">
+      <c r="Q28" t="s">
         <v>78</v>
       </c>
-      <c r="Q28" t="s">
-        <v>71</v>
-      </c>
       <c r="R28" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="S28" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="T28" t="s">
+        <v>80</v>
+      </c>
+      <c r="U28" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="29" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B29" t="s">
         <v>49</v>
       </c>
@@ -3715,32 +3711,32 @@
       <c r="G29">
         <v>0.33123000000000002</v>
       </c>
-      <c r="L29">
+      <c r="M29">
         <v>0.42012333946150526</v>
       </c>
-      <c r="N29" t="s">
-        <v>69</v>
-      </c>
       <c r="O29" t="s">
+        <v>69</v>
+      </c>
+      <c r="P29" t="s">
         <v>55</v>
       </c>
-      <c r="P29" t="s">
+      <c r="Q29" t="s">
         <v>78</v>
       </c>
-      <c r="Q29" t="s">
-        <v>71</v>
-      </c>
       <c r="R29" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="S29" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="T29" t="s">
+        <v>80</v>
+      </c>
+      <c r="U29" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="30" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B30" t="s">
         <v>51</v>
       </c>
@@ -3771,32 +3767,32 @@
       <c r="K30">
         <v>46</v>
       </c>
-      <c r="L30">
+      <c r="M30">
         <v>0.47763777043344691</v>
       </c>
-      <c r="N30" t="s">
-        <v>69</v>
-      </c>
       <c r="O30" t="s">
+        <v>69</v>
+      </c>
+      <c r="P30" t="s">
         <v>57</v>
       </c>
-      <c r="P30" t="s">
+      <c r="Q30" t="s">
         <v>78</v>
       </c>
-      <c r="Q30" t="s">
-        <v>71</v>
-      </c>
       <c r="R30" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="S30" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="T30" t="s">
+        <v>80</v>
+      </c>
+      <c r="U30" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="31" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B31" t="s">
         <v>53</v>
       </c>
@@ -3827,32 +3823,32 @@
       <c r="K31">
         <v>45</v>
       </c>
-      <c r="L31">
+      <c r="M31">
         <v>0.47814004703314078</v>
       </c>
-      <c r="N31" t="s">
-        <v>69</v>
-      </c>
       <c r="O31" t="s">
+        <v>69</v>
+      </c>
+      <c r="P31" t="s">
         <v>59</v>
       </c>
-      <c r="P31" t="s">
+      <c r="Q31" t="s">
         <v>78</v>
       </c>
-      <c r="Q31" t="s">
-        <v>71</v>
-      </c>
       <c r="R31" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="S31" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="T31" t="s">
+        <v>80</v>
+      </c>
+      <c r="U31" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="32" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B32" t="s">
         <v>53</v>
       </c>
@@ -3883,32 +3879,32 @@
       <c r="K32">
         <v>40</v>
       </c>
-      <c r="L32">
+      <c r="M32">
         <v>0.47814004703314084</v>
       </c>
-      <c r="N32" t="s">
-        <v>69</v>
-      </c>
       <c r="O32" t="s">
+        <v>69</v>
+      </c>
+      <c r="P32" t="s">
         <v>61</v>
       </c>
-      <c r="P32" t="s">
+      <c r="Q32" t="s">
         <v>81</v>
       </c>
-      <c r="Q32" t="s">
-        <v>71</v>
-      </c>
       <c r="R32" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="S32" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="T32" t="s">
+        <v>80</v>
+      </c>
+      <c r="U32" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="33" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B33" t="s">
         <v>53</v>
       </c>
@@ -3939,17 +3935,17 @@
       <c r="K33">
         <v>35</v>
       </c>
-      <c r="L33">
+      <c r="M33">
         <v>0.47814004703314078</v>
       </c>
-      <c r="N33" t="s">
+      <c r="O33" t="s">
         <v>140</v>
       </c>
-      <c r="O33" s="1" t="s">
+      <c r="P33" s="1" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="34" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B34" t="s">
         <v>55</v>
       </c>
@@ -3980,32 +3976,32 @@
       <c r="K34">
         <v>48</v>
       </c>
-      <c r="L34">
+      <c r="M34">
         <v>0.40144059976798208</v>
       </c>
-      <c r="N34" t="s">
-        <v>69</v>
-      </c>
       <c r="O34" t="s">
+        <v>69</v>
+      </c>
+      <c r="P34" t="s">
         <v>194</v>
       </c>
-      <c r="P34" t="s">
+      <c r="Q34" t="s">
         <v>163</v>
       </c>
-      <c r="Q34" t="s">
-        <v>71</v>
-      </c>
       <c r="R34" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="S34" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="T34" t="s">
+        <v>80</v>
+      </c>
+      <c r="U34" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="35" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B35" t="s">
         <v>55</v>
       </c>
@@ -4036,32 +4032,32 @@
       <c r="K35">
         <v>44</v>
       </c>
-      <c r="L35">
+      <c r="M35">
         <v>0.40144059976798202</v>
       </c>
-      <c r="N35" t="s">
-        <v>69</v>
-      </c>
       <c r="O35" t="s">
+        <v>69</v>
+      </c>
+      <c r="P35" t="s">
         <v>193</v>
       </c>
-      <c r="P35" t="s">
+      <c r="Q35" t="s">
         <v>148</v>
       </c>
-      <c r="Q35" t="s">
-        <v>71</v>
-      </c>
       <c r="R35" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="S35" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="T35" t="s">
+        <v>80</v>
+      </c>
+      <c r="U35" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="36" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B36" t="s">
         <v>55</v>
       </c>
@@ -4092,32 +4088,32 @@
       <c r="K36">
         <v>43</v>
       </c>
-      <c r="L36">
+      <c r="M36">
         <v>0.40144059976798202</v>
       </c>
-      <c r="N36" t="s">
-        <v>69</v>
-      </c>
       <c r="O36" t="s">
+        <v>69</v>
+      </c>
+      <c r="P36" t="s">
         <v>195</v>
       </c>
-      <c r="P36" t="s">
+      <c r="Q36" t="s">
         <v>149</v>
       </c>
-      <c r="Q36" t="s">
-        <v>71</v>
-      </c>
       <c r="R36" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="S36" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="T36" t="s">
+        <v>80</v>
+      </c>
+      <c r="U36" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="37" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B37" t="s">
         <v>55</v>
       </c>
@@ -4148,32 +4144,32 @@
       <c r="K37">
         <v>32</v>
       </c>
-      <c r="L37">
+      <c r="M37">
         <v>0.40144059976798208</v>
       </c>
-      <c r="N37" t="s">
-        <v>69</v>
-      </c>
       <c r="O37" t="s">
+        <v>69</v>
+      </c>
+      <c r="P37" t="s">
         <v>196</v>
       </c>
-      <c r="P37" t="s">
+      <c r="Q37" t="s">
         <v>150</v>
       </c>
-      <c r="Q37" t="s">
-        <v>71</v>
-      </c>
       <c r="R37" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="S37" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="T37" t="s">
+        <v>80</v>
+      </c>
+      <c r="U37" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="38" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B38" t="s">
         <v>55</v>
       </c>
@@ -4204,32 +4200,32 @@
       <c r="K38">
         <v>31</v>
       </c>
-      <c r="L38">
+      <c r="M38">
         <v>0.40144059976798202</v>
       </c>
-      <c r="N38" t="s">
-        <v>69</v>
-      </c>
       <c r="O38" t="s">
+        <v>69</v>
+      </c>
+      <c r="P38" t="s">
         <v>142</v>
       </c>
-      <c r="P38" t="s">
+      <c r="Q38" t="s">
         <v>161</v>
       </c>
-      <c r="Q38" t="s">
-        <v>71</v>
-      </c>
       <c r="R38" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="S38" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="T38" t="s">
+        <v>80</v>
+      </c>
+      <c r="U38" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="39" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B39" t="s">
         <v>57</v>
       </c>
@@ -4260,32 +4256,32 @@
       <c r="K39">
         <v>32</v>
       </c>
-      <c r="L39">
+      <c r="M39">
         <v>0.365520596150406</v>
       </c>
-      <c r="N39" t="s">
-        <v>69</v>
-      </c>
       <c r="O39" t="s">
+        <v>69</v>
+      </c>
+      <c r="P39" t="s">
         <v>143</v>
       </c>
-      <c r="P39" t="s">
+      <c r="Q39" t="s">
         <v>151</v>
       </c>
-      <c r="Q39" t="s">
-        <v>71</v>
-      </c>
       <c r="R39" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="S39" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="T39" t="s">
+        <v>80</v>
+      </c>
+      <c r="U39" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="40" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B40" t="s">
         <v>59</v>
       </c>
@@ -4316,32 +4312,32 @@
       <c r="K40">
         <v>50</v>
       </c>
-      <c r="L40">
+      <c r="M40">
         <v>0.41047488326249421</v>
       </c>
-      <c r="N40" t="s">
-        <v>69</v>
-      </c>
       <c r="O40" t="s">
+        <v>69</v>
+      </c>
+      <c r="P40" t="s">
         <v>144</v>
       </c>
-      <c r="P40" t="s">
+      <c r="Q40" t="s">
         <v>152</v>
       </c>
-      <c r="Q40" t="s">
-        <v>71</v>
-      </c>
       <c r="R40" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="S40" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="T40" t="s">
+        <v>80</v>
+      </c>
+      <c r="U40" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="41" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B41" t="s">
         <v>59</v>
       </c>
@@ -4372,32 +4368,32 @@
       <c r="K41">
         <v>43</v>
       </c>
-      <c r="L41">
+      <c r="M41">
         <v>0.41047488326249421</v>
       </c>
-      <c r="N41" t="s">
-        <v>69</v>
-      </c>
       <c r="O41" t="s">
+        <v>69</v>
+      </c>
+      <c r="P41" t="s">
         <v>145</v>
       </c>
-      <c r="P41" t="s">
+      <c r="Q41" t="s">
         <v>153</v>
       </c>
-      <c r="Q41" t="s">
-        <v>71</v>
-      </c>
       <c r="R41" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="S41" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="T41" t="s">
+        <v>80</v>
+      </c>
+      <c r="U41" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="42" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B42" t="s">
         <v>59</v>
       </c>
@@ -4428,32 +4424,32 @@
       <c r="K42">
         <v>42</v>
       </c>
-      <c r="L42">
+      <c r="M42">
         <v>0.41047488326249421</v>
       </c>
-      <c r="N42" t="s">
-        <v>69</v>
-      </c>
       <c r="O42" t="s">
+        <v>69</v>
+      </c>
+      <c r="P42" t="s">
         <v>146</v>
       </c>
-      <c r="P42" t="s">
+      <c r="Q42" t="s">
         <v>147</v>
       </c>
-      <c r="Q42" t="s">
-        <v>71</v>
-      </c>
       <c r="R42" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="S42" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="T42" t="s">
+        <v>80</v>
+      </c>
+      <c r="U42" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="43" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B43" t="s">
         <v>61</v>
       </c>
@@ -4484,61 +4480,61 @@
       <c r="K43">
         <v>31</v>
       </c>
-      <c r="L43">
+      <c r="M43">
         <v>0.365520596150406</v>
       </c>
-      <c r="N43" t="s">
-        <v>69</v>
-      </c>
       <c r="O43" t="s">
+        <v>69</v>
+      </c>
+      <c r="P43" t="s">
         <v>197</v>
       </c>
-      <c r="P43" t="s">
+      <c r="Q43" t="s">
         <v>162</v>
       </c>
-      <c r="Q43" t="s">
-        <v>71</v>
-      </c>
       <c r="R43" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="S43" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="T43" t="s">
+        <v>80</v>
+      </c>
+      <c r="U43" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="44" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B44" t="s">
         <v>140</v>
       </c>
       <c r="C44" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="N44" t="s">
-        <v>69</v>
-      </c>
       <c r="O44" t="s">
+        <v>69</v>
+      </c>
+      <c r="P44" t="s">
         <v>154</v>
       </c>
-      <c r="P44" t="s">
+      <c r="Q44" t="s">
         <v>155</v>
       </c>
-      <c r="Q44" t="s">
-        <v>71</v>
-      </c>
       <c r="R44" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="S44" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="T44" t="s">
+        <v>80</v>
+      </c>
+      <c r="U44" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="45" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B45" t="s">
         <v>196</v>
       </c>
@@ -4569,29 +4565,29 @@
       <c r="K45">
         <v>40</v>
       </c>
-      <c r="N45" t="s">
-        <v>69</v>
-      </c>
       <c r="O45" t="s">
+        <v>69</v>
+      </c>
+      <c r="P45" t="s">
         <v>156</v>
       </c>
-      <c r="P45" t="s">
+      <c r="Q45" t="s">
         <v>157</v>
       </c>
-      <c r="Q45" t="s">
-        <v>71</v>
-      </c>
       <c r="R45" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="S45" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="T45" t="s">
+        <v>80</v>
+      </c>
+      <c r="U45" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="46" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B46" t="s">
         <v>194</v>
       </c>
@@ -4622,29 +4618,29 @@
       <c r="K46">
         <v>40</v>
       </c>
-      <c r="N46" t="s">
-        <v>69</v>
-      </c>
       <c r="O46" t="s">
+        <v>69</v>
+      </c>
+      <c r="P46" t="s">
         <v>170</v>
       </c>
-      <c r="P46" t="s">
+      <c r="Q46" t="s">
         <v>171</v>
       </c>
-      <c r="Q46" t="s">
-        <v>71</v>
-      </c>
       <c r="R46" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="S46" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="T46" t="s">
+        <v>80</v>
+      </c>
+      <c r="U46" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="47" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B47" t="s">
         <v>193</v>
       </c>
@@ -4675,29 +4671,29 @@
       <c r="K47">
         <v>40</v>
       </c>
-      <c r="N47" t="s">
-        <v>69</v>
-      </c>
       <c r="O47" t="s">
+        <v>69</v>
+      </c>
+      <c r="P47" t="s">
         <v>158</v>
       </c>
-      <c r="P47" t="s">
+      <c r="Q47" t="s">
         <v>159</v>
       </c>
-      <c r="Q47" t="s">
-        <v>71</v>
-      </c>
       <c r="R47" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="S47" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="T47" t="s">
+        <v>80</v>
+      </c>
+      <c r="U47" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="48" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B48" t="s">
         <v>195</v>
       </c>
@@ -4728,29 +4724,29 @@
       <c r="K48">
         <v>40</v>
       </c>
-      <c r="N48" t="s">
-        <v>69</v>
-      </c>
       <c r="O48" t="s">
+        <v>69</v>
+      </c>
+      <c r="P48" t="s">
         <v>169</v>
       </c>
-      <c r="P48" t="s">
+      <c r="Q48" t="s">
         <v>160</v>
       </c>
-      <c r="Q48" t="s">
-        <v>71</v>
-      </c>
       <c r="R48" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="S48" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="T48" t="s">
+        <v>80</v>
+      </c>
+      <c r="U48" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="49" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B49" t="s">
         <v>142</v>
       </c>
@@ -4781,29 +4777,29 @@
       <c r="K49">
         <v>40</v>
       </c>
-      <c r="N49" t="s">
-        <v>69</v>
-      </c>
       <c r="O49" t="s">
+        <v>69</v>
+      </c>
+      <c r="P49" t="s">
         <v>164</v>
       </c>
-      <c r="P49" t="s">
+      <c r="Q49" t="s">
         <v>165</v>
       </c>
-      <c r="Q49" t="s">
-        <v>71</v>
-      </c>
       <c r="R49" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="S49" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="T49" t="s">
+        <v>80</v>
+      </c>
+      <c r="U49" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="50" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B50" t="s">
         <v>143</v>
       </c>
@@ -4834,29 +4830,29 @@
       <c r="K50">
         <v>40</v>
       </c>
-      <c r="N50" t="s">
-        <v>69</v>
-      </c>
       <c r="O50" t="s">
+        <v>69</v>
+      </c>
+      <c r="P50" t="s">
         <v>168</v>
       </c>
-      <c r="P50" t="s">
+      <c r="Q50" t="s">
         <v>166</v>
       </c>
-      <c r="Q50" t="s">
-        <v>71</v>
-      </c>
       <c r="R50" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="S50" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="T50" t="s">
+        <v>80</v>
+      </c>
+      <c r="U50" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="51" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B51" t="s">
         <v>144</v>
       </c>
@@ -4887,29 +4883,29 @@
       <c r="K51">
         <v>40</v>
       </c>
-      <c r="N51" t="s">
-        <v>69</v>
-      </c>
       <c r="O51" t="s">
+        <v>69</v>
+      </c>
+      <c r="P51" t="s">
         <v>198</v>
       </c>
-      <c r="P51" t="s">
+      <c r="Q51" t="s">
         <v>167</v>
       </c>
-      <c r="Q51" t="s">
-        <v>71</v>
-      </c>
       <c r="R51" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="S51" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="T51" t="s">
+        <v>80</v>
+      </c>
+      <c r="U51" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="52" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B52" t="s">
         <v>145</v>
       </c>
@@ -4940,29 +4936,29 @@
       <c r="K52">
         <v>40</v>
       </c>
-      <c r="N52" t="s">
-        <v>69</v>
-      </c>
       <c r="O52" t="s">
+        <v>69</v>
+      </c>
+      <c r="P52" t="s">
         <v>172</v>
       </c>
-      <c r="P52" t="s">
+      <c r="Q52" t="s">
         <v>173</v>
       </c>
-      <c r="Q52" t="s">
-        <v>71</v>
-      </c>
       <c r="R52" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="S52" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="T52" t="s">
+        <v>80</v>
+      </c>
+      <c r="U52" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="53" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="53" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B53" t="s">
         <v>146</v>
       </c>
@@ -4993,29 +4989,29 @@
       <c r="K53">
         <v>40</v>
       </c>
-      <c r="N53" t="s">
-        <v>69</v>
-      </c>
       <c r="O53" t="s">
+        <v>69</v>
+      </c>
+      <c r="P53" t="s">
         <v>174</v>
       </c>
-      <c r="P53" t="s">
+      <c r="Q53" t="s">
         <v>175</v>
       </c>
-      <c r="Q53" t="s">
-        <v>71</v>
-      </c>
       <c r="R53" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="S53" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="T53" t="s">
+        <v>80</v>
+      </c>
+      <c r="U53" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="54" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="54" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B54" t="s">
         <v>197</v>
       </c>
@@ -5046,29 +5042,29 @@
       <c r="K54">
         <v>40</v>
       </c>
-      <c r="N54" t="s">
-        <v>69</v>
-      </c>
       <c r="O54" t="s">
+        <v>69</v>
+      </c>
+      <c r="P54" t="s">
         <v>176</v>
       </c>
-      <c r="P54" t="s">
+      <c r="Q54" t="s">
         <v>177</v>
       </c>
-      <c r="Q54" t="s">
-        <v>71</v>
-      </c>
       <c r="R54" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="S54" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="T54" t="s">
+        <v>80</v>
+      </c>
+      <c r="U54" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="55" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="55" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B55" t="s">
         <v>154</v>
       </c>
@@ -5099,29 +5095,29 @@
       <c r="K55">
         <v>40</v>
       </c>
-      <c r="N55" t="s">
-        <v>69</v>
-      </c>
       <c r="O55" t="s">
+        <v>69</v>
+      </c>
+      <c r="P55" t="s">
         <v>178</v>
       </c>
-      <c r="P55" t="s">
+      <c r="Q55" t="s">
         <v>179</v>
       </c>
-      <c r="Q55" t="s">
-        <v>71</v>
-      </c>
       <c r="R55" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="S55" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="T55" t="s">
+        <v>80</v>
+      </c>
+      <c r="U55" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="56" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="56" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B56" t="s">
         <v>156</v>
       </c>
@@ -5152,29 +5148,29 @@
       <c r="K56">
         <v>40</v>
       </c>
-      <c r="N56" t="s">
-        <v>69</v>
-      </c>
       <c r="O56" t="s">
+        <v>69</v>
+      </c>
+      <c r="P56" t="s">
         <v>180</v>
       </c>
-      <c r="P56" t="s">
+      <c r="Q56" t="s">
         <v>181</v>
       </c>
-      <c r="Q56" t="s">
-        <v>71</v>
-      </c>
       <c r="R56" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="S56" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="T56" t="s">
+        <v>80</v>
+      </c>
+      <c r="U56" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="57" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="57" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B57" t="s">
         <v>170</v>
       </c>
@@ -5205,29 +5201,29 @@
       <c r="K57">
         <v>40</v>
       </c>
-      <c r="N57" t="s">
-        <v>69</v>
-      </c>
       <c r="O57" t="s">
+        <v>69</v>
+      </c>
+      <c r="P57" t="s">
         <v>182</v>
       </c>
-      <c r="P57" t="s">
+      <c r="Q57" t="s">
         <v>183</v>
       </c>
-      <c r="Q57" t="s">
-        <v>71</v>
-      </c>
       <c r="R57" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="S57" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="T57" t="s">
+        <v>80</v>
+      </c>
+      <c r="U57" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="58" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="58" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B58" t="s">
         <v>158</v>
       </c>
@@ -5258,29 +5254,29 @@
       <c r="K58">
         <v>40</v>
       </c>
-      <c r="N58" t="s">
-        <v>69</v>
-      </c>
       <c r="O58" t="s">
+        <v>69</v>
+      </c>
+      <c r="P58" t="s">
         <v>184</v>
       </c>
-      <c r="P58" t="s">
+      <c r="Q58" t="s">
         <v>185</v>
       </c>
-      <c r="Q58" t="s">
-        <v>71</v>
-      </c>
       <c r="R58" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="S58" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="T58" t="s">
+        <v>80</v>
+      </c>
+      <c r="U58" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="59" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="59" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B59" t="s">
         <v>169</v>
       </c>
@@ -5311,29 +5307,29 @@
       <c r="K59">
         <v>40</v>
       </c>
-      <c r="N59" t="s">
-        <v>69</v>
-      </c>
       <c r="O59" t="s">
+        <v>69</v>
+      </c>
+      <c r="P59" t="s">
         <v>186</v>
       </c>
-      <c r="P59" t="s">
+      <c r="Q59" t="s">
         <v>188</v>
       </c>
-      <c r="Q59" t="s">
-        <v>71</v>
-      </c>
       <c r="R59" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="S59" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="T59" t="s">
+        <v>80</v>
+      </c>
+      <c r="U59" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="60" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="60" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B60" t="s">
         <v>164</v>
       </c>
@@ -5364,29 +5360,29 @@
       <c r="K60">
         <v>40</v>
       </c>
-      <c r="N60" t="s">
-        <v>69</v>
-      </c>
       <c r="O60" t="s">
+        <v>69</v>
+      </c>
+      <c r="P60" t="s">
         <v>187</v>
       </c>
-      <c r="P60" t="s">
+      <c r="Q60" t="s">
         <v>189</v>
       </c>
-      <c r="Q60" t="s">
-        <v>71</v>
-      </c>
       <c r="R60" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="S60" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="T60" t="s">
+        <v>80</v>
+      </c>
+      <c r="U60" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="61" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="61" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B61" t="s">
         <v>168</v>
       </c>
@@ -5417,29 +5413,29 @@
       <c r="K61">
         <v>40</v>
       </c>
-      <c r="N61" t="s">
-        <v>69</v>
-      </c>
       <c r="O61" t="s">
+        <v>69</v>
+      </c>
+      <c r="P61" t="s">
         <v>190</v>
       </c>
-      <c r="P61" t="s">
+      <c r="Q61" t="s">
         <v>191</v>
       </c>
-      <c r="Q61" t="s">
-        <v>71</v>
-      </c>
       <c r="R61" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="S61" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="T61" t="s">
+        <v>80</v>
+      </c>
+      <c r="U61" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="62" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="62" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B62" t="s">
         <v>198</v>
       </c>
@@ -5471,7 +5467,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="63" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="63" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B63" t="s">
         <v>172</v>
       </c>
@@ -5503,7 +5499,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="64" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="64" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B64" t="s">
         <v>174</v>
       </c>
@@ -5535,7 +5531,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="65" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="65" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B65" t="s">
         <v>176</v>
       </c>
@@ -5567,7 +5563,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="66" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="66" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B66" t="s">
         <v>178</v>
       </c>
@@ -5599,7 +5595,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="67" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="67" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B67" t="s">
         <v>180</v>
       </c>
@@ -5631,7 +5627,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="68" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="68" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B68" t="s">
         <v>182</v>
       </c>
@@ -5663,7 +5659,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="69" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="69" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B69" t="s">
         <v>184</v>
       </c>
@@ -5695,7 +5691,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="70" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="70" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B70" t="s">
         <v>186</v>
       </c>
@@ -5727,7 +5723,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="71" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="71" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B71" t="s">
         <v>187</v>
       </c>
@@ -5759,7 +5755,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="72" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="72" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B72" t="s">
         <v>190</v>
       </c>
@@ -5791,7 +5787,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="77" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="77" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B77" t="s">
         <v>20</v>
       </c>
@@ -5822,29 +5818,29 @@
       <c r="K77">
         <v>42</v>
       </c>
-      <c r="N77" t="s">
-        <v>69</v>
-      </c>
       <c r="O77" t="s">
+        <v>69</v>
+      </c>
+      <c r="P77" t="s">
         <v>20</v>
       </c>
-      <c r="P77" t="s">
+      <c r="Q77" t="s">
         <v>79</v>
       </c>
-      <c r="Q77" t="s">
-        <v>71</v>
-      </c>
       <c r="R77" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="S77" t="s">
+        <v>72</v>
+      </c>
+      <c r="T77" t="s">
         <v>73</v>
       </c>
-      <c r="T77" t="s">
+      <c r="U77" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="78" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="78" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B78" t="s">
         <v>15</v>
       </c>
@@ -5863,29 +5859,29 @@
       <c r="G78">
         <v>0.33123000000000002</v>
       </c>
-      <c r="N78" t="s">
-        <v>69</v>
-      </c>
       <c r="O78" t="s">
+        <v>69</v>
+      </c>
+      <c r="P78" t="s">
         <v>15</v>
       </c>
-      <c r="P78" t="s">
+      <c r="Q78" t="s">
         <v>75</v>
       </c>
-      <c r="Q78" t="s">
-        <v>71</v>
-      </c>
       <c r="R78" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="S78" t="s">
+        <v>72</v>
+      </c>
+      <c r="T78" t="s">
         <v>73</v>
       </c>
-      <c r="T78" t="s">
+      <c r="U78" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="79" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="79" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B79" t="s">
         <v>18</v>
       </c>
@@ -5904,29 +5900,29 @@
       <c r="G79">
         <v>0.33123000000000002</v>
       </c>
-      <c r="N79" t="s">
-        <v>69</v>
-      </c>
       <c r="O79" t="s">
+        <v>69</v>
+      </c>
+      <c r="P79" t="s">
         <v>18</v>
       </c>
-      <c r="P79" t="s">
+      <c r="Q79" t="s">
         <v>78</v>
       </c>
-      <c r="Q79" t="s">
-        <v>71</v>
-      </c>
       <c r="R79" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="S79" t="s">
+        <v>72</v>
+      </c>
+      <c r="T79" t="s">
         <v>73</v>
       </c>
-      <c r="T79" t="s">
+      <c r="U79" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="80" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="80" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B80" t="s">
         <v>12</v>
       </c>
@@ -5957,25 +5953,25 @@
       <c r="K80">
         <v>50</v>
       </c>
-      <c r="N80" t="s">
-        <v>69</v>
-      </c>
       <c r="O80" t="s">
+        <v>69</v>
+      </c>
+      <c r="P80" t="s">
         <v>12</v>
       </c>
-      <c r="P80" t="s">
+      <c r="Q80" t="s">
         <v>70</v>
       </c>
-      <c r="Q80" t="s">
-        <v>71</v>
-      </c>
       <c r="R80" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="S80" t="s">
+        <v>72</v>
+      </c>
+      <c r="T80" t="s">
         <v>73</v>
       </c>
-      <c r="T80" t="s">
+      <c r="U80" t="s">
         <v>74</v>
       </c>
     </row>
@@ -5988,7 +5984,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8CEAB3BD-FD82-4128-8F02-FA58B77D374D}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
chanigng FOM of bioenergy
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/vt_EST_ELC_v1.xlsx
+++ b/VerveStacks_EST/vt_EST_ELC_v1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F74BA55-79F9-4208-A8DD-5D96FD3C5C47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D0A5F67-D97C-4A31-9F28-9DE87309EC24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-38520" yWindow="-5220" windowWidth="38640" windowHeight="21120" firstSheet="1" activeTab="2" xr2:uid="{21C51102-B905-44E2-89DF-C1A7E31F8D9F}"/>
   </bookViews>
@@ -4798,13 +4798,16 @@
         <v>3200.7518811800001</v>
       </c>
       <c r="I49" s="3">
-        <v>131.85821703200003</v>
+        <v>20</v>
       </c>
       <c r="J49" s="4">
         <v>1.9778732554800003</v>
       </c>
       <c r="K49">
         <v>40</v>
+      </c>
+      <c r="M49" s="3">
+        <v>131.85821703200003</v>
       </c>
       <c r="O49" t="s">
         <v>69</v>
@@ -4851,13 +4854,16 @@
         <v>3200.7518811800001</v>
       </c>
       <c r="I50" s="3">
-        <v>131.85821703200003</v>
+        <v>20</v>
       </c>
       <c r="J50" s="4">
         <v>1.9778732554800003</v>
       </c>
       <c r="K50">
         <v>40</v>
+      </c>
+      <c r="M50" s="3">
+        <v>131.85821703200003</v>
       </c>
       <c r="O50" t="s">
         <v>69</v>
@@ -4904,13 +4910,16 @@
         <v>3200.7518811800001</v>
       </c>
       <c r="I51" s="3">
-        <v>131.85821703200003</v>
+        <v>20</v>
       </c>
       <c r="J51" s="4">
         <v>1.9778732554800003</v>
       </c>
       <c r="K51">
         <v>40</v>
+      </c>
+      <c r="M51" s="3">
+        <v>131.85821703200003</v>
       </c>
       <c r="O51" t="s">
         <v>69</v>
@@ -4957,13 +4966,16 @@
         <v>3200.7518811800001</v>
       </c>
       <c r="I52" s="3">
-        <v>131.85821703200003</v>
+        <v>20</v>
       </c>
       <c r="J52" s="4">
         <v>1.9778732554800003</v>
       </c>
       <c r="K52">
         <v>40</v>
+      </c>
+      <c r="M52" s="3">
+        <v>131.85821703200003</v>
       </c>
       <c r="O52" t="s">
         <v>69</v>

</xml_diff>

<commit_message>
Iru is bio not gas
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/vt_EST_ELC_v1.xlsx
+++ b/VerveStacks_EST/vt_EST_ELC_v1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9849CC3-C1F1-4279-9AD0-5DA029C188B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92EA16F8-C75C-4769-AB37-A4A5C4D309AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="-5220" windowWidth="38640" windowHeight="21120" firstSheet="1" activeTab="2" xr2:uid="{21C51102-B905-44E2-89DF-C1A7E31F8D9F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="2" xr2:uid="{21C51102-B905-44E2-89DF-C1A7E31F8D9F}"/>
   </bookViews>
   <sheets>
     <sheet name="ccs_retrofits" sheetId="4" state="hidden" r:id="rId1"/>
@@ -148,7 +148,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="911" uniqueCount="219">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="911" uniqueCount="220">
   <si>
     <t>~fi_t</t>
   </si>
@@ -805,6 +805,9 @@
   </si>
   <si>
     <t>Aggregated Plant of windon except sopi plants</t>
+  </si>
+  <si>
+    <t>ep_bioenergy_iru</t>
   </si>
 </sst>
 </file>
@@ -3497,7 +3500,7 @@
         <v>69</v>
       </c>
       <c r="U23" t="s">
-        <v>17</v>
+        <v>219</v>
       </c>
       <c r="V23" t="s">
         <v>76</v>
@@ -3819,7 +3822,7 @@
     </row>
     <row r="30" spans="2:26" x14ac:dyDescent="0.25">
       <c r="B30" t="s">
-        <v>17</v>
+        <v>219</v>
       </c>
       <c r="C30" t="s">
         <v>13</v>

</xml_diff>

<commit_message>
Giving ncap_af to all exisitng plants
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/vt_EST_ELC_v1.xlsx
+++ b/VerveStacks_EST/vt_EST_ELC_v1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B26F173-5A6A-4989-8ECA-E54C352AAEF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAE08A75-8877-4E2D-8649-BCD8DF2547BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="2" xr2:uid="{21C51102-B905-44E2-89DF-C1A7E31F8D9F}"/>
+    <workbookView xWindow="-38520" yWindow="-5220" windowWidth="38640" windowHeight="21120" firstSheet="1" activeTab="2" xr2:uid="{21C51102-B905-44E2-89DF-C1A7E31F8D9F}"/>
   </bookViews>
   <sheets>
     <sheet name="ccs_retrofits" sheetId="4" state="hidden" r:id="rId1"/>
@@ -77,7 +77,7 @@
     <author>tc={3057E3B1-7BF3-4718-B31B-0585028D4313}</author>
   </authors>
   <commentList>
-    <comment ref="Y23" authorId="0" shapeId="0" xr:uid="{D3B26940-5207-4925-84BA-C36AB3766D74}">
+    <comment ref="Z23" authorId="0" shapeId="0" xr:uid="{D3B26940-5207-4925-84BA-C36AB3766D74}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -110,7 +110,7 @@
 </t>
       </text>
     </comment>
-    <comment ref="N43" authorId="4" shapeId="0" xr:uid="{C9FF73F0-A53F-4E15-A8C5-00DAE5061F13}">
+    <comment ref="O43" authorId="4" shapeId="0" xr:uid="{C9FF73F0-A53F-4E15-A8C5-00DAE5061F13}">
       <text>
         <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -119,7 +119,7 @@
 </t>
       </text>
     </comment>
-    <comment ref="Q47" authorId="5" shapeId="0" xr:uid="{C2CA05C3-E9FD-442F-962C-5D4E7F1ADE70}">
+    <comment ref="R47" authorId="5" shapeId="0" xr:uid="{C2CA05C3-E9FD-442F-962C-5D4E7F1ADE70}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -127,7 +127,7 @@
     Took same as chp</t>
       </text>
     </comment>
-    <comment ref="T84" authorId="6" shapeId="0" xr:uid="{1905391B-2A5F-4643-B2AC-720AD8410CDA}">
+    <comment ref="U84" authorId="6" shapeId="0" xr:uid="{1905391B-2A5F-4643-B2AC-720AD8410CDA}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -148,7 +148,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="911" uniqueCount="220">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="911" uniqueCount="221">
   <si>
     <t>~fi_t</t>
   </si>
@@ -808,6 +808,9 @@
   </si>
   <si>
     <t>ep_bioenergy_iru</t>
+  </si>
+  <si>
+    <t>ncap_af</t>
   </si>
 </sst>
 </file>
@@ -1211,7 +1214,7 @@
 
 <file path=xl/threadedComments/threadedComment2.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="Y23" dT="2026-03-05T12:47:49.66" personId="{9CD26280-DD25-46DF-A708-6877D8A68AD8}" id="{D3B26940-5207-4925-84BA-C36AB3766D74}">
+  <threadedComment ref="Z23" dT="2026-03-05T12:47:49.66" personId="{9CD26280-DD25-46DF-A708-6877D8A68AD8}" id="{D3B26940-5207-4925-84BA-C36AB3766D74}">
     <text>Miks daynite (hydro samuti)</text>
   </threadedComment>
   <threadedComment ref="F30" dT="2026-01-22T14:00:05.64" personId="{9CD26280-DD25-46DF-A708-6877D8A68AD8}" id="{E45DD652-654C-4828-8A13-679EDDC53E65}">
@@ -1224,14 +1227,14 @@
     <text xml:space="preserve">Ei tea
 </text>
   </threadedComment>
-  <threadedComment ref="N43" dT="2026-03-05T12:22:32.07" personId="{9CD26280-DD25-46DF-A708-6877D8A68AD8}" id="{C9FF73F0-A53F-4E15-A8C5-00DAE5061F13}">
+  <threadedComment ref="O43" dT="2026-03-05T12:22:32.07" personId="{9CD26280-DD25-46DF-A708-6877D8A68AD8}" id="{C9FF73F0-A53F-4E15-A8C5-00DAE5061F13}">
     <text xml:space="preserve">NCAP_FOM (currency/GW-yr)=100/1.31​×NCAP_COST (currency/GW)
 </text>
   </threadedComment>
-  <threadedComment ref="Q47" dT="2026-03-05T12:58:31.38" personId="{9CD26280-DD25-46DF-A708-6877D8A68AD8}" id="{C2CA05C3-E9FD-442F-962C-5D4E7F1ADE70}">
+  <threadedComment ref="R47" dT="2026-03-05T12:58:31.38" personId="{9CD26280-DD25-46DF-A708-6877D8A68AD8}" id="{C2CA05C3-E9FD-442F-962C-5D4E7F1ADE70}">
     <text>Took same as chp</text>
   </threadedComment>
-  <threadedComment ref="T84" dT="2026-01-28T08:41:02.80" personId="{9CD26280-DD25-46DF-A708-6877D8A68AD8}" id="{1905391B-2A5F-4643-B2AC-720AD8410CDA}">
+  <threadedComment ref="U84" dT="2026-01-28T08:41:02.80" personId="{9CD26280-DD25-46DF-A708-6877D8A68AD8}" id="{1905391B-2A5F-4643-B2AC-720AD8410CDA}">
     <text>Frequency reserve</text>
   </threadedComment>
   <threadedComment ref="J85" dT="2026-01-27T14:26:51.36" personId="{9CD26280-DD25-46DF-A708-6877D8A68AD8}" id="{3057E3B1-7BF3-4718-B31B-0585028D4313}">
@@ -2725,7 +2728,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A79DDA4A-BC9F-4D47-BDC9-53442001A438}">
-  <dimension ref="B9:Z105"/>
+  <dimension ref="B9:AA105"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="40.5703125" bestFit="1" customWidth="1"/>
@@ -2738,25 +2741,26 @@
     <col min="9" max="9" width="9.85546875" style="3" bestFit="1" customWidth="1"/>
     <col min="10" max="11" width="9.28515625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="12" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="17.28515625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="12" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="40.5703125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="64.42578125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="41.42578125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="64.42578125" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="41.42578125" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="64.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12" customWidth="1"/>
+    <col min="14" max="14" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="40.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="64.42578125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="41.42578125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="64.42578125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="41.42578125" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="64.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="9" spans="2:26" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>0</v>
       </c>
-      <c r="T9" t="s">
+      <c r="U9" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="10" spans="2:26" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>1</v>
       </c>
@@ -2788,31 +2792,31 @@
         <v>10</v>
       </c>
       <c r="L10" t="s">
-        <v>11</v>
-      </c>
-      <c r="T10" t="s">
+        <v>220</v>
+      </c>
+      <c r="U10" t="s">
         <v>63</v>
       </c>
-      <c r="U10" t="s">
+      <c r="V10" t="s">
         <v>1</v>
       </c>
-      <c r="V10" t="s">
+      <c r="W10" t="s">
         <v>64</v>
       </c>
-      <c r="W10" t="s">
+      <c r="X10" t="s">
         <v>65</v>
       </c>
-      <c r="X10" t="s">
+      <c r="Y10" t="s">
         <v>66</v>
       </c>
-      <c r="Y10" t="s">
+      <c r="Z10" t="s">
         <v>67</v>
       </c>
-      <c r="Z10" t="s">
+      <c r="AA10" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="11" spans="2:26" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
         <v>22</v>
       </c>
@@ -2834,29 +2838,29 @@
       <c r="L11">
         <v>0.14986856628506873</v>
       </c>
-      <c r="T11" t="s">
-        <v>69</v>
-      </c>
       <c r="U11" t="s">
+        <v>69</v>
+      </c>
+      <c r="V11" t="s">
         <v>22</v>
       </c>
-      <c r="V11" t="s">
+      <c r="W11" t="s">
         <v>78</v>
       </c>
-      <c r="W11" t="s">
-        <v>71</v>
-      </c>
       <c r="X11" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="Y11" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="Z11" t="s">
+        <v>80</v>
+      </c>
+      <c r="AA11" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="12" spans="2:26" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
         <v>25</v>
       </c>
@@ -2878,29 +2882,29 @@
       <c r="L12">
         <v>0.14986856628506873</v>
       </c>
-      <c r="T12" t="s">
-        <v>69</v>
-      </c>
       <c r="U12" t="s">
+        <v>69</v>
+      </c>
+      <c r="V12" t="s">
         <v>25</v>
       </c>
-      <c r="V12" t="s">
+      <c r="W12" t="s">
         <v>78</v>
       </c>
-      <c r="W12" t="s">
-        <v>71</v>
-      </c>
       <c r="X12" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="Y12" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="Z12" t="s">
+        <v>80</v>
+      </c>
+      <c r="AA12" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="13" spans="2:26" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
         <v>27</v>
       </c>
@@ -2922,29 +2926,29 @@
       <c r="L13">
         <v>0.14986856628506873</v>
       </c>
-      <c r="T13" t="s">
-        <v>69</v>
-      </c>
       <c r="U13" t="s">
+        <v>69</v>
+      </c>
+      <c r="V13" t="s">
         <v>27</v>
       </c>
-      <c r="V13" t="s">
+      <c r="W13" t="s">
         <v>78</v>
       </c>
-      <c r="W13" t="s">
-        <v>71</v>
-      </c>
       <c r="X13" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="Y13" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="Z13" t="s">
+        <v>80</v>
+      </c>
+      <c r="AA13" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="14" spans="2:26" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
         <v>29</v>
       </c>
@@ -2978,29 +2982,29 @@
       <c r="L14">
         <v>0.1461854238754417</v>
       </c>
-      <c r="T14" t="s">
-        <v>69</v>
-      </c>
       <c r="U14" t="s">
+        <v>69</v>
+      </c>
+      <c r="V14" t="s">
         <v>29</v>
       </c>
-      <c r="V14" t="s">
+      <c r="W14" t="s">
         <v>78</v>
       </c>
-      <c r="W14" t="s">
-        <v>71</v>
-      </c>
       <c r="X14" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="Y14" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="Z14" t="s">
+        <v>80</v>
+      </c>
+      <c r="AA14" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="15" spans="2:26" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
         <v>29</v>
       </c>
@@ -3034,29 +3038,29 @@
       <c r="L15">
         <v>0.1461854238754417</v>
       </c>
-      <c r="T15" t="s">
-        <v>69</v>
-      </c>
       <c r="U15" t="s">
+        <v>69</v>
+      </c>
+      <c r="V15" t="s">
         <v>30</v>
       </c>
-      <c r="V15" t="s">
+      <c r="W15" t="s">
         <v>78</v>
       </c>
-      <c r="W15" t="s">
-        <v>71</v>
-      </c>
       <c r="X15" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="Y15" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="Z15" t="s">
+        <v>80</v>
+      </c>
+      <c r="AA15" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="16" spans="2:26" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
         <v>30</v>
       </c>
@@ -3090,29 +3094,29 @@
       <c r="L16">
         <v>0.14867925344692126</v>
       </c>
-      <c r="T16" t="s">
-        <v>69</v>
-      </c>
       <c r="U16" t="s">
+        <v>69</v>
+      </c>
+      <c r="V16" t="s">
         <v>32</v>
       </c>
-      <c r="V16" t="s">
+      <c r="W16" t="s">
         <v>78</v>
       </c>
-      <c r="W16" t="s">
-        <v>71</v>
-      </c>
       <c r="X16" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="Y16" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="Z16" t="s">
+        <v>80</v>
+      </c>
+      <c r="AA16" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="17" spans="2:26" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
         <v>32</v>
       </c>
@@ -3146,29 +3150,29 @@
       <c r="L17">
         <v>0.14701259708091721</v>
       </c>
-      <c r="T17" t="s">
-        <v>69</v>
-      </c>
       <c r="U17" t="s">
+        <v>69</v>
+      </c>
+      <c r="V17" t="s">
         <v>34</v>
       </c>
-      <c r="V17" t="s">
+      <c r="W17" t="s">
         <v>78</v>
       </c>
-      <c r="W17" t="s">
-        <v>71</v>
-      </c>
       <c r="X17" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="Y17" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="Z17" t="s">
+        <v>80</v>
+      </c>
+      <c r="AA17" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="18" spans="2:26" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
         <v>34</v>
       </c>
@@ -3202,35 +3206,35 @@
       <c r="L18">
         <v>0.15309859852159369</v>
       </c>
-      <c r="O18">
+      <c r="P18">
         <v>3.9363662143155967E-2</v>
       </c>
-      <c r="P18">
+      <c r="Q18">
         <v>0.28763633785684395</v>
       </c>
-      <c r="T18" t="s">
-        <v>69</v>
-      </c>
       <c r="U18" t="s">
+        <v>69</v>
+      </c>
+      <c r="V18" t="s">
         <v>35</v>
       </c>
-      <c r="V18" t="s">
+      <c r="W18" t="s">
         <v>78</v>
       </c>
-      <c r="W18" t="s">
-        <v>71</v>
-      </c>
       <c r="X18" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="Y18" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="Z18" t="s">
+        <v>80</v>
+      </c>
+      <c r="AA18" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="19" spans="2:26" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
         <v>34</v>
       </c>
@@ -3264,29 +3268,29 @@
       <c r="L19">
         <v>0.15309859852159369</v>
       </c>
-      <c r="T19" t="s">
-        <v>69</v>
-      </c>
       <c r="U19" t="s">
+        <v>69</v>
+      </c>
+      <c r="V19" t="s">
         <v>37</v>
       </c>
-      <c r="V19" t="s">
+      <c r="W19" t="s">
         <v>78</v>
       </c>
-      <c r="W19" t="s">
-        <v>71</v>
-      </c>
       <c r="X19" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="Y19" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="Z19" t="s">
+        <v>80</v>
+      </c>
+      <c r="AA19" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="20" spans="2:26" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B20" t="s">
         <v>35</v>
       </c>
@@ -3320,37 +3324,37 @@
       <c r="L20">
         <v>0.15619560585976827</v>
       </c>
-      <c r="O20">
+      <c r="P20">
         <f>SUM(F11:F25)</f>
         <v>0.92963633785684396</v>
       </c>
-      <c r="P20">
-        <f>0.969-F13-O20</f>
+      <c r="Q20">
+        <f>0.969-F13-P20</f>
         <v>-0.28763633785684384</v>
       </c>
-      <c r="T20" t="s">
-        <v>69</v>
-      </c>
       <c r="U20" t="s">
+        <v>69</v>
+      </c>
+      <c r="V20" t="s">
         <v>39</v>
       </c>
-      <c r="V20" t="s">
+      <c r="W20" t="s">
         <v>78</v>
       </c>
-      <c r="W20" t="s">
-        <v>71</v>
-      </c>
       <c r="X20" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="Y20" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="Z20" t="s">
+        <v>80</v>
+      </c>
+      <c r="AA20" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="21" spans="2:26" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B21" t="s">
         <v>37</v>
       </c>
@@ -3384,29 +3388,29 @@
       <c r="L21">
         <v>0.14537310453496291</v>
       </c>
-      <c r="T21" t="s">
-        <v>69</v>
-      </c>
       <c r="U21" t="s">
+        <v>69</v>
+      </c>
+      <c r="V21" t="s">
         <v>40</v>
       </c>
-      <c r="V21" t="s">
+      <c r="W21" t="s">
         <v>78</v>
       </c>
-      <c r="W21" t="s">
-        <v>71</v>
-      </c>
       <c r="X21" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="Y21" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="Z21" t="s">
+        <v>80</v>
+      </c>
+      <c r="AA21" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="22" spans="2:26" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B22" t="s">
         <v>39</v>
       </c>
@@ -3440,29 +3444,29 @@
       <c r="L22">
         <v>0.14763873655681015</v>
       </c>
-      <c r="T22" t="s">
-        <v>69</v>
-      </c>
       <c r="U22" t="s">
+        <v>69</v>
+      </c>
+      <c r="V22" t="s">
         <v>42</v>
       </c>
-      <c r="V22" t="s">
+      <c r="W22" t="s">
         <v>78</v>
       </c>
-      <c r="W22" t="s">
-        <v>71</v>
-      </c>
       <c r="X22" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="Y22" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="Z22" t="s">
+        <v>80</v>
+      </c>
+      <c r="AA22" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="23" spans="2:26" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B23" t="s">
         <v>40</v>
       </c>
@@ -3496,29 +3500,29 @@
       <c r="L23">
         <v>0.1532628310027955</v>
       </c>
-      <c r="T23" t="s">
-        <v>69</v>
-      </c>
       <c r="U23" t="s">
+        <v>69</v>
+      </c>
+      <c r="V23" t="s">
         <v>219</v>
       </c>
-      <c r="V23" t="s">
+      <c r="W23" t="s">
         <v>76</v>
       </c>
-      <c r="W23" t="s">
-        <v>71</v>
-      </c>
       <c r="X23" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="Y23" t="s">
+        <v>72</v>
+      </c>
+      <c r="Z23" t="s">
         <v>73</v>
       </c>
-      <c r="Z23" t="s">
+      <c r="AA23" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="24" spans="2:26" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B24" t="s">
         <v>40</v>
       </c>
@@ -3552,33 +3556,33 @@
       <c r="L24">
         <v>0.1532628310027955</v>
       </c>
-      <c r="P24">
-        <f>SUM(O20:P20)+F13</f>
+      <c r="Q24">
+        <f>SUM(P20:Q20)+F13</f>
         <v>0.96900000000000008</v>
       </c>
-      <c r="T24" t="s">
-        <v>69</v>
-      </c>
       <c r="U24" t="s">
+        <v>69</v>
+      </c>
+      <c r="V24" t="s">
         <v>61</v>
       </c>
-      <c r="V24" t="s">
+      <c r="W24" t="s">
         <v>81</v>
       </c>
-      <c r="W24" t="s">
-        <v>71</v>
-      </c>
       <c r="X24" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="Y24" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="Z24" t="s">
+        <v>80</v>
+      </c>
+      <c r="AA24" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="25" spans="2:26" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B25" t="s">
         <v>42</v>
       </c>
@@ -3612,29 +3616,29 @@
       <c r="L25">
         <v>0.1451997589052581</v>
       </c>
-      <c r="T25" t="s">
-        <v>69</v>
-      </c>
       <c r="U25" t="s">
+        <v>69</v>
+      </c>
+      <c r="V25" t="s">
         <v>216</v>
       </c>
-      <c r="V25" t="s">
+      <c r="W25" t="s">
         <v>81</v>
       </c>
-      <c r="W25" t="s">
-        <v>71</v>
-      </c>
       <c r="X25" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="Y25" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="Z25" t="s">
+        <v>80</v>
+      </c>
+      <c r="AA25" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="26" spans="2:26" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B26" t="s">
         <v>61</v>
       </c>
@@ -3668,29 +3672,29 @@
       <c r="L26">
         <v>0.365520596150406</v>
       </c>
-      <c r="T26" t="s">
-        <v>69</v>
-      </c>
       <c r="U26" t="s">
+        <v>69</v>
+      </c>
+      <c r="V26" t="s">
         <v>217</v>
       </c>
-      <c r="V26" t="s">
+      <c r="W26" t="s">
         <v>218</v>
       </c>
-      <c r="W26" t="s">
-        <v>71</v>
-      </c>
       <c r="X26" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="Y26" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="Z26" t="s">
+        <v>80</v>
+      </c>
+      <c r="AA26" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="27" spans="2:26" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B27" t="s">
         <v>216</v>
       </c>
@@ -3724,18 +3728,18 @@
       <c r="L27">
         <v>0.365520596150406</v>
       </c>
-      <c r="M27">
+      <c r="N27">
         <f>F90*L90*G90</f>
         <v>2.0930123559331545E-3</v>
       </c>
-      <c r="T27" t="s">
+      <c r="U27" t="s">
         <v>140</v>
       </c>
-      <c r="U27" s="1" t="s">
+      <c r="V27" s="1" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="28" spans="2:26" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B28" t="s">
         <v>217</v>
       </c>
@@ -3769,58 +3773,58 @@
       <c r="L28">
         <v>0.41047488326249421</v>
       </c>
-      <c r="T28" t="s">
-        <v>69</v>
-      </c>
       <c r="U28" t="s">
+        <v>69</v>
+      </c>
+      <c r="V28" t="s">
         <v>194</v>
       </c>
-      <c r="V28" t="s">
+      <c r="W28" t="s">
         <v>163</v>
       </c>
-      <c r="W28" t="s">
-        <v>71</v>
-      </c>
       <c r="X28" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="Y28" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="Z28" t="s">
+        <v>80</v>
+      </c>
+      <c r="AA28" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="29" spans="2:26" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B29" t="s">
         <v>140</v>
       </c>
       <c r="C29" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="T29" t="s">
-        <v>69</v>
-      </c>
       <c r="U29" t="s">
+        <v>69</v>
+      </c>
+      <c r="V29" t="s">
         <v>193</v>
       </c>
-      <c r="V29" t="s">
+      <c r="W29" t="s">
         <v>148</v>
       </c>
-      <c r="W29" t="s">
-        <v>71</v>
-      </c>
       <c r="X29" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="Y29" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="Z29" t="s">
+        <v>80</v>
+      </c>
+      <c r="AA29" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="30" spans="2:26" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B30" t="s">
         <v>219</v>
       </c>
@@ -3837,46 +3841,49 @@
         <v>1.7000000000000001E-2</v>
       </c>
       <c r="G30">
-        <f>P45</f>
+        <f>Q45</f>
         <v>0.56000000000000005</v>
       </c>
       <c r="H30" s="2">
         <v>1175.5066999999999</v>
       </c>
       <c r="I30" s="3">
-        <f>(N45/100)*H31</f>
+        <f>(O45/100)*H31</f>
         <v>160.216352398</v>
       </c>
       <c r="J30">
-        <f>Q45</f>
+        <f>R45</f>
         <v>5.8775000000000004</v>
       </c>
       <c r="K30">
         <v>53</v>
       </c>
-      <c r="T30" t="s">
-        <v>69</v>
+      <c r="L30">
+        <v>0.8</v>
       </c>
       <c r="U30" t="s">
+        <v>69</v>
+      </c>
+      <c r="V30" t="s">
         <v>195</v>
       </c>
-      <c r="V30" t="s">
+      <c r="W30" t="s">
         <v>149</v>
       </c>
-      <c r="W30" t="s">
-        <v>71</v>
-      </c>
       <c r="X30" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="Y30" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="Z30" t="s">
+        <v>80</v>
+      </c>
+      <c r="AA30" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="31" spans="2:26" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B31" t="s">
         <v>196</v>
       </c>
@@ -3893,7 +3900,7 @@
         <v>0.77</v>
       </c>
       <c r="G31">
-        <f>$P$44</f>
+        <f>$Q$44</f>
         <v>0.33</v>
       </c>
       <c r="H31" s="2">
@@ -3904,35 +3911,38 @@
         <v>63.037519640000006</v>
       </c>
       <c r="J31">
-        <f>$Q$44</f>
+        <f>$R$44</f>
         <v>4.1005000000000003</v>
       </c>
       <c r="K31">
         <v>70</v>
       </c>
-      <c r="T31" t="s">
-        <v>69</v>
+      <c r="L31">
+        <v>0.8</v>
       </c>
       <c r="U31" t="s">
+        <v>69</v>
+      </c>
+      <c r="V31" t="s">
         <v>196</v>
       </c>
-      <c r="V31" t="s">
+      <c r="W31" t="s">
         <v>150</v>
       </c>
-      <c r="W31" t="s">
-        <v>71</v>
-      </c>
       <c r="X31" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="Y31" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="Z31" t="s">
+        <v>80</v>
+      </c>
+      <c r="AA31" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="32" spans="2:26" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B32" t="s">
         <v>194</v>
       </c>
@@ -3949,7 +3959,7 @@
         <v>0.26</v>
       </c>
       <c r="G32">
-        <f t="shared" ref="G32:G34" si="0">$P$44</f>
+        <f t="shared" ref="G32:G34" si="0">$Q$44</f>
         <v>0.33</v>
       </c>
       <c r="H32" s="2">
@@ -3960,35 +3970,38 @@
         <v>63.037519640000006</v>
       </c>
       <c r="J32">
-        <f t="shared" ref="J32:J48" si="1">$Q$44</f>
+        <f t="shared" ref="J32:J48" si="1">$R$44</f>
         <v>4.1005000000000003</v>
       </c>
       <c r="K32">
         <v>40</v>
       </c>
-      <c r="T32" t="s">
-        <v>69</v>
+      <c r="L32">
+        <v>0.7</v>
       </c>
       <c r="U32" t="s">
+        <v>69</v>
+      </c>
+      <c r="V32" t="s">
         <v>142</v>
       </c>
-      <c r="V32" t="s">
+      <c r="W32" t="s">
         <v>161</v>
       </c>
-      <c r="W32" t="s">
-        <v>71</v>
-      </c>
       <c r="X32" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="Y32" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="Z32" t="s">
+        <v>80</v>
+      </c>
+      <c r="AA32" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="33" spans="2:26" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B33" t="s">
         <v>195</v>
       </c>
@@ -4016,35 +4029,38 @@
         <v>63.037519640000006</v>
       </c>
       <c r="J33">
-        <f>$Q$44</f>
+        <f>$R$44</f>
         <v>4.1005000000000003</v>
       </c>
       <c r="K33">
         <v>40</v>
       </c>
-      <c r="T33" t="s">
-        <v>69</v>
+      <c r="L33">
+        <v>0.8</v>
       </c>
       <c r="U33" t="s">
+        <v>69</v>
+      </c>
+      <c r="V33" t="s">
         <v>143</v>
       </c>
-      <c r="V33" t="s">
+      <c r="W33" t="s">
         <v>151</v>
       </c>
-      <c r="W33" t="s">
-        <v>71</v>
-      </c>
       <c r="X33" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="Y33" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="Z33" t="s">
+        <v>80</v>
+      </c>
+      <c r="AA33" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="34" spans="2:26" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B34" t="s">
         <v>193</v>
       </c>
@@ -4078,29 +4094,32 @@
       <c r="K34">
         <v>73</v>
       </c>
-      <c r="T34" t="s">
-        <v>69</v>
+      <c r="L34">
+        <v>0.8</v>
       </c>
       <c r="U34" t="s">
+        <v>69</v>
+      </c>
+      <c r="V34" t="s">
         <v>144</v>
       </c>
-      <c r="V34" t="s">
+      <c r="W34" t="s">
         <v>152</v>
       </c>
-      <c r="W34" t="s">
-        <v>71</v>
-      </c>
       <c r="X34" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="Y34" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="Z34" t="s">
+        <v>80</v>
+      </c>
+      <c r="AA34" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="35" spans="2:26" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B35" t="s">
         <v>142</v>
       </c>
@@ -4117,47 +4136,50 @@
         <v>7.6999999999999999E-2</v>
       </c>
       <c r="G35">
+        <f>Q45</f>
+        <v>0.56000000000000005</v>
+      </c>
+      <c r="H35" s="2">
         <f>P45</f>
-        <v>0.56000000000000005</v>
-      </c>
-      <c r="H35" s="2">
-        <f>O45</f>
         <v>1175.5066999999999</v>
       </c>
       <c r="I35" s="3">
-        <f>(N45/100)*H35</f>
+        <f>(O45/100)*H35</f>
         <v>39.138495576499992</v>
       </c>
       <c r="J35">
-        <f>$Q$45</f>
+        <f>$R$45</f>
         <v>5.8775000000000004</v>
       </c>
       <c r="K35">
         <v>40</v>
       </c>
-      <c r="T35" t="s">
-        <v>69</v>
+      <c r="L35">
+        <v>0.8</v>
       </c>
       <c r="U35" t="s">
+        <v>69</v>
+      </c>
+      <c r="V35" t="s">
         <v>145</v>
       </c>
-      <c r="V35" t="s">
+      <c r="W35" t="s">
         <v>153</v>
       </c>
-      <c r="W35" t="s">
-        <v>71</v>
-      </c>
       <c r="X35" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="Y35" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="Z35" t="s">
+        <v>80</v>
+      </c>
+      <c r="AA35" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="36" spans="2:26" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B36" t="s">
         <v>143</v>
       </c>
@@ -4174,11 +4196,11 @@
         <v>3.9E-2</v>
       </c>
       <c r="G36">
-        <f>P47</f>
+        <f>Q47</f>
         <v>0.46800000000000003</v>
       </c>
       <c r="H36" s="2">
-        <f>$O$47</f>
+        <f>$P$47</f>
         <v>2950.7891</v>
       </c>
       <c r="I36" s="3">
@@ -4186,35 +4208,38 @@
         <v>133.5792717679</v>
       </c>
       <c r="J36">
-        <f>$Q$47</f>
+        <f>$R$47</f>
         <v>2.8138000000000001</v>
       </c>
       <c r="K36">
         <v>40</v>
       </c>
-      <c r="T36" t="s">
-        <v>69</v>
+      <c r="L36">
+        <v>0.8</v>
       </c>
       <c r="U36" t="s">
+        <v>69</v>
+      </c>
+      <c r="V36" t="s">
         <v>146</v>
       </c>
-      <c r="V36" t="s">
+      <c r="W36" t="s">
         <v>147</v>
       </c>
-      <c r="W36" t="s">
-        <v>71</v>
-      </c>
       <c r="X36" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="Y36" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="Z36" t="s">
+        <v>80</v>
+      </c>
+      <c r="AA36" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="37" spans="2:26" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B37" t="s">
         <v>144</v>
       </c>
@@ -4234,7 +4259,7 @@
         <v>0.46800000000000003</v>
       </c>
       <c r="H37" s="2">
-        <f t="shared" ref="H37:H39" si="2">$O$47</f>
+        <f t="shared" ref="H37:H39" si="2">$P$47</f>
         <v>2950.7891</v>
       </c>
       <c r="I37" s="3">
@@ -4242,35 +4267,38 @@
         <v>133.5792717679</v>
       </c>
       <c r="J37">
-        <f t="shared" ref="J37:J39" si="4">$Q$47</f>
+        <f t="shared" ref="J37:J39" si="4">$R$47</f>
         <v>2.8138000000000001</v>
       </c>
       <c r="K37">
         <v>40</v>
       </c>
-      <c r="T37" t="s">
-        <v>69</v>
+      <c r="L37">
+        <v>0.8</v>
       </c>
       <c r="U37" t="s">
+        <v>69</v>
+      </c>
+      <c r="V37" t="s">
         <v>197</v>
       </c>
-      <c r="V37" t="s">
+      <c r="W37" t="s">
         <v>162</v>
       </c>
-      <c r="W37" t="s">
-        <v>71</v>
-      </c>
       <c r="X37" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="Y37" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="Z37" t="s">
+        <v>80</v>
+      </c>
+      <c r="AA37" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="38" spans="2:26" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B38" t="s">
         <v>145</v>
       </c>
@@ -4304,29 +4332,32 @@
       <c r="K38">
         <v>40</v>
       </c>
-      <c r="T38" t="s">
-        <v>69</v>
+      <c r="L38">
+        <v>0.8</v>
       </c>
       <c r="U38" t="s">
+        <v>69</v>
+      </c>
+      <c r="V38" t="s">
         <v>154</v>
       </c>
-      <c r="V38" t="s">
+      <c r="W38" t="s">
         <v>155</v>
       </c>
-      <c r="W38" t="s">
-        <v>71</v>
-      </c>
       <c r="X38" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="Y38" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="Z38" t="s">
+        <v>80</v>
+      </c>
+      <c r="AA38" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="39" spans="2:26" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B39" t="s">
         <v>146</v>
       </c>
@@ -4360,29 +4391,32 @@
       <c r="K39">
         <v>40</v>
       </c>
-      <c r="T39" t="s">
-        <v>69</v>
+      <c r="L39">
+        <v>0.8</v>
       </c>
       <c r="U39" t="s">
+        <v>69</v>
+      </c>
+      <c r="V39" t="s">
         <v>156</v>
       </c>
-      <c r="V39" t="s">
+      <c r="W39" t="s">
         <v>157</v>
       </c>
-      <c r="W39" t="s">
-        <v>71</v>
-      </c>
       <c r="X39" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="Y39" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="Z39" t="s">
+        <v>80</v>
+      </c>
+      <c r="AA39" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="40" spans="2:26" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B40" t="s">
         <v>197</v>
       </c>
@@ -4399,47 +4433,50 @@
         <v>0.01</v>
       </c>
       <c r="G40">
+        <f>Q44</f>
+        <v>0.33</v>
+      </c>
+      <c r="H40" s="2">
         <f>P44</f>
-        <v>0.33</v>
-      </c>
-      <c r="H40" s="2">
-        <f>O44</f>
         <v>4812.0244000000002</v>
       </c>
       <c r="I40" s="3">
-        <f>($N$44/100)*H40</f>
+        <f>($O$44/100)*H40</f>
         <v>63.037519640000006</v>
       </c>
       <c r="J40">
-        <f>$Q$44</f>
+        <f>$R$44</f>
         <v>4.1005000000000003</v>
       </c>
       <c r="K40">
         <v>40</v>
       </c>
-      <c r="T40" t="s">
-        <v>69</v>
+      <c r="L40">
+        <v>0.8</v>
       </c>
       <c r="U40" t="s">
+        <v>69</v>
+      </c>
+      <c r="V40" t="s">
         <v>170</v>
       </c>
-      <c r="V40" t="s">
+      <c r="W40" t="s">
         <v>171</v>
       </c>
-      <c r="W40" t="s">
-        <v>71</v>
-      </c>
       <c r="X40" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="Y40" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="Z40" t="s">
+        <v>80</v>
+      </c>
+      <c r="AA40" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="41" spans="2:26" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B41" t="s">
         <v>154</v>
       </c>
@@ -4459,43 +4496,46 @@
         <v>0.28999999999999998</v>
       </c>
       <c r="H41" s="2">
-        <f>$O$48</f>
+        <f>$P$48</f>
         <v>4516.7133000000003</v>
       </c>
       <c r="I41" s="3">
-        <f>($N$48/100)*H41</f>
+        <f>($O$48/100)*H41</f>
         <v>162.96753257730003</v>
       </c>
       <c r="J41">
-        <f>$Q$48</f>
+        <f>$R$48</f>
         <v>2.8138000000000001</v>
       </c>
       <c r="K41">
         <v>40</v>
       </c>
-      <c r="T41" t="s">
-        <v>69</v>
+      <c r="L41">
+        <v>0.8</v>
       </c>
       <c r="U41" t="s">
+        <v>69</v>
+      </c>
+      <c r="V41" t="s">
         <v>158</v>
       </c>
-      <c r="V41" t="s">
+      <c r="W41" t="s">
         <v>159</v>
       </c>
-      <c r="W41" t="s">
-        <v>71</v>
-      </c>
       <c r="X41" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="Y41" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="Z41" t="s">
+        <v>80</v>
+      </c>
+      <c r="AA41" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="42" spans="2:26" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B42" t="s">
         <v>156</v>
       </c>
@@ -4515,43 +4555,46 @@
         <v>0.28999999999999998</v>
       </c>
       <c r="H42" s="2">
-        <f t="shared" ref="H42:H44" si="5">$O$48</f>
+        <f t="shared" ref="H42:H44" si="5">$P$48</f>
         <v>4516.7133000000003</v>
       </c>
       <c r="I42" s="3">
-        <f t="shared" ref="I42:I44" si="6">($N$48/100)*H42</f>
+        <f t="shared" ref="I42:I44" si="6">($O$48/100)*H42</f>
         <v>162.96753257730003</v>
       </c>
       <c r="J42">
-        <f t="shared" ref="J42:J44" si="7">$Q$48</f>
+        <f t="shared" ref="J42:J44" si="7">$R$48</f>
         <v>2.8138000000000001</v>
       </c>
       <c r="K42">
         <v>40</v>
       </c>
-      <c r="T42" t="s">
-        <v>69</v>
+      <c r="L42">
+        <v>0.8</v>
       </c>
       <c r="U42" t="s">
+        <v>69</v>
+      </c>
+      <c r="V42" t="s">
         <v>169</v>
       </c>
-      <c r="V42" t="s">
+      <c r="W42" t="s">
         <v>160</v>
       </c>
-      <c r="W42" t="s">
-        <v>71</v>
-      </c>
       <c r="X42" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="Y42" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="Z42" t="s">
+        <v>80</v>
+      </c>
+      <c r="AA42" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="43" spans="2:26" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B43" t="s">
         <v>170</v>
       </c>
@@ -4585,41 +4628,44 @@
       <c r="K43">
         <v>40</v>
       </c>
-      <c r="N43" t="s">
+      <c r="L43">
+        <v>0.8</v>
+      </c>
+      <c r="O43" t="s">
         <v>206</v>
       </c>
-      <c r="O43" t="s">
+      <c r="P43" t="s">
         <v>213</v>
       </c>
-      <c r="P43" t="s">
+      <c r="Q43" t="s">
         <v>214</v>
       </c>
-      <c r="Q43" t="s">
+      <c r="R43" t="s">
         <v>215</v>
       </c>
-      <c r="T43" t="s">
-        <v>69</v>
-      </c>
       <c r="U43" t="s">
+        <v>69</v>
+      </c>
+      <c r="V43" t="s">
         <v>164</v>
       </c>
-      <c r="V43" t="s">
+      <c r="W43" t="s">
         <v>165</v>
       </c>
-      <c r="W43" t="s">
-        <v>71</v>
-      </c>
       <c r="X43" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="Y43" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="Z43" t="s">
+        <v>80</v>
+      </c>
+      <c r="AA43" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="44" spans="2:26" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B44" t="s">
         <v>158</v>
       </c>
@@ -4653,44 +4699,47 @@
       <c r="K44">
         <v>72</v>
       </c>
-      <c r="M44" t="s">
+      <c r="L44">
+        <v>0.8</v>
+      </c>
+      <c r="N44" t="s">
         <v>192</v>
       </c>
-      <c r="N44" s="4">
+      <c r="O44" s="4">
         <v>1.31</v>
       </c>
-      <c r="O44" s="2">
+      <c r="P44" s="2">
         <v>4812.0244000000002</v>
       </c>
-      <c r="P44">
+      <c r="Q44">
         <v>0.33</v>
       </c>
-      <c r="Q44">
+      <c r="R44">
         <v>4.1005000000000003</v>
       </c>
-      <c r="T44" t="s">
-        <v>69</v>
-      </c>
       <c r="U44" t="s">
+        <v>69</v>
+      </c>
+      <c r="V44" t="s">
         <v>168</v>
       </c>
-      <c r="V44" t="s">
+      <c r="W44" t="s">
         <v>166</v>
       </c>
-      <c r="W44" t="s">
-        <v>71</v>
-      </c>
       <c r="X44" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="Y44" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="Z44" t="s">
+        <v>80</v>
+      </c>
+      <c r="AA44" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="45" spans="2:26" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B45" t="s">
         <v>169</v>
       </c>
@@ -4707,62 +4756,65 @@
         <v>5.7999999999999996E-3</v>
       </c>
       <c r="G45">
+        <f>Q45</f>
+        <v>0.56000000000000005</v>
+      </c>
+      <c r="H45" s="2">
         <f>P45</f>
-        <v>0.56000000000000005</v>
-      </c>
-      <c r="H45" s="2">
-        <f>O45</f>
         <v>1175.5066999999999</v>
       </c>
       <c r="I45" s="3">
-        <f>($N$45/100)*H45</f>
+        <f>($O$45/100)*H45</f>
         <v>39.138495576499992</v>
       </c>
       <c r="J45">
-        <f>$Q$45</f>
+        <f>$R$45</f>
         <v>5.8775000000000004</v>
       </c>
       <c r="K45">
         <v>40</v>
       </c>
-      <c r="M45" t="s">
+      <c r="L45">
+        <v>0.8</v>
+      </c>
+      <c r="N45" t="s">
         <v>211</v>
       </c>
-      <c r="N45" s="4">
+      <c r="O45" s="4">
         <v>3.3294999999999999</v>
       </c>
-      <c r="O45" s="2">
+      <c r="P45" s="2">
         <v>1175.5066999999999</v>
       </c>
-      <c r="P45">
+      <c r="Q45">
         <v>0.56000000000000005</v>
       </c>
-      <c r="Q45">
+      <c r="R45">
         <v>5.8775000000000004</v>
       </c>
-      <c r="T45" t="s">
-        <v>69</v>
-      </c>
       <c r="U45" t="s">
+        <v>69</v>
+      </c>
+      <c r="V45" t="s">
         <v>198</v>
       </c>
-      <c r="V45" t="s">
+      <c r="W45" t="s">
         <v>167</v>
       </c>
-      <c r="W45" t="s">
-        <v>71</v>
-      </c>
       <c r="X45" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="Y45" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="Z45" t="s">
+        <v>80</v>
+      </c>
+      <c r="AA45" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="46" spans="2:26" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B46" t="s">
         <v>164</v>
       </c>
@@ -4782,48 +4834,51 @@
         <v>0.28999999999999998</v>
       </c>
       <c r="H46" s="2">
-        <f>O48</f>
+        <f>P48</f>
         <v>4516.7133000000003</v>
       </c>
       <c r="I46" s="3">
-        <f>($N$48/100)*H46</f>
+        <f>($O$48/100)*H46</f>
         <v>162.96753257730003</v>
       </c>
       <c r="J46">
-        <f>$Q$48</f>
+        <f>$R$48</f>
         <v>2.8138000000000001</v>
       </c>
       <c r="K46">
         <v>40</v>
       </c>
-      <c r="M46" t="s">
+      <c r="L46">
+        <v>0.8</v>
+      </c>
+      <c r="N46" t="s">
         <v>212</v>
       </c>
-      <c r="N46" s="4"/>
-      <c r="O46" s="2"/>
-      <c r="T46" t="s">
-        <v>69</v>
-      </c>
+      <c r="O46" s="4"/>
+      <c r="P46" s="2"/>
       <c r="U46" t="s">
+        <v>69</v>
+      </c>
+      <c r="V46" t="s">
         <v>172</v>
       </c>
-      <c r="V46" t="s">
+      <c r="W46" t="s">
         <v>173</v>
       </c>
-      <c r="W46" t="s">
-        <v>71</v>
-      </c>
       <c r="X46" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="Y46" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="Z46" t="s">
+        <v>80</v>
+      </c>
+      <c r="AA46" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="47" spans="2:26" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B47" t="s">
         <v>168</v>
       </c>
@@ -4840,62 +4895,65 @@
         <v>4.0999999999999995E-3</v>
       </c>
       <c r="G47">
+        <f>Q45</f>
+        <v>0.56000000000000005</v>
+      </c>
+      <c r="H47" s="2">
         <f>P45</f>
-        <v>0.56000000000000005</v>
-      </c>
-      <c r="H47" s="2">
-        <f>O45</f>
         <v>1175.5066999999999</v>
       </c>
       <c r="I47" s="3">
-        <f>($N$45/100)*H47</f>
+        <f>($O$45/100)*H47</f>
         <v>39.138495576499992</v>
       </c>
       <c r="J47">
-        <f>$Q$45</f>
+        <f>$R$45</f>
         <v>5.8775000000000004</v>
       </c>
       <c r="K47">
         <v>40</v>
       </c>
-      <c r="M47" t="s">
+      <c r="L47">
+        <v>0.8</v>
+      </c>
+      <c r="N47" t="s">
         <v>209</v>
       </c>
-      <c r="N47">
+      <c r="O47">
         <v>4.5269000000000004</v>
       </c>
-      <c r="O47" s="2">
+      <c r="P47" s="2">
         <v>2950.7891</v>
       </c>
-      <c r="P47">
+      <c r="Q47">
         <v>0.46800000000000003</v>
       </c>
-      <c r="Q47">
+      <c r="R47">
         <v>2.8138000000000001</v>
       </c>
-      <c r="T47" t="s">
-        <v>69</v>
-      </c>
       <c r="U47" t="s">
+        <v>69</v>
+      </c>
+      <c r="V47" t="s">
         <v>174</v>
       </c>
-      <c r="V47" t="s">
+      <c r="W47" t="s">
         <v>175</v>
       </c>
-      <c r="W47" t="s">
-        <v>71</v>
-      </c>
       <c r="X47" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="Y47" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="Z47" t="s">
+        <v>80</v>
+      </c>
+      <c r="AA47" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="48" spans="2:26" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B48" t="s">
         <v>198</v>
       </c>
@@ -4912,15 +4970,15 @@
         <v>1.4E-3</v>
       </c>
       <c r="G48">
+        <f>Q44</f>
+        <v>0.33</v>
+      </c>
+      <c r="H48" s="2">
         <f>P44</f>
-        <v>0.33</v>
-      </c>
-      <c r="H48" s="2">
-        <f>O44</f>
         <v>4812.0244000000002</v>
       </c>
       <c r="I48" s="3">
-        <f>($N$48/100)*H48</f>
+        <f>($O$48/100)*H48</f>
         <v>173.62265237640003</v>
       </c>
       <c r="J48">
@@ -4930,44 +4988,47 @@
       <c r="K48">
         <v>40</v>
       </c>
-      <c r="M48" t="s">
+      <c r="L48">
+        <v>0.8</v>
+      </c>
+      <c r="N48" t="s">
         <v>210</v>
       </c>
-      <c r="N48">
+      <c r="O48">
         <v>3.6080999999999999</v>
       </c>
-      <c r="O48" s="2">
+      <c r="P48" s="2">
         <v>4516.7133000000003</v>
       </c>
-      <c r="P48">
+      <c r="Q48">
         <v>0.2994</v>
       </c>
-      <c r="Q48">
+      <c r="R48">
         <v>2.8138000000000001</v>
       </c>
-      <c r="T48" t="s">
-        <v>69</v>
-      </c>
       <c r="U48" t="s">
+        <v>69</v>
+      </c>
+      <c r="V48" t="s">
         <v>176</v>
       </c>
-      <c r="V48" t="s">
+      <c r="W48" t="s">
         <v>177</v>
       </c>
-      <c r="W48" t="s">
-        <v>71</v>
-      </c>
       <c r="X48" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="Y48" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="Z48" t="s">
+        <v>80</v>
+      </c>
+      <c r="AA48" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="49" spans="2:26" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B49" t="s">
         <v>172</v>
       </c>
@@ -4987,45 +5048,48 @@
         <v>0.28999999999999998</v>
       </c>
       <c r="H49" s="2">
-        <f>O48</f>
+        <f>P48</f>
         <v>4516.7133000000003</v>
       </c>
       <c r="I49" s="3">
-        <f>($N$48/100)*H49</f>
+        <f>($O$48/100)*H49</f>
         <v>162.96753257730003</v>
       </c>
       <c r="J49">
-        <f>$Q$48</f>
+        <f>$R$48</f>
         <v>2.8138000000000001</v>
       </c>
       <c r="K49">
         <v>40</v>
       </c>
-      <c r="N49" s="3"/>
-      <c r="O49" s="4"/>
-      <c r="T49" t="s">
-        <v>69</v>
-      </c>
+      <c r="L49">
+        <v>0.8</v>
+      </c>
+      <c r="O49" s="3"/>
+      <c r="P49" s="4"/>
       <c r="U49" t="s">
+        <v>69</v>
+      </c>
+      <c r="V49" t="s">
         <v>178</v>
       </c>
-      <c r="V49" t="s">
+      <c r="W49" t="s">
         <v>179</v>
       </c>
-      <c r="W49" t="s">
-        <v>71</v>
-      </c>
       <c r="X49" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="Y49" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="Z49" t="s">
+        <v>80</v>
+      </c>
+      <c r="AA49" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="50" spans="2:26" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B50" t="s">
         <v>174</v>
       </c>
@@ -5045,45 +5109,48 @@
         <v>0.28999999999999998</v>
       </c>
       <c r="H50" s="2">
-        <f>O48</f>
+        <f>P48</f>
         <v>4516.7133000000003</v>
       </c>
       <c r="I50" s="3">
-        <f>($N$48/100)*H50</f>
+        <f>($O$48/100)*H50</f>
         <v>162.96753257730003</v>
       </c>
       <c r="J50">
-        <f>$Q$48</f>
+        <f>$R$48</f>
         <v>2.8138000000000001</v>
       </c>
       <c r="K50">
         <v>40</v>
       </c>
-      <c r="N50" s="3"/>
-      <c r="O50" s="4"/>
-      <c r="T50" t="s">
-        <v>69</v>
-      </c>
+      <c r="L50">
+        <v>0.8</v>
+      </c>
+      <c r="O50" s="3"/>
+      <c r="P50" s="4"/>
       <c r="U50" t="s">
+        <v>69</v>
+      </c>
+      <c r="V50" t="s">
         <v>180</v>
       </c>
-      <c r="V50" t="s">
+      <c r="W50" t="s">
         <v>181</v>
       </c>
-      <c r="W50" t="s">
-        <v>71</v>
-      </c>
       <c r="X50" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="Y50" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="Z50" t="s">
+        <v>80</v>
+      </c>
+      <c r="AA50" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="51" spans="2:26" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B51" t="s">
         <v>176</v>
       </c>
@@ -5100,49 +5167,52 @@
         <v>1.8E-3</v>
       </c>
       <c r="G51">
+        <f>Q45</f>
+        <v>0.56000000000000005</v>
+      </c>
+      <c r="H51" s="2">
         <f>P45</f>
-        <v>0.56000000000000005</v>
-      </c>
-      <c r="H51" s="2">
-        <f>O45</f>
         <v>1175.5066999999999</v>
       </c>
       <c r="I51" s="3">
-        <f t="shared" ref="I51:I52" si="8">($N$45/100)*H51</f>
+        <f t="shared" ref="I51:I52" si="8">($O$45/100)*H51</f>
         <v>39.138495576499992</v>
       </c>
       <c r="J51">
-        <f>$Q$45</f>
+        <f>$R$45</f>
         <v>5.8775000000000004</v>
       </c>
       <c r="K51">
         <v>40</v>
       </c>
-      <c r="N51" s="3"/>
-      <c r="O51" s="4"/>
-      <c r="T51" t="s">
-        <v>69</v>
-      </c>
+      <c r="L51">
+        <v>0.8</v>
+      </c>
+      <c r="O51" s="3"/>
+      <c r="P51" s="4"/>
       <c r="U51" t="s">
+        <v>69</v>
+      </c>
+      <c r="V51" t="s">
         <v>182</v>
       </c>
-      <c r="V51" t="s">
+      <c r="W51" t="s">
         <v>183</v>
       </c>
-      <c r="W51" t="s">
-        <v>71</v>
-      </c>
       <c r="X51" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="Y51" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="Z51" t="s">
+        <v>80</v>
+      </c>
+      <c r="AA51" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="52" spans="2:26" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B52" t="s">
         <v>178</v>
       </c>
@@ -5159,11 +5229,11 @@
         <v>1.8E-3</v>
       </c>
       <c r="G52">
+        <f>Q45</f>
+        <v>0.56000000000000005</v>
+      </c>
+      <c r="H52" s="2">
         <f>P45</f>
-        <v>0.56000000000000005</v>
-      </c>
-      <c r="H52" s="2">
-        <f>O45</f>
         <v>1175.5066999999999</v>
       </c>
       <c r="I52" s="3">
@@ -5171,37 +5241,40 @@
         <v>39.138495576499992</v>
       </c>
       <c r="J52">
-        <f>$Q$45</f>
+        <f>$R$45</f>
         <v>5.8775000000000004</v>
       </c>
       <c r="K52">
         <v>40</v>
       </c>
-      <c r="N52" s="3"/>
-      <c r="O52" s="4"/>
-      <c r="T52" t="s">
-        <v>69</v>
-      </c>
+      <c r="L52">
+        <v>0.8</v>
+      </c>
+      <c r="O52" s="3"/>
+      <c r="P52" s="4"/>
       <c r="U52" t="s">
+        <v>69</v>
+      </c>
+      <c r="V52" t="s">
         <v>184</v>
       </c>
-      <c r="V52" t="s">
+      <c r="W52" t="s">
         <v>185</v>
       </c>
-      <c r="W52" t="s">
-        <v>71</v>
-      </c>
       <c r="X52" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="Y52" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="Z52" t="s">
+        <v>80</v>
+      </c>
+      <c r="AA52" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="53" spans="2:26" x14ac:dyDescent="0.25">
+    <row r="53" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B53" t="s">
         <v>180</v>
       </c>
@@ -5221,43 +5294,46 @@
         <v>0.28999999999999998</v>
       </c>
       <c r="H53" s="2">
-        <f>O48</f>
+        <f>P48</f>
         <v>4516.7133000000003</v>
       </c>
       <c r="I53" s="3">
-        <f>($N$48/100)*H53</f>
+        <f>($O$48/100)*H53</f>
         <v>162.96753257730003</v>
       </c>
       <c r="J53">
-        <f>$Q$48</f>
+        <f>$R$48</f>
         <v>2.8138000000000001</v>
       </c>
       <c r="K53">
         <v>40</v>
       </c>
-      <c r="T53" t="s">
-        <v>69</v>
+      <c r="L53">
+        <v>0.8</v>
       </c>
       <c r="U53" t="s">
+        <v>69</v>
+      </c>
+      <c r="V53" t="s">
         <v>186</v>
       </c>
-      <c r="V53" t="s">
+      <c r="W53" t="s">
         <v>188</v>
       </c>
-      <c r="W53" t="s">
-        <v>71</v>
-      </c>
       <c r="X53" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="Y53" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="Z53" t="s">
+        <v>80</v>
+      </c>
+      <c r="AA53" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="54" spans="2:26" x14ac:dyDescent="0.25">
+    <row r="54" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B54" t="s">
         <v>182</v>
       </c>
@@ -5277,43 +5353,46 @@
         <v>0.28999999999999998</v>
       </c>
       <c r="H54" s="2">
-        <f>$O$48</f>
+        <f>$P$48</f>
         <v>4516.7133000000003</v>
       </c>
       <c r="I54" s="3">
-        <f t="shared" ref="I54:I58" si="9">($N$48/100)*H54</f>
+        <f t="shared" ref="I54:I58" si="9">($O$48/100)*H54</f>
         <v>162.96753257730003</v>
       </c>
       <c r="J54">
-        <f t="shared" ref="J54:J58" si="10">$Q$48</f>
+        <f t="shared" ref="J54:J58" si="10">$R$48</f>
         <v>2.8138000000000001</v>
       </c>
       <c r="K54">
         <v>40</v>
       </c>
-      <c r="T54" t="s">
-        <v>69</v>
+      <c r="L54">
+        <v>0.8</v>
       </c>
       <c r="U54" t="s">
+        <v>69</v>
+      </c>
+      <c r="V54" t="s">
         <v>187</v>
       </c>
-      <c r="V54" t="s">
+      <c r="W54" t="s">
         <v>189</v>
       </c>
-      <c r="W54" t="s">
-        <v>71</v>
-      </c>
       <c r="X54" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="Y54" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="Z54" t="s">
+        <v>80</v>
+      </c>
+      <c r="AA54" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="55" spans="2:26" x14ac:dyDescent="0.25">
+    <row r="55" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B55" t="s">
         <v>184</v>
       </c>
@@ -5333,7 +5412,7 @@
         <v>0.28999999999999998</v>
       </c>
       <c r="H55" s="2">
-        <f>$O$48</f>
+        <f>$P$48</f>
         <v>4516.7133000000003</v>
       </c>
       <c r="I55" s="3">
@@ -5347,29 +5426,32 @@
       <c r="K55">
         <v>40</v>
       </c>
-      <c r="T55" t="s">
-        <v>69</v>
+      <c r="L55">
+        <v>0.8</v>
       </c>
       <c r="U55" t="s">
+        <v>69</v>
+      </c>
+      <c r="V55" t="s">
         <v>190</v>
       </c>
-      <c r="V55" t="s">
+      <c r="W55" t="s">
         <v>191</v>
       </c>
-      <c r="W55" t="s">
-        <v>71</v>
-      </c>
       <c r="X55" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="Y55" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="Z55" t="s">
+        <v>80</v>
+      </c>
+      <c r="AA55" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="56" spans="2:26" x14ac:dyDescent="0.25">
+    <row r="56" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B56" t="s">
         <v>186</v>
       </c>
@@ -5389,7 +5471,7 @@
         <v>0.28999999999999998</v>
       </c>
       <c r="H56" s="2">
-        <f>O48</f>
+        <f>P48</f>
         <v>4516.7133000000003</v>
       </c>
       <c r="I56" s="3">
@@ -5403,29 +5485,32 @@
       <c r="K56">
         <v>40</v>
       </c>
-      <c r="T56" t="s">
-        <v>69</v>
+      <c r="L56">
+        <v>0.8</v>
       </c>
       <c r="U56" t="s">
+        <v>69</v>
+      </c>
+      <c r="V56" t="s">
         <v>18</v>
       </c>
-      <c r="V56" t="s">
+      <c r="W56" t="s">
         <v>78</v>
       </c>
-      <c r="W56" t="s">
-        <v>71</v>
-      </c>
       <c r="X56" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="Y56" t="s">
+        <v>72</v>
+      </c>
+      <c r="Z56" t="s">
         <v>73</v>
       </c>
-      <c r="Z56" t="s">
+      <c r="AA56" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="57" spans="2:26" x14ac:dyDescent="0.25">
+    <row r="57" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B57" t="s">
         <v>187</v>
       </c>
@@ -5445,7 +5530,7 @@
         <v>0.28999999999999998</v>
       </c>
       <c r="H57" s="2">
-        <f>O48</f>
+        <f>P48</f>
         <v>4516.7133000000003</v>
       </c>
       <c r="I57" s="3">
@@ -5459,8 +5544,11 @@
       <c r="K57">
         <v>40</v>
       </c>
-    </row>
-    <row r="58" spans="2:26" x14ac:dyDescent="0.25">
+      <c r="L57">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="58" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B58" t="s">
         <v>190</v>
       </c>
@@ -5480,7 +5568,7 @@
         <v>0.28999999999999998</v>
       </c>
       <c r="H58" s="2">
-        <f>O48</f>
+        <f>P48</f>
         <v>4516.7133000000003</v>
       </c>
       <c r="I58" s="3">
@@ -5494,8 +5582,11 @@
       <c r="K58">
         <v>40</v>
       </c>
-    </row>
-    <row r="59" spans="2:26" x14ac:dyDescent="0.25">
+      <c r="L58">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="59" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B59" t="s">
         <v>18</v>
       </c>
@@ -5514,151 +5605,154 @@
       <c r="G59">
         <v>0.33123000000000002</v>
       </c>
-    </row>
-    <row r="75" spans="20:26" x14ac:dyDescent="0.25">
-      <c r="U75" t="s">
+      <c r="L59">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="75" spans="21:27" x14ac:dyDescent="0.25">
+      <c r="V75" t="s">
         <v>207</v>
       </c>
     </row>
-    <row r="76" spans="20:26" x14ac:dyDescent="0.25">
-      <c r="T76" t="s">
-        <v>69</v>
-      </c>
+    <row r="76" spans="21:27" x14ac:dyDescent="0.25">
       <c r="U76" t="s">
+        <v>69</v>
+      </c>
+      <c r="V76" t="s">
         <v>44</v>
       </c>
-      <c r="V76" t="s">
+      <c r="W76" t="s">
         <v>78</v>
       </c>
-      <c r="W76" t="s">
-        <v>71</v>
-      </c>
       <c r="X76" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="Y76" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="Z76" t="s">
+        <v>80</v>
+      </c>
+      <c r="AA76" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="77" spans="20:26" x14ac:dyDescent="0.25">
-      <c r="T77" t="s">
-        <v>69</v>
-      </c>
+    <row r="77" spans="21:27" x14ac:dyDescent="0.25">
       <c r="U77" t="s">
+        <v>69</v>
+      </c>
+      <c r="V77" t="s">
         <v>47</v>
       </c>
-      <c r="V77" t="s">
+      <c r="W77" t="s">
         <v>78</v>
       </c>
-      <c r="W77" t="s">
-        <v>71</v>
-      </c>
       <c r="X77" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="Y77" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="Z77" t="s">
+        <v>80</v>
+      </c>
+      <c r="AA77" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="78" spans="20:26" x14ac:dyDescent="0.25">
-      <c r="T78" t="s">
-        <v>69</v>
-      </c>
+    <row r="78" spans="21:27" x14ac:dyDescent="0.25">
       <c r="U78" t="s">
+        <v>69</v>
+      </c>
+      <c r="V78" t="s">
         <v>49</v>
       </c>
-      <c r="V78" t="s">
+      <c r="W78" t="s">
         <v>78</v>
       </c>
-      <c r="W78" t="s">
-        <v>71</v>
-      </c>
       <c r="X78" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="Y78" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="Z78" t="s">
+        <v>80</v>
+      </c>
+      <c r="AA78" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="79" spans="20:26" x14ac:dyDescent="0.25">
-      <c r="T79" t="s">
-        <v>69</v>
-      </c>
+    <row r="79" spans="21:27" x14ac:dyDescent="0.25">
       <c r="U79" t="s">
+        <v>69</v>
+      </c>
+      <c r="V79" t="s">
         <v>51</v>
       </c>
-      <c r="V79" t="s">
+      <c r="W79" t="s">
         <v>78</v>
       </c>
-      <c r="W79" t="s">
-        <v>71</v>
-      </c>
       <c r="X79" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="Y79" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="Z79" t="s">
+        <v>80</v>
+      </c>
+      <c r="AA79" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="80" spans="20:26" x14ac:dyDescent="0.25">
-      <c r="T80" t="s">
-        <v>69</v>
-      </c>
+    <row r="80" spans="21:27" x14ac:dyDescent="0.25">
       <c r="U80" t="s">
+        <v>69</v>
+      </c>
+      <c r="V80" t="s">
         <v>53</v>
       </c>
-      <c r="V80" t="s">
+      <c r="W80" t="s">
         <v>78</v>
       </c>
-      <c r="W80" t="s">
-        <v>71</v>
-      </c>
       <c r="X80" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="Y80" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="Z80" t="s">
+        <v>80</v>
+      </c>
+      <c r="AA80" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="81" spans="2:26" x14ac:dyDescent="0.25">
-      <c r="T81" t="s">
-        <v>69</v>
-      </c>
+    <row r="81" spans="2:27" x14ac:dyDescent="0.25">
       <c r="U81" t="s">
+        <v>69</v>
+      </c>
+      <c r="V81" t="s">
         <v>55</v>
       </c>
-      <c r="V81" t="s">
+      <c r="W81" t="s">
         <v>78</v>
       </c>
-      <c r="W81" t="s">
-        <v>71</v>
-      </c>
       <c r="X81" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="Y81" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="Z81" t="s">
+        <v>80</v>
+      </c>
+      <c r="AA81" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="82" spans="2:26" x14ac:dyDescent="0.25">
+    <row r="82" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B82" t="s">
         <v>20</v>
       </c>
@@ -5689,29 +5783,29 @@
       <c r="K82">
         <v>42</v>
       </c>
-      <c r="T82" t="s">
-        <v>69</v>
-      </c>
       <c r="U82" t="s">
+        <v>69</v>
+      </c>
+      <c r="V82" t="s">
         <v>57</v>
       </c>
-      <c r="V82" t="s">
+      <c r="W82" t="s">
         <v>78</v>
       </c>
-      <c r="W82" t="s">
-        <v>71</v>
-      </c>
       <c r="X82" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="Y82" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="Z82" t="s">
+        <v>80</v>
+      </c>
+      <c r="AA82" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="83" spans="2:26" x14ac:dyDescent="0.25">
+    <row r="83" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B83" t="s">
         <v>15</v>
       </c>
@@ -5730,52 +5824,52 @@
       <c r="G83">
         <v>0.33123000000000002</v>
       </c>
-      <c r="T83" t="s">
-        <v>69</v>
-      </c>
       <c r="U83" t="s">
+        <v>69</v>
+      </c>
+      <c r="V83" t="s">
         <v>59</v>
       </c>
-      <c r="V83" t="s">
+      <c r="W83" t="s">
         <v>78</v>
       </c>
-      <c r="W83" t="s">
-        <v>71</v>
-      </c>
       <c r="X83" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="Y83" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="Z83" t="s">
+        <v>80</v>
+      </c>
+      <c r="AA83" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="84" spans="2:26" x14ac:dyDescent="0.25">
-      <c r="T84" t="s">
-        <v>69</v>
-      </c>
+    <row r="84" spans="2:27" x14ac:dyDescent="0.25">
       <c r="U84" t="s">
+        <v>69</v>
+      </c>
+      <c r="V84" t="s">
         <v>20</v>
       </c>
-      <c r="V84" t="s">
+      <c r="W84" t="s">
         <v>79</v>
       </c>
-      <c r="W84" t="s">
-        <v>71</v>
-      </c>
       <c r="X84" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="Y84" t="s">
+        <v>72</v>
+      </c>
+      <c r="Z84" t="s">
         <v>73</v>
       </c>
-      <c r="Z84" t="s">
+      <c r="AA84" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="85" spans="2:26" x14ac:dyDescent="0.25">
+    <row r="85" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B85" t="s">
         <v>12</v>
       </c>
@@ -5806,52 +5900,52 @@
       <c r="K85">
         <v>50</v>
       </c>
-      <c r="T85" t="s">
-        <v>69</v>
-      </c>
       <c r="U85" t="s">
+        <v>69</v>
+      </c>
+      <c r="V85" t="s">
         <v>15</v>
       </c>
-      <c r="V85" t="s">
+      <c r="W85" t="s">
         <v>75</v>
       </c>
-      <c r="W85" t="s">
-        <v>71</v>
-      </c>
       <c r="X85" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="Y85" t="s">
+        <v>72</v>
+      </c>
+      <c r="Z85" t="s">
         <v>73</v>
       </c>
-      <c r="Z85" t="s">
+      <c r="AA85" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="87" spans="2:26" x14ac:dyDescent="0.25">
-      <c r="T87" t="s">
-        <v>69</v>
-      </c>
+    <row r="87" spans="2:27" x14ac:dyDescent="0.25">
       <c r="U87" t="s">
+        <v>69</v>
+      </c>
+      <c r="V87" t="s">
         <v>12</v>
       </c>
-      <c r="V87" t="s">
+      <c r="W87" t="s">
         <v>70</v>
       </c>
-      <c r="W87" t="s">
-        <v>71</v>
-      </c>
       <c r="X87" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="Y87" t="s">
+        <v>72</v>
+      </c>
+      <c r="Z87" t="s">
         <v>73</v>
       </c>
-      <c r="Z87" t="s">
+      <c r="AA87" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="90" spans="2:26" x14ac:dyDescent="0.25">
+    <row r="90" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B90" t="s">
         <v>44</v>
       </c>
@@ -5873,11 +5967,11 @@
       <c r="L90">
         <v>0.42012333946150526</v>
       </c>
-      <c r="P90" t="s">
+      <c r="Q90" t="s">
         <v>208</v>
       </c>
     </row>
-    <row r="91" spans="2:26" x14ac:dyDescent="0.25">
+    <row r="91" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B91" t="s">
         <v>47</v>
       </c>
@@ -5900,7 +5994,7 @@
         <v>0.42012333946150526</v>
       </c>
     </row>
-    <row r="92" spans="2:26" x14ac:dyDescent="0.25">
+    <row r="92" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B92" t="s">
         <v>49</v>
       </c>
@@ -5923,7 +6017,7 @@
         <v>0.42012333946150526</v>
       </c>
     </row>
-    <row r="93" spans="2:26" x14ac:dyDescent="0.25">
+    <row r="93" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B93" t="s">
         <v>51</v>
       </c>
@@ -5958,7 +6052,7 @@
         <v>0.47763777043344691</v>
       </c>
     </row>
-    <row r="94" spans="2:26" x14ac:dyDescent="0.25">
+    <row r="94" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B94" t="s">
         <v>53</v>
       </c>
@@ -5993,7 +6087,7 @@
         <v>0.47814004703314078</v>
       </c>
     </row>
-    <row r="95" spans="2:26" x14ac:dyDescent="0.25">
+    <row r="95" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B95" t="s">
         <v>53</v>
       </c>
@@ -6028,7 +6122,7 @@
         <v>0.47814004703314084</v>
       </c>
     </row>
-    <row r="96" spans="2:26" x14ac:dyDescent="0.25">
+    <row r="96" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B96" t="s">
         <v>53</v>
       </c>

</xml_diff>

<commit_message>
adding power plants to nodes
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/vt_EST_ELC_v1.xlsx
+++ b/VerveStacks_EST/vt_EST_ELC_v1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B695A222-C6ED-44AE-9780-8B7CF5007B2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FB4E033-3C5E-4352-A9FC-7D64A1EB4045}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="2" xr2:uid="{21C51102-B905-44E2-89DF-C1A7E31F8D9F}"/>
+    <workbookView xWindow="-38520" yWindow="-5220" windowWidth="38640" windowHeight="21120" firstSheet="1" activeTab="2" xr2:uid="{21C51102-B905-44E2-89DF-C1A7E31F8D9F}"/>
   </bookViews>
   <sheets>
     <sheet name="ccs_retrofits" sheetId="4" state="hidden" r:id="rId1"/>
@@ -148,7 +148,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="912" uniqueCount="222">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="912" uniqueCount="232">
   <si>
     <t>~fi_t</t>
   </si>
@@ -723,9 +723,6 @@
     <t>ep_bioenergy_tartuaardlapalu</t>
   </si>
   <si>
-    <t>Tartu Aardlapalu CHP</t>
-  </si>
-  <si>
     <t>coal</t>
   </si>
   <si>
@@ -813,7 +810,40 @@
     <t>ncap_af</t>
   </si>
   <si>
-    <t>Aggregated Plant -- operating agg</t>
+    <t>Tartu Aardlapalu CHP plant</t>
+  </si>
+  <si>
+    <t>e_harku_330</t>
+  </si>
+  <si>
+    <t>e_tartu_330</t>
+  </si>
+  <si>
+    <t>e_rakvere_330</t>
+  </si>
+  <si>
+    <t>e_paide_330</t>
+  </si>
+  <si>
+    <t>e_pussi_330</t>
+  </si>
+  <si>
+    <t>e_kilingi_nomme_330</t>
+  </si>
+  <si>
+    <t>e_sindi_330</t>
+  </si>
+  <si>
+    <t>e_tsirguliina_330</t>
+  </si>
+  <si>
+    <t>e_arukula_330</t>
+  </si>
+  <si>
+    <t>e_baltiej_330</t>
+  </si>
+  <si>
+    <t>e_viru_330</t>
   </si>
 </sst>
 </file>
@@ -1258,10 +1288,10 @@
   <sheetData>
     <row r="9" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="N9" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="10" spans="2:20" x14ac:dyDescent="0.25">
@@ -1618,10 +1648,10 @@
   <sheetData>
     <row r="9" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="N9" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="10" spans="2:20" x14ac:dyDescent="0.25">
@@ -1682,10 +1712,10 @@
     </row>
     <row r="11" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C11" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D11" t="s">
         <v>14</v>
@@ -1715,7 +1745,7 @@
         <v>69</v>
       </c>
       <c r="O11" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="P11" t="s">
         <v>108</v>
@@ -1735,10 +1765,10 @@
     </row>
     <row r="12" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C12" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D12" t="s">
         <v>14</v>
@@ -1768,7 +1798,7 @@
         <v>69</v>
       </c>
       <c r="O12" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="P12" t="s">
         <v>109</v>
@@ -2672,10 +2702,10 @@
     </row>
     <row r="30" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B30" t="s">
+        <v>200</v>
+      </c>
+      <c r="C30" t="s">
         <v>201</v>
-      </c>
-      <c r="C30" t="s">
-        <v>202</v>
       </c>
       <c r="D30" t="s">
         <v>14</v>
@@ -2705,10 +2735,10 @@
         <v>69</v>
       </c>
       <c r="O30" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="P30" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="Q30" t="s">
         <v>71</v>
@@ -2736,7 +2766,7 @@
   <cols>
     <col min="2" max="2" width="40.5703125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12.85546875" customWidth="1"/>
-    <col min="4" max="4" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.85546875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="9.28515625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="12.5703125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="9.28515625" bestFit="1" customWidth="1"/>
@@ -2798,7 +2828,7 @@
         <v>11</v>
       </c>
       <c r="M10" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="U10" t="s">
         <v>63</v>
@@ -3496,7 +3526,7 @@
         <v>69</v>
       </c>
       <c r="V23" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="W23" t="s">
         <v>76</v>
@@ -3608,7 +3638,7 @@
         <v>69</v>
       </c>
       <c r="V25" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="W25" t="s">
         <v>81</v>
@@ -3664,10 +3694,10 @@
         <v>69</v>
       </c>
       <c r="V26" t="s">
+        <v>216</v>
+      </c>
+      <c r="W26" t="s">
         <v>217</v>
-      </c>
-      <c r="W26" t="s">
-        <v>218</v>
       </c>
       <c r="X26" t="s">
         <v>71</v>
@@ -3684,7 +3714,7 @@
     </row>
     <row r="27" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B27" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C27" t="s">
         <v>45</v>
@@ -3725,7 +3755,7 @@
     </row>
     <row r="28" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B28" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C28" t="s">
         <v>45</v>
@@ -3761,7 +3791,7 @@
         <v>69</v>
       </c>
       <c r="V28" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="W28" t="s">
         <v>163</v>
@@ -3790,7 +3820,7 @@
         <v>69</v>
       </c>
       <c r="V29" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="W29" t="s">
         <v>148</v>
@@ -3810,13 +3840,13 @@
     </row>
     <row r="30" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B30" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C30" t="s">
         <v>13</v>
       </c>
       <c r="D30" t="s">
-        <v>14</v>
+        <v>229</v>
       </c>
       <c r="E30">
         <v>1982</v>
@@ -3849,7 +3879,7 @@
         <v>69</v>
       </c>
       <c r="V30" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="W30" t="s">
         <v>149</v>
@@ -3869,13 +3899,13 @@
     </row>
     <row r="31" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B31" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C31" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D31" t="s">
-        <v>14</v>
+        <v>231</v>
       </c>
       <c r="E31">
         <v>1965</v>
@@ -3908,7 +3938,7 @@
         <v>69</v>
       </c>
       <c r="V31" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="W31" t="s">
         <v>150</v>
@@ -3928,13 +3958,13 @@
     </row>
     <row r="32" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B32" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C32" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D32" t="s">
-        <v>14</v>
+        <v>231</v>
       </c>
       <c r="E32">
         <v>2015</v>
@@ -3987,13 +4017,13 @@
     </row>
     <row r="33" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B33" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C33" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D33" t="s">
-        <v>14</v>
+        <v>231</v>
       </c>
       <c r="E33">
         <v>2025</v>
@@ -4046,13 +4076,13 @@
     </row>
     <row r="34" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B34" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C34" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D34" t="s">
-        <v>14</v>
+        <v>230</v>
       </c>
       <c r="E34">
         <v>1956</v>
@@ -4111,7 +4141,7 @@
         <v>16</v>
       </c>
       <c r="D35" t="s">
-        <v>14</v>
+        <v>225</v>
       </c>
       <c r="E35">
         <v>2021</v>
@@ -4171,7 +4201,7 @@
         <v>13</v>
       </c>
       <c r="D36" t="s">
-        <v>14</v>
+        <v>221</v>
       </c>
       <c r="E36">
         <v>2018</v>
@@ -4231,7 +4261,7 @@
         <v>13</v>
       </c>
       <c r="D37" t="s">
-        <v>14</v>
+        <v>222</v>
       </c>
       <c r="E37">
         <v>2009</v>
@@ -4264,7 +4294,7 @@
         <v>69</v>
       </c>
       <c r="V37" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="W37" t="s">
         <v>162</v>
@@ -4290,7 +4320,7 @@
         <v>13</v>
       </c>
       <c r="D38" t="s">
-        <v>14</v>
+        <v>227</v>
       </c>
       <c r="E38">
         <v>2011</v>
@@ -4349,7 +4379,7 @@
         <v>13</v>
       </c>
       <c r="D39" t="s">
-        <v>14</v>
+        <v>229</v>
       </c>
       <c r="E39">
         <v>2010</v>
@@ -4402,13 +4432,13 @@
     </row>
     <row r="40" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B40" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C40" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D40" t="s">
-        <v>14</v>
+        <v>225</v>
       </c>
       <c r="E40">
         <v>1997</v>
@@ -4468,7 +4498,7 @@
         <v>13</v>
       </c>
       <c r="D41" t="s">
-        <v>14</v>
+        <v>224</v>
       </c>
       <c r="E41">
         <v>2016</v>
@@ -4527,7 +4557,7 @@
         <v>13</v>
       </c>
       <c r="D42" t="s">
-        <v>14</v>
+        <v>228</v>
       </c>
       <c r="E42">
         <v>2017</v>
@@ -4586,7 +4616,7 @@
         <v>13</v>
       </c>
       <c r="D43" t="s">
-        <v>14</v>
+        <v>221</v>
       </c>
       <c r="E43">
         <v>2019</v>
@@ -4616,16 +4646,16 @@
         <v>0.8</v>
       </c>
       <c r="O43" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="P43" t="s">
+        <v>212</v>
+      </c>
+      <c r="Q43" t="s">
         <v>213</v>
       </c>
-      <c r="Q43" t="s">
+      <c r="R43" t="s">
         <v>214</v>
-      </c>
-      <c r="R43" t="s">
-        <v>215</v>
       </c>
       <c r="U43" t="s">
         <v>69</v>
@@ -4657,7 +4687,7 @@
         <v>13</v>
       </c>
       <c r="D44" t="s">
-        <v>14</v>
+        <v>225</v>
       </c>
       <c r="E44">
         <v>1963</v>
@@ -4687,7 +4717,7 @@
         <v>0.8</v>
       </c>
       <c r="N44" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="O44" s="4">
         <v>1.31</v>
@@ -4731,7 +4761,7 @@
         <v>16</v>
       </c>
       <c r="D45" t="s">
-        <v>14</v>
+        <v>225</v>
       </c>
       <c r="E45">
         <v>2020</v>
@@ -4762,7 +4792,7 @@
         <v>0.8</v>
       </c>
       <c r="N45" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="O45" s="4">
         <v>3.3294999999999999</v>
@@ -4780,7 +4810,7 @@
         <v>69</v>
       </c>
       <c r="V45" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="W45" t="s">
         <v>167</v>
@@ -4806,7 +4836,7 @@
         <v>13</v>
       </c>
       <c r="D46" t="s">
-        <v>14</v>
+        <v>226</v>
       </c>
       <c r="E46">
         <v>2013</v>
@@ -4836,7 +4866,7 @@
         <v>0.8</v>
       </c>
       <c r="N46" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="O46" s="4"/>
       <c r="P46" s="2"/>
@@ -4870,7 +4900,7 @@
         <v>16</v>
       </c>
       <c r="D47" t="s">
-        <v>14</v>
+        <v>222</v>
       </c>
       <c r="E47">
         <v>2015</v>
@@ -4901,7 +4931,7 @@
         <v>0.8</v>
       </c>
       <c r="N47" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="O47">
         <v>4.5269000000000004</v>
@@ -4939,13 +4969,13 @@
     </row>
     <row r="48" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B48" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C48" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D48" t="s">
-        <v>14</v>
+        <v>225</v>
       </c>
       <c r="E48">
         <v>2012</v>
@@ -4976,7 +5006,7 @@
         <v>0.8</v>
       </c>
       <c r="N48" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="O48">
         <v>3.6080999999999999</v>
@@ -5020,7 +5050,7 @@
         <v>13</v>
       </c>
       <c r="D49" t="s">
-        <v>14</v>
+        <v>227</v>
       </c>
       <c r="E49">
         <v>2013</v>
@@ -5081,7 +5111,7 @@
         <v>13</v>
       </c>
       <c r="D50" t="s">
-        <v>14</v>
+        <v>224</v>
       </c>
       <c r="E50">
         <v>2015</v>
@@ -5142,7 +5172,7 @@
         <v>16</v>
       </c>
       <c r="D51" t="s">
-        <v>14</v>
+        <v>226</v>
       </c>
       <c r="E51">
         <v>2009</v>
@@ -5204,7 +5234,7 @@
         <v>16</v>
       </c>
       <c r="D52" t="s">
-        <v>14</v>
+        <v>225</v>
       </c>
       <c r="E52">
         <v>2015</v>
@@ -5266,7 +5296,7 @@
         <v>13</v>
       </c>
       <c r="D53" t="s">
-        <v>14</v>
+        <v>222</v>
       </c>
       <c r="E53">
         <v>2022</v>
@@ -5325,7 +5355,7 @@
         <v>13</v>
       </c>
       <c r="D54" t="s">
-        <v>14</v>
+        <v>223</v>
       </c>
       <c r="E54">
         <v>2013</v>
@@ -5384,7 +5414,7 @@
         <v>13</v>
       </c>
       <c r="D55" t="s">
-        <v>14</v>
+        <v>224</v>
       </c>
       <c r="E55">
         <v>2016</v>
@@ -5420,7 +5450,7 @@
         <v>190</v>
       </c>
       <c r="W55" t="s">
-        <v>191</v>
+        <v>220</v>
       </c>
       <c r="X55" t="s">
         <v>71</v>
@@ -5443,7 +5473,7 @@
         <v>13</v>
       </c>
       <c r="D56" t="s">
-        <v>14</v>
+        <v>221</v>
       </c>
       <c r="E56">
         <v>2009</v>
@@ -5479,7 +5509,7 @@
         <v>18</v>
       </c>
       <c r="W56" t="s">
-        <v>221</v>
+        <v>78</v>
       </c>
       <c r="X56" t="s">
         <v>71</v>
@@ -5502,7 +5532,7 @@
         <v>13</v>
       </c>
       <c r="D57" t="s">
-        <v>14</v>
+        <v>223</v>
       </c>
       <c r="E57">
         <v>2012</v>
@@ -5540,7 +5570,7 @@
         <v>13</v>
       </c>
       <c r="D58" t="s">
-        <v>14</v>
+        <v>222</v>
       </c>
       <c r="E58">
         <v>2015</v>
@@ -5578,7 +5608,7 @@
         <v>19</v>
       </c>
       <c r="D59" t="s">
-        <v>14</v>
+        <v>221</v>
       </c>
       <c r="E59">
         <v>2022</v>
@@ -5595,7 +5625,7 @@
     </row>
     <row r="75" spans="21:27" x14ac:dyDescent="0.25">
       <c r="V75" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
     <row r="76" spans="21:27" x14ac:dyDescent="0.25">
@@ -5952,7 +5982,7 @@
         <v>0.42012333946150526</v>
       </c>
       <c r="Q90" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
     </row>
     <row r="91" spans="2:27" x14ac:dyDescent="0.25">

</xml_diff>